<commit_message>
22th Commit : Swipe Mobile Action Implement In ABCD Framwork
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBC3F74-F9B5-4905-8275-F7F4F4840F3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D712BE5-B5E0-4499-8FFD-A3DEC01B2368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="38">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -643,7 +643,10 @@
     <t>If in case emulators crashes wipe data and  cold reboot all emulators and run this test to make the emultators and web browser into initial state before running other tests</t>
   </si>
   <si>
-    <t>1.wait,3000,,
+    <t>c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.wait,3000,,
 2.Load Driver App,switch_to,driver,
 3.wait,2000,,
 4.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
@@ -653,7 +656,17 @@
 8.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
 9.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
 10.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-10.wait,5000,,</t>
+11.wait,20000,,
+12.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+13.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+14.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+15.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+16.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+17.Drag Page Layout Upward,swipe,up,
+18.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+19.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+20.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+</t>
   </si>
 </sst>
 </file>
@@ -1257,7 +1270,7 @@
     <col min="2" max="2" width="21.5546875" customWidth="1"/>
     <col min="3" max="3" width="28.77734375" customWidth="1"/>
     <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="57.44140625" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
     <col min="6" max="6" width="40.44140625" customWidth="1"/>
     <col min="7" max="7" width="16.33203125" customWidth="1"/>
     <col min="8" max="8" width="15.21875" customWidth="1"/>
@@ -1303,7 +1316,7 @@
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>29</v>
@@ -1314,7 +1327,9 @@
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>

</xml_diff>

<commit_message>
23th Commit : Type Function Efficiency Improved
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D712BE5-B5E0-4499-8FFD-A3DEC01B2368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7B70795-6105-4E6A-82A6-C2C231B59547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -653,10 +653,10 @@
 5.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
 6.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
 7.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-8.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
+8..Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
 9.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
 10.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-11.wait,20000,,
+11.wait,10000,,
 12.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
 13.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
 14.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
@@ -666,6 +666,10 @@
 18.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
 19.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
 20.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+21.Click Agree,tap,,"//android.widget.Button[@content-desc='AGREE &amp; CONTINUE']"
+22.wait,5000,,
+23.Enter OTP,type,123456,"(//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText)[1]"
+24.wait,5000,,
 </t>
   </si>
 </sst>

</xml_diff>

<commit_message>
24th Commit : Test Starts From Begining
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7B70795-6105-4E6A-82A6-C2C231B59547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C3F40CE-C2D1-4676-91F1-9E51FEE68CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -574,26 +574,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">1.wait,3000,,
-2.Load User App,switch_to,user,
-3.wait,2000,,
-4.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-5.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-6.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-7.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-8.wait,2000,,
-9.Load Driver App,switch_to,driver,
-10.wait,2000,,
-11.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-12.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-13.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-14.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-15.wait,1000,,
-16.Load  Super Admin,switch_to,web,
-17.wait,2000,,
-</t>
-  </si>
-  <si>
     <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
 3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
@@ -647,29 +627,59 @@
   </si>
   <si>
     <t xml:space="preserve">1.wait,3000,,
+2.Load User App,switch_to,user,
+3.wait,2000,,
+4.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+5.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
+6.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+11.wait,2000,,
+12.Load Driver App,switch_to,driver,
+13.wait,2000,,
+14.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+15.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
+16.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+17.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+18.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+19.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+20.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+21.wait,1000,,
+22.Load  Super Admin,switch_to,web,
+23.wait,2000,,
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.wait,2000,,
 2.Load Driver App,switch_to,driver,
 3.wait,2000,,
-4.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-5.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-6.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-7.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-8..Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
-9.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
-10.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-11.wait,10000,,
-12.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
-13.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
-14.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
-15.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
-16.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
-17.Drag Page Layout Upward,swipe,up,
-18.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
-19.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
-20.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
-21.Click Agree,tap,,"//android.widget.Button[@content-desc='AGREE &amp; CONTINUE']"
-22.wait,5000,,
-23.Enter OTP,type,123456,"(//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText)[1]"
-24.wait,5000,,
+4.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+5.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
+6.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+11.Enter Auto Mobile,type,{autoMobile},"//android.widget.EditText"
+12.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+13.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+14.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
+15.wait,20000,,
+16.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+17.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+18.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+19.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+20.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+21.Drag Page Layout Upward,swipe,up,
+22.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+23.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+24.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+25.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+26.wait,10000,,
+27.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+28.wait,10000,,
 </t>
   </si>
 </sst>
@@ -1084,19 +1094,19 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>29</v>
@@ -1247,7 +1257,7 @@
         <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>22</v>
@@ -1332,7 +1342,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>

</xml_diff>

<commit_message>
25th Commit : Intialization Crash Fixed
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C3F40CE-C2D1-4676-91F1-9E51FEE68CFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65658657-9CC7-4EB3-AF38-87F7C3562535}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="39">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -626,32 +626,6 @@
     <t>c</t>
   </si>
   <si>
-    <t xml:space="preserve">1.wait,3000,,
-2.Load User App,switch_to,user,
-3.wait,2000,,
-4.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-5.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
-6.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-11.wait,2000,,
-12.Load Driver App,switch_to,driver,
-13.wait,2000,,
-14.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-15.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
-16.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-17.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-18.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-19.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-20.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-21.wait,1000,,
-22.Load  Super Admin,switch_to,web,
-23.wait,2000,,
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">1.wait,2000,,
 2.Load Driver App,switch_to,driver,
 3.wait,2000,,
@@ -676,10 +650,149 @@
 22.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
 23.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
 24.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
-25.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
-26.wait,10000,,
-27.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-28.wait,10000,,
+25.wait,3000,,
+26.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+27.wait,10000,,
+28.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+29.wait,10000,,
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin and AddAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">RunSheet: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SuperAdminLogin
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">1.wait,3000,,
+2.Load User App,switch_to,user,
+3.wait,2000,,
+4.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+5.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+11.wait,2000,,
+12.Load Driver App,switch_to,driver,
+13.wait,2000,,
+14.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+15.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
+16.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+17.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+18.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+19.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+20.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+21.wait,1000,,
+22.Load  Super Admin,switch_to,web,
+23.wait,2000,,
 </t>
   </si>
 </sst>
@@ -1106,10 +1219,10 @@
         <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1330,7 +1443,7 @@
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
30th Commit :Driver Document Upload Finished
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2886B7F1-F7D3-472E-B344-AF4802A6EDE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A39F430-5D35-4615-AE63-96A0FD90CF49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -823,8 +823,18 @@
 31.Click Document,tap,,"//android.view.View[@content-desc='Documents']"
 32.Click Upload,tap,,"//android.widget.Button[@content-desc='Upload']"
 33.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","//android.widget.ImageView[@content-desc='Upload Documents']"
-34..Click License,tap,,"//*[contains(@text, 'license.JPG')] or //*[@text='license.JPG']"
-35.wait,10000,,</t>
+34.Click Sort,tap,,"//android.widget.TextView[@resource-id="com.google.android.documentsui:id/title" and @text="Sort by..."]"
+35.Click Modified,tap,,"//android.widget.CheckedTextView[@resource-id="android:id/text1" and @text="Modified (newest first)"]"
+36.Click License,tap,,"//android.widget.ImageView[@resource-id="com.google.android.documentsui:id/icon_thumb"]"
+37.Click Crop,tap,,"//android.widget.Button[@content-desc="Crop"]"
+38.Click Calender,tap,,"//android.widget.ImageView[contains(@content-desc, 'Driving Licence')]/android.view.View[2]/android.view.View"
+39.Click Month,tap,"//android.widget.Button[@content-desc="Next month"]"
+40.Click Date,tap,,"//android.widget.Button[contains(@content-desc, '25')]"
+41. Click Ok,tap,,"//android.widget.Button[@content-desc="OK"]"
+42.Click Upload,tap,,"//android.widget.Button[@content-desc="Upload Documents"]"
+43.wait,4000,,
+44.Click Back,tap,,"//android.view.View[@content-desc="Back"]"
+45.wait,10000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
37th Commit :Power Tap Implemented To Pass Tests
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7173322F-1D68-4EF4-B364-BE6C38CCFA31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F83576BE-DB8E-41F7-9603-AD31B4AFB240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1233,7 +1233,6 @@
 48.wait,2000,,
 49.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
 50.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-51.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
 52.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
 53.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
 54.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
@@ -1252,7 +1251,6 @@
 67.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
 68.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
 69.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-70.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
 71.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
 72.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
 73.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"

</xml_diff>

<commit_message>
41th Commit :Subscrption Plan Test Completed
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1DC461-CC63-49C6-9AE2-78C1CCFE914E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83CD3D17-167C-40E7-BE69-0769FB09B760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1040,103 +1040,6 @@
       </rPr>
       <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
     </r>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
-2.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-3.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-3.Click Driver subscription plan,click,,"//span[normalize-space()='Driver Subscription Plan']"
-4.Verify Driver Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Driver']"
-5.Click  Add New Subscription,click,,"//button[normalize-space()='ADD']"
-6.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
-7.Select Auto Ride,click,,"//li[@aria-label='Auto Ride']"
-8.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "//input[@placeholder='Plan Name']"
-9.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
-10.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil)']"
-11.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi)']"
-12.Enter Number Of Days, type,100, "//input[@placeholder='No. of Days ']"
-13.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No of Rides with Zero admin commission']"
-14.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
-15.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
-16.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description Arabic']"
-17.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description Tamil']"
-18.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description Hindi']"
-19.Open status Dropdown,click,,"//span[@aria-label='select Status']"
-20.Select On,click,,"//li[@aria-label='on']"
-21.Click Submit ,click,,"//button[normalize-space()='Submit']"
-22.Filter Services List,type,{driverSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-23.wait,2000,,
-24.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
-25.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-26.Click Customer subscription plan,click,,"//span[normalize-space()='Customer Subscription Plan']"
-27.Verify Customer Subscription Plan Lists ,verify,,"//div[normalize-space()='Customer Subscription Plans']"
-28.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
-29.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
-30.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
-31.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; custometSubscriptionName, "//input[@placeholder='Plan Name']"
-32.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
-33.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
-34.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
-35.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
-36.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No Of Free Rides']"
-37.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
-38.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
-39.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
-40.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
-41.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
-42.Open status Dropdown,click,,"//span[@aria-label='select Status']"
-43.Select On,click,,"//li[@aria-label='on']"
-44.Click Submit ,click,,"//button[normalize-space()='Submit']"
-45.Filter Services List,type,{custometSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-46.wait,3000,,
-47.Load User App,switch_to,user,
-48.wait,2000,,
-49.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-50.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-52.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-53.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-54.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-55.wait,2000,,
-56.Enter Mobile Number,type,{userPhone},"//android.widget.EditText"
-57.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
-58.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
-59.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-60.Click Finish,tap,,"//android.widget.Button[@content-desc="Finish"]"
-61.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
-62.Profile, tap_coordinate ,978:2224,COORDINATE_MODE
-63.Click Subscription,tap,,"//android.view.View[@content-desc="Subscription"]"
-64.wait,5000,,
-65.Load Driver App,switch_to,driver,
-66.wait,2000,,
-67.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
-68.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
-69.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
-71.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-72.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-73.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-74.Enter Mobile Number,type,{autoPhone},"//android.widget.EditText"
-75.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
-76.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
-77.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-78.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
-79.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
-80.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
-81.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
-82.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
-83.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
-84.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
-85.Drag Page Layout Upward,swipe,up,
-86.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
-87.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
-88.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
-89.wait,3000,,
-90.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
-91.Wait For OTP,wait_until_visible,,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-92.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
-93.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
-94.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
-95.Click Subscription,tap,,"//android.view.View[@content-desc="Subscription"]"
-96.wait,10000,,</t>
   </si>
   <si>
     <t>1.Load Driver App,switch_to,driver,
@@ -1285,6 +1188,107 @@
 19.Load  Super Admin,switch_to,web,
 20.wait,2000,,
 </t>
+  </si>
+  <si>
+    <t>1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+2.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+3.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+3.Click Driver subscription plan,click,,"//span[normalize-space()='Driver Subscription Plan']"
+4.Verify Driver Subscription Plan Lists ,verify,,"//div[normalize-space()='Subscription Plan Lists - Driver']"
+5.Click  Add New Subscription,click,,"//button[normalize-space()='ADD']"
+6.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+7.Select Auto Ride,click,,"//li[@aria-label='Auto Ride']"
+8.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "//input[@placeholder='Plan Name']"
+9.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+10.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil)']"
+11.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi)']"
+12.Enter Number Of Days, type,100, "//input[@placeholder='No. of Days ']"
+13.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No of Rides with Zero admin commission']"
+14.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+15.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+16.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description Arabic']"
+17.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description Tamil']"
+18.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description Hindi']"
+19.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+20.Select On,click,,"//li[@aria-label='on']"
+21.Click Submit ,click,,"//button[normalize-space()='Submit']"
+22.Filter Services List,type,{driverSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+23.wait,2000,,
+24.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+25.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+26.Click Customer subscription plan,click,,"//span[normalize-space()='Customer Subscription Plan']"
+27.Verify Customer Subscription Plan Lists ,verify,,"//div[normalize-space()='Customer Subscription Plans']"
+28.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
+29.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+30.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
+31.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "//input[@placeholder='Plan Name']"
+32.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+33.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
+34.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
+35.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
+36.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No Of Free Rides']"
+37.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+38.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+39.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
+40.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
+41.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
+42.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+43.Select On,click,,"//li[@aria-label='on']"
+44.Click Submit ,click,,"//button[normalize-space()='Submit']"
+45.Filter Services List,type,{custometSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+46.wait,3000,,
+47.Load User App,switch_to,user,
+48.wait,2000,,
+49.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+50.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+52.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+53.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+54.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+55.wait,2000,,
+56.Enter Mobile Number,type,{userPhone},"//android.widget.EditText"
+57.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
+58.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+59.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+60.Click Finish,tap,,"//android.widget.Button[@content-desc="Finish"]"
+61.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
+62.Profile, tap_coordinate ,978:2224,COORDINATE_MODE
+63.Click Subscription,tap,,"//android.view.View[@content-desc="Subscription"]"
+64.Wait Customer Plan,wait_until_visible,,"//android.view.View[contains(@content-desc, '{customerSubscriptionName}')]"
+65.Click Customer Plan,tap,,"//android.view.View[contains(@content-desc, '{customerSubscriptionName}')]"
+66.wait,5000,,
+67.Load Driver App,switch_to,driver,
+68.wait,2000,,
+69.Click Allow Notification,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_button"]"
+70.Click Agree,tap,,"//android.widget.Button[@content-desc="Agree"]"
+71.Click Get Started,tap,,"//android.view.View[@content-desc="Get Started"]"
+72.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+73.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+74.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+75.Enter Mobile Number,type,{autoPhone},"//android.widget.EditText"
+76.Wait for Continue,wait_until_visible,,"//android.widget.Button[@content-desc="Continue"]"
+77.Click Continue,tap,,"//android.widget.Button[@content-desc="Continue"]"
+78.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+79.Click Allow Location,tap,,"//android.widget.Button[@resource-id="com.android.permissioncontroller:id/permission_allow_foreground_only_button"]"
+80.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+81.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+82.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+83.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+84.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+85.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+86.Drag Page Layout Upward,swipe,up,
+87.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+88.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+89.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+90.wait,3000,,
+91.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+92.Wait For OTP,wait_until_visible,,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+93.Enter OTP,type,123456,"//android.view.View[contains(@content-desc,'Verify Your Phone')]/../descendant::android.widget.EditText"
+94.Wait For Hamburger,wait_until_visible,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+95.Click Hamburge,tap,,"//android.view.View[@content-desc="Driver App"]/preceding-sibling::android.view.View"
+96.Click Subscription,tap,,"//android.view.View[@content-desc="Subscription"]"
+97.Wait Driver Plan,wait_until_visible,,"//android.view.View[contains(@content-desc, '{driverSubscriptionName}')]"
+98.Click Driver Plan,tap,,"//android.view.View[contains(@content-desc, '{driverSubscriptionName}')]"
+99.wait,10000,,</t>
   </si>
 </sst>
 </file>
@@ -1710,7 +1714,7 @@
         <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>36</v>
@@ -1934,7 +1938,7 @@
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>29</v>
@@ -2160,7 +2164,7 @@
         <v>47</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
42th Commit :Sheet Loop Running For Database Stress Test Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83CD3D17-167C-40E7-BE69-0769FB09B760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BCDDE57-385F-4FDC-9E76-765FB7F5716B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
-    <sheet name="SuperAdminLogin" sheetId="6" r:id="rId2"/>
+    <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
+    <sheet name="Rebooter" sheetId="34" r:id="rId2"/>
     <sheet name="AddAutoDriver" sheetId="32" r:id="rId3"/>
     <sheet name="AutoRideLifecycleTest" sheetId="35" r:id="rId4"/>
     <sheet name="AddCustomer" sheetId="36" r:id="rId5"/>
@@ -835,80 +835,6 @@
   </si>
   <si>
     <t>Customer</t>
-  </si>
-  <si>
-    <t>1. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-2.Click  Add Customers,click,,"//span[normalize-space()='Add Customers']"
-3. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
-4.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
-5.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
-6.Enter Contact Number, type, {randomPhone}&gt;&gt;userPhone,"//input[@type='tel']"
-7.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
-8.Open Gender,click,,"//span[@aria-label='select gender']"
-9.Select Male,click,,"//li[@aria-label='Male']"
-10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
-11.Click Submit, click, , "//button[normalize-space()='Submit']"
-12.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
-13. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-14. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
-15.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
-16. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-17.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-18.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-7. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-9. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
-10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-13.Select  Auto Option,click,,"//span[normalize-space()='Auto']"
-14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-15.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-17. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-18. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-19. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-20. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-21. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-22. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-23. Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-24. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-25. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-26. Click Submit, click, , "//button[contains(.,'Submit')]"
-27. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-28. Wait for Toast to hide, wait, 1000,
-29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-31.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-33.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-35. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-36.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-37.Add Driving License,click,,"//i[@title='Edit']"
-38.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-40.Click Submit, click, , "//button[normalize-space()='Submit']"
-41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-42.Click Approve Driver,click,,"//i[@title='Approve']"
-43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-43.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-47.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-48.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-50.Click Doc Icon,click,,"//i[@title='Document']"
-51.Click Eye Icon,click,,"//i[@title='View']"
-52.wait,1000,,</t>
   </si>
   <si>
     <t>TC_CA_04_add_customer</t>
@@ -1289,6 +1215,86 @@
 97.Wait Driver Plan,wait_until_visible,,"//android.view.View[contains(@content-desc, '{driverSubscriptionName}')]"
 98.Click Driver Plan,tap,,"//android.view.View[contains(@content-desc, '{driverSubscriptionName}')]"
 99.wait,10000,,</t>
+  </si>
+  <si>
+    <t>1.Click Dashboard  Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
+2. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+3.Click  Add Customers,click,,"//span[normalize-space()='Add Customers']"
+4. Verify Add Customer Heading,verify,,"//div[normalize-space()='Add Customer']"
+5.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "//label[contains(., 'Customer Full Name')]/following::input[1]"
+6.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "//input[@type='email']"
+7.Enter Contact Number, type, {randomPhone}&gt;&gt;userPhone,"//input[@type='tel']"
+8.Enter Video Call Limit, type, 60, "//label[contains(., 'User Used Video Call Limit in Minutes')]/following::input[1]"
+9.Open Gender,click,,"//span[@aria-label='select gender']"
+10.Select Male,click,,"//li[@aria-label='Male']"
+11.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "//input[@type='file' and @accept='image/*']"
+12.Click Submit, click, , "//button[normalize-space()='Submit']"
+13.Verify Added Succesfully, verify, , "//div[@aria-label='Info']"
+14. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+15. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
+16.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
+17. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
+18.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
+19.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6.wait,5000,,
+7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox//input[@type='checkbox']"
+8. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+9. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+10. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
+11.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+12.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
+13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+14.Select Source,click,,"//span[@aria-label='Select Source']"
+15.Select Instagram,click,,"//span[normalize-space()='From Instagramj']"
+16.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+17.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+18.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
+19. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+20.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
+21.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+22.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+23.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+24. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
+25. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+26. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+27.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+28.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+29. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+30. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+31. Click Submit, click, , "//button[contains(.,'Submit')]"
+32. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+33. Wait for Toast to hide, wait, 1000,
+34.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+35.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+36.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+37.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+38.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+39.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+40. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+41.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+42.Add Driving License,click,,"//i[@title='Edit']"
+43.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+44.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+45.Click Submit, click, , "//button[normalize-space()='Submit']"
+46.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+47.Click Approve Driver,click,,"//i[@title='Approve']"
+48.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+49.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+50.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+51.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+52.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+53.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+54.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+55.Click Doc Icon,click,,"//i[@title='Document']"
+56.Click Eye Icon,click,,"//i[@title='View']"
+57.wait,1000,,</t>
   </si>
 </sst>
 </file>
@@ -1660,6 +1666,82 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{452F96D9-3311-4A18-82B5-F5729925CB8A}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="26.6640625" customWidth="1"/>
+    <col min="5" max="5" width="53.21875" customWidth="1"/>
+    <col min="6" max="6" width="36.88671875" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC5AE23A-69EB-46F0-86E8-8B9CD1BA86DE}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1714,86 +1796,10 @@
         <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{452F96D9-3311-4A18-82B5-F5729925CB8A}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="26.6640625" customWidth="1"/>
-    <col min="5" max="5" width="53.21875" customWidth="1"/>
-    <col min="6" max="6" width="36.88671875" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1938,7 +1944,7 @@
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>29</v>
@@ -2010,13 +2016,13 @@
         <v>39</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>37</v>
@@ -2079,19 +2085,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>22</v>
@@ -2152,22 +2158,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
45th Commit : Auto Ride Booking Test Started
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83BC08C6-E44E-444B-9C8A-CF70BE5A4623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B86D7CFE-E530-4813-A4D8-03098758AC04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
     <sheet name="RebooterAccess" sheetId="39" r:id="rId2"/>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId3"/>
     <sheet name="AddAutoDriver" sheetId="32" r:id="rId4"/>
-    <sheet name="AutoRideLifecycleTest" sheetId="35" r:id="rId5"/>
+    <sheet name="ApprovedAutoDriver" sheetId="38" r:id="rId5"/>
     <sheet name="AddCustomer" sheetId="36" r:id="rId6"/>
-    <sheet name="ApprovedAutoDriver" sheetId="38" r:id="rId7"/>
-    <sheet name="SubscriptionPlanCheck" sheetId="37" r:id="rId8"/>
-    <sheet name="SubscriptionPlanAccess" sheetId="40" r:id="rId9"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId10"/>
+    <sheet name="AutoRideLifecycleTest" sheetId="35" r:id="rId7"/>
+    <sheet name="AutoRideAccessTest" sheetId="41" r:id="rId8"/>
+    <sheet name="SubscriptionPlanCheck" sheetId="37" r:id="rId9"/>
+    <sheet name="SubscriptionPlanAccess" sheetId="40" r:id="rId10"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId11"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="66">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -564,43 +565,6 @@
     </r>
   </si>
   <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6. Click Checkbox, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-7. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-8. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-9. Enter Contact Number, type, {randomPhone}&gt;&gt;autoMobile, "//input[@type='tel']"
-10. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-11. Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-12.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-13.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
-14. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-15.Enter Vehicle Company, type, autoCompany{randomAlpha}&gt;&gt; autoCompanyName, "//label[contains(.,'Vehicle Company')]/following::input[1]"
-16. Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-17. Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-18. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-19. Enter Vehicle Color, type, Red, "//label[contains(.,'Vehicle Color')]/following::input[1]"
-20. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-21. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-22. Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-23. Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-24. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-25. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-26. Click Submit, click, , "//button[contains(.,'Submit')]"
-27. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-28. Wait for Toast to hide, wait, 1000,
-29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-31.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-33.wait,1000,,
-34.Click  Dashboard Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
-35.wait,1000,,</t>
-  </si>
-  <si>
     <t>SA_TS_00</t>
   </si>
   <si>
@@ -828,9 +792,6 @@
   </si>
   <si>
     <t>SA_TS_7</t>
-  </si>
-  <si>
-    <t>TC_CA_07_Subscription_Plan_Test</t>
   </si>
   <si>
     <t>This comprehensive end-to-end hybrid test validates the configuration and onboarding lifecycle of the ABCD Framework by creating distinct Driver and Customer Subscription Plans via the Super Admin portal. The execution then transitions to mobile applications, logging into the User App and Driver App using the exact mobile numbers registered during creation. The test concludes by navigating into each respective mobile app's profile layout to successfully verify that the newly generated subscription plans are correctly existing and visible under each platform interface.</t>
@@ -1240,19 +1201,10 @@
     <t>TC_CA_04_Autoride_Lifecycle_Test</t>
   </si>
   <si>
-    <t>TC_CA_05_add_customer</t>
-  </si>
-  <si>
     <t>SA_TS_6</t>
   </si>
   <si>
-    <t>TC_CA_06_add_approved_auto_driver</t>
-  </si>
-  <si>
     <t>SA_TS_8</t>
-  </si>
-  <si>
-    <t>TC_CA_08_test_data_cleanup</t>
   </si>
   <si>
     <t>1.wait,3000,,
@@ -1275,66 +1227,6 @@
 18.wait,1000,,
 19.Load  Super Admin,switch_to,web,
 20.wait,2000,,</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6.wait,3000,,
-7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-8. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-9. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-10. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
-11.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-12.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
-13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-14.Select Source,click,,"//span[@aria-label='Select Source']"
-15.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
-16.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-17.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-18.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
-19. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-20.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-21.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-22.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-25.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-26.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-27. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-29. Click Submit, click, , "//button[contains(.,'Submit')]"
-30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-31. Wait for Toast to hide, wait, 1000,
-32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-36.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-37.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-38. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-39.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-40.Add Driving License,click,,"//i[@title='Edit']"
-41.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-42.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-43.Click Submit, click, , "//button[normalize-space()='Submit']"
-44.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-45.Click Approve Driver,click,,"//i[@title='Approve']"
-46.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-47.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-49.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-50.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-51.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-52.Scroll Grid, tab, 10, "//input[@aria-label='Driver Name Filter Input']"
-53.Click Doc Icon,click,,"//i[@title='Document']"
-54.Click Eye Icon,click,,"//i[@title='View']"
-55.wait,1000,,</t>
-  </si>
-  <si>
-    <t>TC_CA_08_Subscription_Plan_Access_Test</t>
   </si>
   <si>
     <t>This comprehensive end-to-end hybrid test validates the configuration and onboarding lifecycle of the ABCD Framework by creating distinct Driver and Customer Subscription Plans via the Super Admin portal. The execution then transitions to mobile applications, logging into the User App and Driver App using the exact mobile numbers registered during creation. The test concludes by navigating into each respective mobile app's profile layout to successfully verify that the newly generated subscription plans are correctly existing and visible under each platform interface.This test case uses accessibility id instead of xpath for mobile automation</t>
@@ -1437,6 +1329,336 @@
 95.Wait Driver Plan,wait_until_visible,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
 96.Click Driver Plan,tap,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
 97.wait,5000,,</t>
+  </si>
+  <si>
+    <t>TC_CA_05_Autoride_Access_Test</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_customer</t>
+  </si>
+  <si>
+    <t>TC_CA_07_add_approved_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_08_Subscription_Plan_Test</t>
+  </si>
+  <si>
+    <t>SA_TS_9</t>
+  </si>
+  <si>
+    <t>TC_CA_09_Subscription_Plan_Access_Test</t>
+  </si>
+  <si>
+    <t>SA_TS_10</t>
+  </si>
+  <si>
+    <t>TC_CA_10_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6.wait,3000,,
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+8. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+9. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+10. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
+11.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+12.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
+13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+14.Select Source,click,,"//span[@aria-label='Select Source']"
+15.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
+16.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+17.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+18.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
+19. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+20.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+21.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+22.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+25.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+26.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+27. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+29. Click Submit, click, , "//button[contains(.,'Submit')]"
+30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+31. Wait for Toast to hide, wait, 1000,
+32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+36.wait,1000,,
+37.Click  Dashboard Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
+38.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6.wait,3000,,
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+8. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+9. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+10. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
+11.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+12.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
+13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+14.Select Source,click,,"//span[@aria-label='Select Source']"
+15.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
+16.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+17.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+18.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
+19. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+20.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+21.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+22.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+25.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+26.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+27. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+29. Click Submit, click, , "//button[contains(.,'Submit')]"
+30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+31. Wait for Toast to hide, wait, 1000,
+32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+36.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+37.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+38. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+39.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+40.Add Driving License,click,,"//i[@title='Edit']"
+41.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+42.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+43.Click Submit, click, , "//button[normalize-space()='Submit']"
+44.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+45.Click Approve Driver,click,,"//i[@title='Approve']"
+46.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+47.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+49.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+50.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+51.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+52.Scroll Grid, tab, 10, "//input[@aria-label='Driver Name Filter Input']"
+53.Click Doc Icon,click,,"//i[@title='Document']"
+54.Click Eye Icon,click,,"//i[@title='View']"
+55.wait,1000,,</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin and AddAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SuperAdminLogin,AddCustomer,AddAutoDriver
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
+    <t>1.Load Driver App,switch_to,driver,
+2.Wait For Notification,wait_until_visible,,"id=com.android.permissioncontroller:id/permission_allow_button"
+3.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+4.Click Agree,tap,,"accessibility=Agree"
+5.Click Get Started,tap,,"accessibility=Get Started"
+6.Click Next,tap,,"accessibility=Next"
+7.Click Mobile Number,tap,,"accessibility=Mobile Number"
+8.Click Close,tap,,"accessibility=Cancel"
+9.Enter Mobile Number,type,{autoPhone},"automator=new UiSelector().className("android.widget.EditText")"
+10.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+11.Click Continue,tap,,"accessibility=Continue"
+12.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+13.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+14.wait,3000,,
+15.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+16.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+17.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+18.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+19.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+20.Drag Page Layout Upward,swipe,up,
+21.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+22.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+23.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+24.wait,3000,,
+25.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+26.Wait For OTP,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
+27.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+28.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+29.Click Document,tap,,"accessibility=Documents"
+30.Click Upload,tap,,"accessibility=Upload"
+31.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","accessibility=Upload Documents"
+32.Click Sort,tap_coordinate ,776:313,COORDINATE_MODE
+33.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
+34.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
+35.Click Crop,tap,,"accessibility=Crop"
+36.Click Calender,tap_coordinate ,123:1627,COORDINATE_MODE
+37..Click Month,tap,"accessibility=Next month"
+38.Click Date,tap_coordinate ,922:1381,COORDINATE_MODE
+39.Click Ok,tap,,"accessibility=OK"
+40.Click Upload,tap,,"accessibility=Upload Documents"
+41.Wait For Back,wait_until_visible,,"accessibility=Back"
+42.Click Back,tap,,"accessibility=Back"
+43.Click Back,tap,,"accessibility=Back"
+44.Load Admin App,switch_to,web,
+45.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+46.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+47.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+48.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+50.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+51.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+52.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+53.Click Approve Driver,click,,"//i[@title='Approve']"
+54.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+55.wait,3000,,
+56.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+57.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+58.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+59.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+60.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+61.wait,2000,,
+62.Load Driver App,switch_to,driver,
+63.wait,2000,,
+64.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+65.Click Document,tap,,"accessibility=Documents"
+66.Wait For Back,wait_until_visible,,"accessibility=Back"
+67.Click Back,tap,,"accessibility=Back"
+68.Click Back,tap,,"accessibility=Back"
+69.Click Online,tap_coordinate,989:2045,
+70.wait,3000,,
+71.Load User App,switch_to,user,
+72.wait,2000,,
+73.Click Get Started,tap,,"accessibility=Get Started"
+74.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+75.Click Next,tap,,"accessibility=Next"
+76.Click Mobile Number,tap,,"accessibility=Mobile Number"
+77.Click Close,tap,,"accessibility=Cancel"
+78.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
+79.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+80.Click Continue,tap,,"accessibility=Continue"
+81.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+82.Click Finish,tap,,"accessibility=Finish"
+83.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+84.wait,2000,,
+85.Click Auto Ride,tap,,"accessibility=Auto Ride"
+86.Enter Destination, type, Parsn Manare, "automator=new UiSelector().descriptionContains("Drop Location")"
+87.wait,3000,,
+88.Select Destination, tap ,, "automator=new UiSelector().description("0.1 km Parsn Manere, Gangai Karai Puram, T. Nagar, Chennai, Tamil Nadu Gangai Karai Puram, T. Nagar, Chennai, Tamil Nadu")"
+89.Click Confirm,tap,,"accessibility=Confirm"
+90.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
+91.Ride Now,tap,,"accessibility=Ride Now"
+92.wait,3000,,</t>
   </si>
 </sst>
 </file>
@@ -1850,22 +2072,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1884,6 +2106,84 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA5DCFAC-B912-41EA-9964-A3839A72D798}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1925,13 +2225,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>15</v>
@@ -2000,22 +2300,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2082,7 +2382,7 @@
         <v>17</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>12</v>
@@ -2157,13 +2457,13 @@
         <v>19</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
@@ -2182,25 +2482,24 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B79BE6A4-9FA5-4B28-B734-40C3B7520402}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8946E02E-8751-499F-BD67-2B828D4C435E}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="4" max="4" width="35.5546875" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -2222,24 +2521,24 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>50</v>
+        <v>35</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>56</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2247,12 +2546,7 @@
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="E3" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2302,22 +2596,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2336,24 +2630,25 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8946E02E-8751-499F-BD67-2B828D4C435E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B79BE6A4-9FA5-4B28-B734-40C3B7520402}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="30.88671875" customWidth="1"/>
-    <col min="4" max="4" width="35.5546875" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="29.6640625" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -2375,24 +2670,24 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>53</v>
+        <v>10</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2400,7 +2695,12 @@
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="7"/>
+      <c r="E3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2408,6 +2708,84 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAC49636-EBC0-4581-9799-1B4190D9E9BA}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="8" max="8" width="15.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF6BCA45-0614-4137-B63C-BCC5F13F9786}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2450,22 +2828,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2474,85 +2852,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA5DCFAC-B912-41EA-9964-A3839A72D798}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>

</xml_diff>

<commit_message>
46th Commit : Auto Ride Booking Test Stage One
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B86D7CFE-E530-4813-A4D8-03098758AC04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C01A4B9-B4B4-4C2C-89FC-2FAC734602F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1652,13 +1652,18 @@
 83.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
 84.wait,2000,,
 85.Click Auto Ride,tap,,"accessibility=Auto Ride"
-86.Enter Destination, type, Parsn Manare, "automator=new UiSelector().descriptionContains("Drop Location")"
+86.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
 87.wait,3000,,
 88.Select Destination, tap ,, "automator=new UiSelector().description("0.1 km Parsn Manere, Gangai Karai Puram, T. Nagar, Chennai, Tamil Nadu Gangai Karai Puram, T. Nagar, Chennai, Tamil Nadu")"
 89.Click Confirm,tap,,"accessibility=Confirm"
 90.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
 91.Ride Now,tap,,"accessibility=Ride Now"
-92.wait,3000,,</t>
+92.wait,2000,,
+93.Load Driver App,switch_to,driver,
+94.wait,2000,,
+95.Wait for Accept,wait_until_visible,,"automator=new UiSelector().description("Accept Accept")"
+96.Accept Ride,tap,,"automator=new UiSelector().description("Accept Accept")"
+97.wait,2000,,</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
47th Commit : Auto Ride Booking Test Stage One Updated
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C01A4B9-B4B4-4C2C-89FC-2FAC734602F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B16D4C8-EA99-4011-9670-54DA1FA9F90A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -1232,6 +1232,242 @@
     <t>This comprehensive end-to-end hybrid test validates the configuration and onboarding lifecycle of the ABCD Framework by creating distinct Driver and Customer Subscription Plans via the Super Admin portal. The execution then transitions to mobile applications, logging into the User App and Driver App using the exact mobile numbers registered during creation. The test concludes by navigating into each respective mobile app's profile layout to successfully verify that the newly generated subscription plans are correctly existing and visible under each platform interface.This test case uses accessibility id instead of xpath for mobile automation</t>
   </si>
   <si>
+    <t>TC_CA_05_Autoride_Access_Test</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_customer</t>
+  </si>
+  <si>
+    <t>TC_CA_07_add_approved_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_08_Subscription_Plan_Test</t>
+  </si>
+  <si>
+    <t>SA_TS_9</t>
+  </si>
+  <si>
+    <t>TC_CA_09_Subscription_Plan_Access_Test</t>
+  </si>
+  <si>
+    <t>SA_TS_10</t>
+  </si>
+  <si>
+    <t>TC_CA_10_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6.wait,3000,,
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+8. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+9. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+10. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
+11.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+12.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
+13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+14.Select Source,click,,"//span[@aria-label='Select Source']"
+15.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
+16.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+17.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+18.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
+19. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+20.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+21.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+22.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+25.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+26.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+27. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+29. Click Submit, click, , "//button[contains(.,'Submit')]"
+30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+31. Wait for Toast to hide, wait, 1000,
+32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+36.wait,1000,,
+37.Click  Dashboard Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
+38.wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6.wait,3000,,
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+8. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+9. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+10. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
+11.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+12.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
+13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+14.Select Source,click,,"//span[@aria-label='Select Source']"
+15.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
+16.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+17.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+18.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
+19. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+20.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+21.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+22.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+25.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+26.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+27. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+29. Click Submit, click, , "//button[contains(.,'Submit')]"
+30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+31. Wait for Toast to hide, wait, 1000,
+32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+36.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+37.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+38. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+39.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+40.Add Driving License,click,,"//i[@title='Edit']"
+41.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+42.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+43.Click Submit, click, , "//button[normalize-space()='Submit']"
+44.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+45.Click Approve Driver,click,,"//i[@title='Approve']"
+46.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+47.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+49.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+50.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+51.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+52.Scroll Grid, tab, 10, "//input[@aria-label='Driver Name Filter Input']"
+53.Click Doc Icon,click,,"//i[@title='Document']"
+54.Click Eye Icon,click,,"//i[@title='View']"
+55.wait,1000,,</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin and AddAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SuperAdminLogin,AddCustomer,AddAutoDriver
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
 2.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
 3.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
@@ -1324,247 +1560,12 @@
 90.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
 91.Wait For OTP,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
 92.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-93.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-94.Click Subscription,tap,,"accessibility=Subscription"
-95.Wait Driver Plan,wait_until_visible,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
-96.Click Driver Plan,tap,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
-97.wait,5000,,</t>
-  </si>
-  <si>
-    <t>TC_CA_05_Autoride_Access_Test</t>
-  </si>
-  <si>
-    <t>TC_CA_06_add_customer</t>
-  </si>
-  <si>
-    <t>TC_CA_07_add_approved_auto_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_08_Subscription_Plan_Test</t>
-  </si>
-  <si>
-    <t>SA_TS_9</t>
-  </si>
-  <si>
-    <t>TC_CA_09_Subscription_Plan_Access_Test</t>
-  </si>
-  <si>
-    <t>SA_TS_10</t>
-  </si>
-  <si>
-    <t>TC_CA_10_test_data_cleanup</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6.wait,3000,,
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-8. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-9. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-10. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
-11.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-12.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
-13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-14.Select Source,click,,"//span[@aria-label='Select Source']"
-15.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
-16.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-17.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-18.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
-19. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-20.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-21.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-22.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-25.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-26.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-27. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-29. Click Submit, click, , "//button[contains(.,'Submit')]"
-30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-31. Wait for Toast to hide, wait, 1000,
-32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-36.wait,1000,,
-37.Click  Dashboard Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
-38.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6.wait,3000,,
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-8. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-9. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-10. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
-11.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-12.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
-13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-14.Select Source,click,,"//span[@aria-label='Select Source']"
-15.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
-16.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-17.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-18.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
-19. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-20.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-21.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-22.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-25.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-26.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-27. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-29. Click Submit, click, , "//button[contains(.,'Submit')]"
-30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-31. Wait for Toast to hide, wait, 1000,
-32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-36.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-37.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-38. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-39.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-40.Add Driving License,click,,"//i[@title='Edit']"
-41.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-42.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-43.Click Submit, click, , "//button[normalize-space()='Submit']"
-44.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-45.Click Approve Driver,click,,"//i[@title='Approve']"
-46.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-47.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-49.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-50.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-51.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-52.Scroll Grid, tab, 10, "//input[@aria-label='Driver Name Filter Input']"
-53.Click Doc Icon,click,,"//i[@title='Document']"
-54.Click Eye Icon,click,,"//i[@title='View']"
-55.wait,1000,,</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The SuperAdminLogin and AddAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RunSheet:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">SuperAdminLogin,AddCustomer,AddAutoDriver
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
-    </r>
+93.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
+94.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+95.Click Subscription,tap,,"accessibility=Subscription"
+96.Wait Driver Plan,wait_until_visible,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
+97.Click Driver Plan,tap,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
+98.wait,5000,,</t>
   </si>
   <si>
     <t>1.Load Driver App,switch_to,driver,
@@ -1594,76 +1595,78 @@
 25.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
 26.Wait For OTP,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
 27.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-28.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-29.Click Document,tap,,"accessibility=Documents"
-30.Click Upload,tap,,"accessibility=Upload"
-31.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","accessibility=Upload Documents"
-32.Click Sort,tap_coordinate ,776:313,COORDINATE_MODE
-33.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
-34.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
-35.Click Crop,tap,,"accessibility=Crop"
-36.Click Calender,tap_coordinate ,123:1627,COORDINATE_MODE
-37..Click Month,tap,"accessibility=Next month"
-38.Click Date,tap_coordinate ,922:1381,COORDINATE_MODE
-39.Click Ok,tap,,"accessibility=OK"
-40.Click Upload,tap,,"accessibility=Upload Documents"
-41.Wait For Back,wait_until_visible,,"accessibility=Back"
-42.Click Back,tap,,"accessibility=Back"
+28.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
+29.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+30.Click Document,tap,,"accessibility=Documents"
+31.Click Upload,tap,,"accessibility=Upload"
+32.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","accessibility=Upload Documents"
+33.Click Sort,tap_coordinate ,776:313,COORDINATE_MODE
+34.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
+35.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
+36.Click Crop,tap,,"accessibility=Crop"
+37.Click Calender,tap_coordinate ,123:1627,COORDINATE_MODE
+38..Click Month,tap,"accessibility=Next month"
+39.Click Date,tap_coordinate ,922:1381,COORDINATE_MODE
+40.Click Ok,tap,,"accessibility=OK"
+41.Click Upload,tap,,"accessibility=Upload Documents"
+42.Wait For Back,wait_until_visible,,"accessibility=Back"
 43.Click Back,tap,,"accessibility=Back"
-44.Load Admin App,switch_to,web,
-45.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-46.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-47.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-48.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-49.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-50.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-51.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-52.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-53.Click Approve Driver,click,,"//i[@title='Approve']"
-54.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-55.wait,3000,,
-56.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+44.Click Back,tap,,"accessibility=Back"
+45.Load Admin App,switch_to,web,
+46.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+47.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+48.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+49.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+50.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+51.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+52.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+53.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+54.Click Approve Driver,click,,"//i[@title='Approve']"
+55.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+56.wait,3000,,
 57.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-58.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-59.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-60.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-61.wait,2000,,
-62.Load Driver App,switch_to,driver,
-63.wait,2000,,
-64.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-65.Click Document,tap,,"accessibility=Documents"
-66.Wait For Back,wait_until_visible,,"accessibility=Back"
-67.Click Back,tap,,"accessibility=Back"
-68.Click Back,tap,,"accessibility=Back"
-69.Click Online,tap_coordinate,989:2045,
-70.wait,3000,,
-71.Load User App,switch_to,user,
-72.wait,2000,,
-73.Click Get Started,tap,,"accessibility=Get Started"
-74.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
-75.Click Next,tap,,"accessibility=Next"
-76.Click Mobile Number,tap,,"accessibility=Mobile Number"
-77.Click Close,tap,,"accessibility=Cancel"
-78.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
-79.Wait for Continue,wait_until_visible,,"accessibility=Continue"
-80.Click Continue,tap,,"accessibility=Continue"
-81.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-82.Click Finish,tap,,"accessibility=Finish"
-83.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
-84.wait,2000,,
-85.Click Auto Ride,tap,,"accessibility=Auto Ride"
-86.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
-87.wait,3000,,
-88.Select Destination, tap ,, "automator=new UiSelector().description("0.1 km Parsn Manere, Gangai Karai Puram, T. Nagar, Chennai, Tamil Nadu Gangai Karai Puram, T. Nagar, Chennai, Tamil Nadu")"
-89.Click Confirm,tap,,"accessibility=Confirm"
-90.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
-91.Ride Now,tap,,"accessibility=Ride Now"
-92.wait,2000,,
-93.Load Driver App,switch_to,driver,
+58.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+59.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+60.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+61.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+62.wait,2000,,
+63.Load Driver App,switch_to,driver,
+64.wait,2000,,
+65.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
+66.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+67.Click Document,tap,,"accessibility=Documents"
+68.Wait For Back,wait_until_visible,,"accessibility=Back"
+69.Click Back,tap,,"accessibility=Back"
+70.Click Back,tap,,"accessibility=Back"
+71.Click Online,tap_coordinate,989:2045,
+72.wait,3000,,
+73.Load User App,switch_to,user,
+74.wait,2000,,
+75.Click Get Started,tap,,"accessibility=Get Started"
+76.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+77.Click Next,tap,,"accessibility=Next"
+78.Click Mobile Number,tap,,"accessibility=Mobile Number"
+79.Click Close,tap,,"accessibility=Cancel"
+80.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
+81.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+82.Click Continue,tap,,"accessibility=Continue"
+83.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+84.Click Finish,tap,,"accessibility=Finish"
+85.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+86.wait,2000,,
+87.Click Auto Ride,tap,,"accessibility=Auto Ride"
+88.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
+89.wait,3000,,
+90.Select Destination, tap ,, "automator=new UiSelector().description("0.1 km Parsn Manere, Gangai Karai Puram, T. Nagar, Chennai, Tamil Nadu Gangai Karai Puram, T. Nagar, Chennai, Tamil Nadu")"
+91.Click Confirm,tap,,"accessibility=Confirm"
+92.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
+93.Ride Now,tap,,"accessibility=Ride Now"
 94.wait,2000,,
-95.Wait for Accept,wait_until_visible,,"automator=new UiSelector().description("Accept Accept")"
-96.Accept Ride,tap,,"automator=new UiSelector().description("Accept Accept")"
-97.wait,2000,,</t>
+95.Load Driver App,switch_to,driver,
+96.wait,2000,,
+97.Wait for Accept,wait_until_visible,,"automator=new UiSelector().description("Accept Accept")"
+98.Accept Ride,tap,,"automator=new UiSelector().description("Accept Accept")"
+99.wait,2000,,</t>
   </si>
 </sst>
 </file>
@@ -2153,19 +2156,19 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>37</v>
@@ -2230,13 +2233,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>15</v>
@@ -2468,7 +2471,7 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
@@ -2534,13 +2537,13 @@
         <v>19</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
@@ -2607,7 +2610,7 @@
         <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>
@@ -2761,7 +2764,7 @@
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
@@ -2770,7 +2773,7 @@
         <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2839,7 +2842,7 @@
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
49th Commit : Auto Ride Booking Test Suite Updated
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4414F07B-C8B7-49AB-822A-C16A3E0811A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7906DE6D-3D1C-44C1-81B6-7D72D2872048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1664,7 +1664,7 @@
 94.wait,2000,,
 95.Load Driver App,switch_to,driver,
 96.wait,2000,,
-97.Wait for Accept,wait_until_visible,,"automator=new UiSelector().description("Accept Accept")"
+97.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
 98.Accept Ride,tap,,"automator=new UiSelector().description("Accept Accept")"
 99.wait,2000,,
 100.Ride Arrived,tap,,"accessibility=Arrived"

</xml_diff>

<commit_message>
51th Commit : Removed Forced Waits From Timesheets
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C4FE79-6653-4227-948C-53F6EDA1D7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{576409A5-8081-4212-AB28-F4178FA7CD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1159,6 +1159,173 @@
 99.wait,10000,,</t>
   </si>
   <si>
+    <t>SA_TS_01</t>
+  </si>
+  <si>
+    <t>Rebooter Access Test</t>
+  </si>
+  <si>
+    <t>TC_CA_01_Reboot_Access_Test</t>
+  </si>
+  <si>
+    <t>If in case emulators crashes wipe data and  cold reboot all emulators and run this test to make the emultators and web browser into initial state before running other tests.This test uses access id instead of xpath for mobile testing.</t>
+  </si>
+  <si>
+    <t>TC_CA_02_super_admin_login</t>
+  </si>
+  <si>
+    <t>TC_CA_03_add_verify_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_04_Autoride_Lifecycle_Test</t>
+  </si>
+  <si>
+    <t>SA_TS_6</t>
+  </si>
+  <si>
+    <t>SA_TS_8</t>
+  </si>
+  <si>
+    <t>This comprehensive end-to-end hybrid test validates the configuration and onboarding lifecycle of the ABCD Framework by creating distinct Driver and Customer Subscription Plans via the Super Admin portal. The execution then transitions to mobile applications, logging into the User App and Driver App using the exact mobile numbers registered during creation. The test concludes by navigating into each respective mobile app's profile layout to successfully verify that the newly generated subscription plans are correctly existing and visible under each platform interface.This test case uses accessibility id instead of xpath for mobile automation</t>
+  </si>
+  <si>
+    <t>TC_CA_05_Autoride_Access_Test</t>
+  </si>
+  <si>
+    <t>TC_CA_06_add_customer</t>
+  </si>
+  <si>
+    <t>TC_CA_07_add_approved_auto_driver</t>
+  </si>
+  <si>
+    <t>TC_CA_08_Subscription_Plan_Test</t>
+  </si>
+  <si>
+    <t>SA_TS_9</t>
+  </si>
+  <si>
+    <t>TC_CA_09_Subscription_Plan_Access_Test</t>
+  </si>
+  <si>
+    <t>SA_TS_10</t>
+  </si>
+  <si>
+    <t>TC_CA_10_test_data_cleanup</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The SuperAdminLogin and AddAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">SuperAdminLogin,AddCustomer,AddAutoDriver
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
     <t>1.Click Dashboard  Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
 2. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
 3.Click  Add Customers,click,,"//span[normalize-space()='Add Customers']"
@@ -1176,166 +1343,105 @@
 15. Click Customer  Icon,click,,"//i[@class='fa-solid fa-users fas iconstyle']"
 16.Click  Verified Customers,click,,"//span[normalize-space()='Verified Customers']"
 17. Verify Verified Customer List Heading,verify,,"//div[normalize-space()='Verified Customer List']"
-18.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"
-19.wait,1000,,</t>
-  </si>
-  <si>
-    <t>SA_TS_01</t>
-  </si>
-  <si>
-    <t>Rebooter Access Test</t>
-  </si>
-  <si>
-    <t>TC_CA_01_Reboot_Access_Test</t>
-  </si>
-  <si>
-    <t>If in case emulators crashes wipe data and  cold reboot all emulators and run this test to make the emultators and web browser into initial state before running other tests.This test uses access id instead of xpath for mobile testing.</t>
-  </si>
-  <si>
-    <t>TC_CA_02_super_admin_login</t>
-  </si>
-  <si>
-    <t>TC_CA_03_add_verify_auto_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_04_Autoride_Lifecycle_Test</t>
-  </si>
-  <si>
-    <t>SA_TS_6</t>
-  </si>
-  <si>
-    <t>SA_TS_8</t>
-  </si>
-  <si>
-    <t>1.wait,3000,,
-2.Load User App,switch_to,user,
-3.wait,2000,,
-4.Click Get Started,tap,,"accessibility=Get Started"
-5.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
-6.Click Next,tap,,"accessibility=Next"
-7.Click Mobile Number,tap,,"accessibility=Mobile Number"
-8.Click Close,tap,,"accessibility=Cancel"
-9.wait,2000,,
-10.Load Driver App,switch_to,driver,
-11.wait,2000,,
-12.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
-13.Click Agree,tap,,"accessibility=Agree"
-14.Click Get Started,tap,,"accessibility=Get Started"
-15.Click Next,tap,,"accessibility=Next"
-16.Click Mobile Number,tap,,"accessibility=Mobile Number"
-17.Click Close,tap,,"accessibility=Cancel"
-18.wait,1000,,
-19.Load  Super Admin,switch_to,web,
-20.wait,2000,,</t>
-  </si>
-  <si>
-    <t>This comprehensive end-to-end hybrid test validates the configuration and onboarding lifecycle of the ABCD Framework by creating distinct Driver and Customer Subscription Plans via the Super Admin portal. The execution then transitions to mobile applications, logging into the User App and Driver App using the exact mobile numbers registered during creation. The test concludes by navigating into each respective mobile app's profile layout to successfully verify that the newly generated subscription plans are correctly existing and visible under each platform interface.This test case uses accessibility id instead of xpath for mobile automation</t>
-  </si>
-  <si>
-    <t>TC_CA_05_Autoride_Access_Test</t>
-  </si>
-  <si>
-    <t>TC_CA_06_add_customer</t>
-  </si>
-  <si>
-    <t>TC_CA_07_add_approved_auto_driver</t>
-  </si>
-  <si>
-    <t>TC_CA_08_Subscription_Plan_Test</t>
-  </si>
-  <si>
-    <t>SA_TS_9</t>
-  </si>
-  <si>
-    <t>TC_CA_09_Subscription_Plan_Access_Test</t>
-  </si>
-  <si>
-    <t>SA_TS_10</t>
-  </si>
-  <si>
-    <t>TC_CA_10_test_data_cleanup</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+18.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
 3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
 4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
 5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6.wait,3000,,
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-8. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-9. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-10. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
-11.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-12.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
-13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-14.Select Source,click,,"//span[@aria-label='Select Source']"
-15.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
-16.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-17.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-18.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
-19. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-20.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-21.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-22.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-25.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-26.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-27. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-29. Click Submit, click, , "//button[contains(.,'Submit')]"
-30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-31. Wait for Toast to hide, wait, 1000,
-32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+6.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+7.Wait for Auto Ride,wait_until_visible,,"//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+8.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+9. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+10. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+11. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
+12.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+13.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
+14.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+15.Select Source,click,,"//span[@aria-label='Select Source']"
+16.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
+17.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+19.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
+20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+21.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+22.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+23.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+24. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+25. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+26.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+27.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+28. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+29. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+30. Click Submit, click, , "//button[contains(.,'Submit')]"
+31. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+32. Wait for Toast to hide, wait, 1000,
 33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-36.wait,1000,,
+34.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+35.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+36.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
 37.Click  Dashboard Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
-38.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+</t>
+  </si>
+  <si>
+    <t>1.Load User App,switch_to,user,
+2.Wait For Get Started,wait_until_visible,,"accessibility=Get Started"
+3.Click Get Started,tap,,"accessibility=Get Started"
+4.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+5.Click Next,tap,,"accessibility=Next"
+6.Click Mobile Number,tap,,"accessibility=Mobile Number"
+7.Click Close,tap,,"accessibility=Cancel"
+8.Load Driver App,switch_to,driver,
+9.Wait For Notification,wait_until_visible,,"id=com.android.permissioncontroller:id/permission_allow_button"
+10.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+11.Click Agree,tap,,"accessibility=Agree"
+12.Click Get Started,tap,,"accessibility=Get Started"
+13.Click Next,tap,,"accessibility=Next"
+14.Click Mobile Number,tap,,"accessibility=Mobile Number"
+15.Click Close,tap,,"accessibility=Cancel"
+16.Load  Super Admin,switch_to,web,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
 3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
 4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
 5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6.wait,3000,,
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-7.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-8. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-9. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-10. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
-11.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-12.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
-13. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-14.Select Source,click,,"//span[@aria-label='Select Source']"
-15.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
-16.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-17.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-18.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
-19. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-20.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-21.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-22.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-23. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-24. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-25.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-26.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-27. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-28. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-29. Click Submit, click, , "//button[contains(.,'Submit')]"
-30. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-31. Wait for Toast to hide, wait, 1000,
+6.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+7.Wait for Auto Ride,wait_until_visible,,"//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+8.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+9. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+10. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+11. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
+12.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+13.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
+14.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+15.Select Source,click,,"//span[@aria-label='Select Source']"
+16.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
+17.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+19.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
+20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+21.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+22.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+23.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+24. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+25. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+26.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+27.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+28. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+29. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+30. Click Submit, click, , "//button[contains(.,'Submit')]"
+31. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
 32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
 35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
 36.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
 37.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-38. Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+38.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
 39.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
 40.Add Driving License,click,,"//i[@title='Edit']"
 41.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
@@ -1349,123 +1455,7 @@
 49.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
 50.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
 51.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-52.Scroll Grid, tab, 10, "//input[@aria-label='Driver Name Filter Input']"
-53.Click Doc Icon,click,,"//i[@title='Document']"
-54.Click Eye Icon,click,,"//i[@title='View']"
-55.wait,1000,,</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The SuperAdminLogin and AddAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RunSheet:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">SuperAdminLogin,AddCustomer,AddAutoDriver
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
-    </r>
+</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
@@ -1491,81 +1481,77 @@
 21.Select On,click,,"//li[@aria-label='on']"
 22.Click Submit ,click,,"//button[normalize-space()='Submit']"
 23.Filter Services List,type,{driverSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-24.wait,2000,,
-25.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
-26.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
-27.Click Customer subscription plan,click,,"//span[normalize-space()='Customer Subscription Plan']"
-28.Verify Customer Subscription Plan Lists ,verify,,"//div[normalize-space()='Customer Subscription Plans']"
-29.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
-30.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
-31.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
-32.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "//input[@placeholder='Plan Name']"
-33.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
-34.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
-35.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
-36.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
-37.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No Of Free Rides']"
-38.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
-39.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
-40.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
-41.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
-42.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
-43.Open status Dropdown,click,,"//span[@aria-label='select Status']"
-44.Select On,click,,"//li[@aria-label='on']"
-45.Click Submit ,click,,"//button[normalize-space()='Submit']"
-46.Filter Services List,type,{custometSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
-47.wait,3000,,
-48.Load User App,switch_to,user,
-49.wait,2000,,
-50.Click Get Started,tap,,"accessibility=Get Started"
-51.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
-52.Click Next,tap,,"accessibility=Next"
-53.Click Mobile Number,tap,,"accessibility=Mobile Number"
-54.Click Close,tap,,"accessibility=Cancel"
-55.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
-56.Wait for Continue,wait_until_visible,,"accessibility=Continue"
-57.Click Continue,tap,,"accessibility=Continue"
-58.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-59.Click Finish,tap,,"accessibility=Finish"
-60.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
-61.Profile, tap_coordinate ,978:2224,COORDINATE_MODE
-62.Click Subscription,tap,,"accessibility=Subscription"
-63.Wait Customer Plan,wait_until_visible,,"automator=new UiSelector().descriptionStartsWith("{customerSubscriptionName}")"
-64.Click Customer Plan,tap,,"automator=new UiSelector().descriptionStartsWith("{customerSubscriptionName}")"
-65.wait,3000,,
-66.Load Driver App,switch_to,driver,
-67.wait,2000,,
-68.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
-69.Click Agree,tap,,"accessibility=Agree"
-70.Click Get Started,tap,,"accessibility=Get Started"
-71.Click Next,tap,,"accessibility=Next"
-72.Click Mobile Number,tap,,"accessibility=Mobile Number"
-73.Click Close,tap,,"accessibility=Cancel"
-74.Enter Mobile Number,type,{autoPhone},"automator=new UiSelector().className("android.widget.EditText")"
-75.Wait for Continue,wait_until_visible,,"accessibility=Continue"
-76.Click Continue,tap,,"accessibility=Continue"
-77.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-78.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
-79.wait,3000,,
-80.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
-81.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
-82.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
-83.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
-84.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
-85.Drag Page Layout Upward,swipe,up,
-86.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
-87.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
-88.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
-89.wait,3000,,
-90.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
-91.Wait For OTP,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
-92.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-93.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
-94.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-95.Click Subscription,tap,,"accessibility=Subscription"
-96.Wait Driver Plan,wait_until_visible,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
-97.Click Driver Plan,tap,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
-98.wait,5000,,</t>
+24.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
+25.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
+26.Click Customer subscription plan,click,,"//span[normalize-space()='Customer Subscription Plan']"
+27.Verify Customer Subscription Plan Lists ,verify,,"//div[normalize-space()='Customer Subscription Plans']"
+28.Click  Add New Subscription,click,,"//button[@class='buttonWidget']"
+29.Open Service Category Dropdown,click,,"//span[@aria-label='Select Service Category']"
+30.Select Pest Control,click,,"//li[@aria-label='Pest Control']"
+31.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "//input[@placeholder='Plan Name']"
+32.Enter Driver Plan Name Arabic, type,عضو ذهبي, "//input[@placeholder='Plan Name (in Arabic)']"
+33.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "//input[@placeholder='Plan Name (in Tamil):']"
+34.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "//input[@placeholder='Plan Name (in Hindi):']"
+35.Enter Number Of Days, type,100, "//input[@placeholder='Enter No. of Days ']"
+36.Enter Number Of Free Rides, type,2, "//input[@placeholder='Enter No Of Free Rides']"
+37.Enter Price, type,5000, "//input[@placeholder='Enter Plan Price']"
+38.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "//textarea[@placeholder='Page Description English']"
+39.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "//textarea[@placeholder='Page Description(in Arabic)']"
+40.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "//textarea[@placeholder='Page Description(in Tamil)']"
+41.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "//textarea[@placeholder='Page Description(in Hindi)']"
+42.Open status Dropdown,click,,"//span[@aria-label='select Status']"
+43.Select On,click,,"//li[@aria-label='on']"
+44.Click Submit ,click,,"//button[normalize-space()='Submit']"
+45.Filter Services List,type,{custometSubscriptionName},"//input[@aria-label='Plan Name Filter Input']"
+46.Load User App,switch_to,user,
+47.Wait for Get Started,wait_until_visible,,"accessibility=Get Started"
+48.Click Get Started,tap,,"accessibility=Get Started"
+49.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+50.Click Next,tap,,"accessibility=Next"
+51.Click Mobile Number,tap,,"accessibility=Mobile Number"
+52.Click Close,tap,,"accessibility=Cancel"
+53.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
+54.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+55.Click Continue,tap,,"accessibility=Continue"
+56.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+57.Click Finish,tap,,"accessibility=Finish"
+58.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+59.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
+60.Click Subscription,tap,,"accessibility=Subscription"
+61.Wait Customer Plan,wait_until_visible,,"automator=new UiSelector().descriptionStartsWith("{customerSubscriptionName}")"
+62.Click Customer Plan,tap,,"automator=new UiSelector().descriptionStartsWith("{customerSubscriptionName}")"
+63.Load Driver App,switch_to,driver,
+64.Wait for Popup,wait_until_visible,,"id=com.android.permissioncontroller:id/permission_allow_button"
+65.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+66.Click Agree,tap,,"accessibility=Agree"
+67.Click Get Started,tap,,"accessibility=Get Started"
+68.Click Next,tap,,"accessibility=Next"
+69.Click Mobile Number,tap,,"accessibility=Mobile Number"
+70.Click Close,tap,,"accessibility=Cancel"
+71.Enter Mobile Number,type,{autoPhone},"automator=new UiSelector().className("android.widget.EditText")"
+72.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+73.Click Continue,tap,,"accessibility=Continue"
+74.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+75.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+76.Wait for Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+77.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+78.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+79.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+80.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+81.Drag Page Layout Upward,swipe,up,
+82.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+83.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+84.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+85.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+86.Wait for Agree,wait_until_visible,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+87.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+88.Wait For OTP,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
+89.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+90.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
+91.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+92.Click Subscription,tap,,"accessibility=Subscription"
+93.Wait Driver Plan,wait_until_visible,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
+94.Click Driver Plan,tap,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"</t>
   </si>
   <si>
     <t>1.Load Driver App,switch_to,driver,
@@ -1586,8 +1572,8 @@
 16.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
 17.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
 18.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
-19.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
-20.Drag Page Layout Upward,swipe,up,
+19.Drag Page Layout Upward,swipe,up,
+20.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
 21.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
 22.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
 23.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
@@ -1598,47 +1584,46 @@
 28.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
 29.Click Hamburger,tap_coordinate ,75:209,COORDINATE_MODE
 30.Click Document,tap,,"accessibility=Documents"
-31.Wait For Upload,wait_until_visible,,"accessibility=Upload"
-32.Click Upload,tap,,"accessibility=Upload"
-33.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","accessibility=Upload Documents"
-34.Click Sort,tap_coordinate ,776:313,COORDINATE_MODE
-35.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
-36.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
-37.Click Crop,tap,,"accessibility=Crop"
-38.Click Calender,tap_coordinate ,123:1627,COORDINATE_MODE
-39.Click Month,tap,"accessibility=Next month"
-40.Click Date,tap_coordinate ,922:1381,COORDINATE_MODE
-41.Click Ok,tap,,"accessibility=OK"
-42.Click Upload,tap,,"accessibility=Upload Documents"
-43.Wait For Back,wait_until_visible,,"accessibility=Back"
-44.Click Back,tap,,"accessibility=Back"
-45.Click Back,tap,,"accessibility=Back"
-46.Load Admin App,switch_to,web,
-47.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-49.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-50.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-51.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-52.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-53.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-54.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-55.Click Approve Driver,click,,"//i[@title='Approve']"
-56.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-57.wait,2000,,
-58.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Wait For Document Page,wait_until_visible,,"accessibility=Add Documents"
+32.Wait For Upload,wait_until_visible,,"accessibility=Upload"
+33.Click Upload,tap,,"accessibility=Upload"
+34.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","accessibility=Upload Documents"
+35.Click Sort,tap_coordinate ,776:313,COORDINATE_MODE
+36.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
+37.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
+38.Click Crop,tap,,"accessibility=Crop"
+39.Click Calender,tap_coordinate ,121:1539,COORDINATE_MODE
+41.Click Month,tap,"accessibility=Next month"
+42.Click Date,tap_coordinate ,943:1290,COORDINATE_MODE
+43.Click Ok,tap,,"accessibility=OK"
+44.Click Upload,tap,,"accessibility=Upload Documents"
+45.Wait For Back,wait_until_visible,,"accessibility=Back"
+46.Click Back,tap,,"accessibility=Back"
+47.Click Back,tap,,"accessibility=Back"
+48.Load Admin App,switch_to,web,
+49.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+50.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+51.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+52.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+53.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+54.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+55.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+56.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+57.Click Approve Driver,click,,"//i[@title='Approve']"
+58.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
 59.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-60.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-61.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-62.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-63.Load Driver App,switch_to,driver,
-64.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
-65.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-66.Click Document,tap,,"accessibility=Documents"
-67.Wait For Back,wait_until_visible,,"accessibility=Back"
-68.Click Back,tap,,"accessibility=Back"
+60.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+61.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+62.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+63.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+64.Load Driver App,switch_to,driver,
+65.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
+66.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+67.Click Document,tap,,"accessibility=Documents"
+68.Wait For Back,wait_until_visible,,"accessibility=Back"
 69.Click Back,tap,,"accessibility=Back"
-70.Click Online,tap_coordinate,989:2045,
-71.wait,2000,,
+70.Click Back,tap,,"accessibility=Back"
+71.Click Online,tap_coordinate,989:2045,
 72.Load User App,switch_to,user,
 73.Wait For Get Started,wait_until_visible,,"accessibility=Get Started"
 74.Click Get Started,tap,,"accessibility=Get Started"
@@ -1660,41 +1645,38 @@
 90.Click Confirm,tap,,"accessibility=Confirm"
 91.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
 92.Ride Now,tap,,"accessibility=Ride Now"
-93.wait,2000,,
-94.Load Driver App,switch_to,driver,
-95.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
-96.Accept Ride,tap_coordinate,784:2224,
-97.Wait for Arrived,wait_until_visible,,"accessibility=Arrived"
-98.Ride Arrived,tap,,"accessibility=Arrived"
-99.Wait for Yes,wait_until_visible,,"accessibility=Yes"
-100.Yes Arrived,tap,,"accessibility=Yes"
-101.Wait for Start Ride,wait_until_visible,,"accessibility=Start Ride"
-102.Start Ride,tap,,"accessibility=Start Ride"
-103.Wait for OTP,wait_until_visible,,"automator=new UiSelector().className("android.view.View").instance(6)"
-104.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
-105.Wait for Start Ride,wait_until_visible,,"accessibility=Start"
-106.Start Ride,tap,,"accessibility=Start"
-107.Wait for Complete Ride,wait_until_visible,,"accessibility=Complete Ride"
-108.Complete Ride,tap,,"accessibility=Complete Ride"
-109.Wait for Collect Payment,wait_until_visible,,"accessibility=Collect Payment"
-110.Collect Payment,tap,,"accessibility=Collect Payment"
-111.Wait for Yes,wait_until_visible,,"accessibility=Yes"
-112.Confirm Payment,tap,,"accessibility=Yes"
-113.wait,2000,,
-114.Give Rating,tap_coordinate,444:1642,
-115.Submit Rating,tap,,"accessibility=Submit"
-116.Load User App,switch_to,user,
-117.Wait for Proceed Payment,wait_until_visible,,"accessibility=Proceed To Pay"
-118.Proceed Payment,tap,,"accessibility=Proceed To Pay"
-119.Wait for Proceed Pay,wait_until_visible,,"accessibility=Proceed To Pay"
-120.Pay Cash,tap,,"accessibility=Proceed To Pay"
-121.Wait for Review,wait_until_visible,,"accessibility=Give Review"
-122.Give Review,tap,,"accessibility=Give Review"
-123.wait,2000,,
-124.Give Rating,tap_coordinate,444:1642,
-125.Submit Rating,tap,,"accessibility=Submit"
-126.Wait for Done,wait_until_visible,,"accessibility=Done"
-127.Trip Finished,tap,,"accessibility=Done"</t>
+93.Load Driver App,switch_to,driver,
+94.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
+95.Accept Ride,tap_coordinate,784:2224,
+96.Wait for Arrived,wait_until_visible,,"accessibility=Arrived"
+97.Ride Arrived,tap,,"accessibility=Arrived"
+98.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+99.Yes Arrived,tap,,"accessibility=Yes"
+100.Wait for Start Ride,wait_until_visible,,"accessibility=Start Ride"
+101.Start Ride,tap,,"accessibility=Start Ride"
+102.Wait for OTP,wait_until_visible,,"automator=new UiSelector().className("android.view.View").instance(6)"
+103.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
+104.Wait for Start Ride,wait_until_visible,,"accessibility=Start"
+105.Start Ride,tap,,"accessibility=Start"
+106.Wait for Complete Ride,wait_until_visible,,"accessibility=Complete Ride"
+107.Complete Ride,tap,,"accessibility=Complete Ride"
+108.Wait for Collect Payment,wait_until_visible,,"accessibility=Collect Payment"
+109.Collect Payment,tap,,"accessibility=Collect Payment"
+110.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+111.Confirm Payment,tap,,"accessibility=Yes"
+112.Give Rating,tap_coordinate,444:1642,
+113.Submit Rating,tap,,"accessibility=Submit"
+114.Load User App,switch_to,user,
+115.Wait for Proceed Payment,wait_until_visible,,"accessibility=Proceed To Pay"
+116.Proceed Payment,tap,,"accessibility=Proceed To Pay"
+117.Wait for Proceed Pay,wait_until_visible,,"accessibility=Proceed To Pay"
+118.Pay Cash,tap,,"accessibility=Proceed To Pay"
+119.Wait for Review,wait_until_visible,,"accessibility=Give Review"
+120.Give Review,tap,,"accessibility=Give Review"
+121.Give Rating,tap_coordinate,444:1642,
+122.Submit Rating,tap,,"accessibility=Submit"
+123.Wait for Done,wait_until_visible,,"accessibility=Done"
+124.Trip Finished,tap,,"accessibility=Done"</t>
   </si>
 </sst>
 </file>
@@ -2184,16 +2166,16 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>64</v>
@@ -2261,13 +2243,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>15</v>
@@ -2336,19 +2318,19 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>30</v>
@@ -2418,7 +2400,7 @@
         <v>17</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>12</v>
@@ -2493,7 +2475,7 @@
         <v>19</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
@@ -2565,13 +2547,13 @@
         <v>19</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
@@ -2632,19 +2614,19 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>31</v>
@@ -2714,7 +2696,7 @@
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
@@ -2792,7 +2774,7 @@
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
@@ -2801,7 +2783,7 @@
         <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2864,13 +2846,13 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
52th Commit : Stabilized ABCD HYBRID FRAMEWORK
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{576409A5-8081-4212-AB28-F4178FA7CD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BAF2AD2-2162-4A81-8E83-BE3C08508DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -1404,60 +1404,6 @@
 16.Load  Super Admin,switch_to,web,</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-7.Wait for Auto Ride,wait_until_visible,,"//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-8.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-9. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-10. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-11. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
-12.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-13.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
-14.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-15.Select Source,click,,"//span[@aria-label='Select Source']"
-16.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
-17.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-19.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
-20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-21.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-22.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-23.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-24. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-25. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-26.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-27.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-28. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-29. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-30. Click Submit, click, , "//button[contains(.,'Submit')]"
-31. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-36.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-37.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-38.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-39.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-40.Add Driving License,click,,"//i[@title='Edit']"
-41.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-42.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-43.Click Submit, click, , "//button[normalize-space()='Submit']"
-44.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-45.Click Approve Driver,click,,"//i[@title='Approve']"
-46.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-47.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-49.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-50.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-51.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-</t>
-  </si>
-  <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
 2.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
 3.Click Subscription Plan,click,,"//h2[normalize-space()='Subscription Plan']"
@@ -1593,12 +1539,13 @@
 37.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
 38.Click Crop,tap,,"accessibility=Crop"
 39.Click Calender,tap_coordinate ,121:1539,COORDINATE_MODE
-41.Click Month,tap,"accessibility=Next month"
-42.Click Date,tap_coordinate ,943:1290,COORDINATE_MODE
-43.Click Ok,tap,,"accessibility=OK"
-44.Click Upload,tap,,"accessibility=Upload Documents"
-45.Wait For Back,wait_until_visible,,"accessibility=Back"
-46.Click Back,tap,,"accessibility=Back"
+40.Click Month,tap,"accessibility=Next month"
+41.Click Date,tap_coordinate ,943:1290,COORDINATE_MODE
+42.Click Ok,tap,,"accessibility=OK"
+43.Click Upload,tap,,"accessibility=Upload Documents"
+44.Wait For Back,wait_until_visible,,"accessibility=Back"
+45.Click Back,tap,,"accessibility=Back"
+46.Wait For Back,wait_until_visible,,"accessibility=Back"
 47.Click Back,tap,,"accessibility=Back"
 48.Load Admin App,switch_to,web,
 49.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
@@ -1622,61 +1569,117 @@
 67.Click Document,tap,,"accessibility=Documents"
 68.Wait For Back,wait_until_visible,,"accessibility=Back"
 69.Click Back,tap,,"accessibility=Back"
-70.Click Back,tap,,"accessibility=Back"
-71.Click Online,tap_coordinate,989:2045,
-72.Load User App,switch_to,user,
-73.Wait For Get Started,wait_until_visible,,"accessibility=Get Started"
-74.Click Get Started,tap,,"accessibility=Get Started"
-75.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
-76.Click Next,tap,,"accessibility=Next"
-77.Click Mobile Number,tap,,"accessibility=Mobile Number"
-78.Click Close,tap,,"accessibility=Cancel"
-79.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
-80.Wait for Continue,wait_until_visible,,"accessibility=Continue"
-81.Click Continue,tap,,"accessibility=Continue"
-82.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-83.Click Finish,tap,,"accessibility=Finish"
-84.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
-85.Wait For Auto Ride,wait_until_visible,,"accessibility=Auto Ride"
-86.Click Auto Ride,tap,,"accessibility=Auto Ride"
-87.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
-88.Wait for Location,wait_until_visible,,"accessibility=Set location on the map"
-89.Select Destination,tap_coordinate,545:1299,
-90.Click Confirm,tap,,"accessibility=Confirm"
-91.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
-92.Ride Now,tap,,"accessibility=Ride Now"
-93.Load Driver App,switch_to,driver,
-94.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
-95.Accept Ride,tap_coordinate,784:2224,
-96.Wait for Arrived,wait_until_visible,,"accessibility=Arrived"
-97.Ride Arrived,tap,,"accessibility=Arrived"
-98.Wait for Yes,wait_until_visible,,"accessibility=Yes"
-99.Yes Arrived,tap,,"accessibility=Yes"
-100.Wait for Start Ride,wait_until_visible,,"accessibility=Start Ride"
-101.Start Ride,tap,,"accessibility=Start Ride"
-102.Wait for OTP,wait_until_visible,,"automator=new UiSelector().className("android.view.View").instance(6)"
-103.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
-104.Wait for Start Ride,wait_until_visible,,"accessibility=Start"
-105.Start Ride,tap,,"accessibility=Start"
-106.Wait for Complete Ride,wait_until_visible,,"accessibility=Complete Ride"
-107.Complete Ride,tap,,"accessibility=Complete Ride"
-108.Wait for Collect Payment,wait_until_visible,,"accessibility=Collect Payment"
-109.Collect Payment,tap,,"accessibility=Collect Payment"
-110.Wait for Yes,wait_until_visible,,"accessibility=Yes"
-111.Confirm Payment,tap,,"accessibility=Yes"
-112.Give Rating,tap_coordinate,444:1642,
-113.Submit Rating,tap,,"accessibility=Submit"
-114.Load User App,switch_to,user,
-115.Wait for Proceed Payment,wait_until_visible,,"accessibility=Proceed To Pay"
-116.Proceed Payment,tap,,"accessibility=Proceed To Pay"
-117.Wait for Proceed Pay,wait_until_visible,,"accessibility=Proceed To Pay"
-118.Pay Cash,tap,,"accessibility=Proceed To Pay"
-119.Wait for Review,wait_until_visible,,"accessibility=Give Review"
-120.Give Review,tap,,"accessibility=Give Review"
-121.Give Rating,tap_coordinate,444:1642,
-122.Submit Rating,tap,,"accessibility=Submit"
-123.Wait for Done,wait_until_visible,,"accessibility=Done"
-124.Trip Finished,tap,,"accessibility=Done"</t>
+70.Wait For Back,wait_until_visible,,"accessibility=Back"
+71.Click Back,tap,,"accessibility=Back"
+72.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
+73.Click Online,tap_coordinate,986:1936,
+74.Load User App,switch_to,user,
+75.Wait For Get Started,wait_until_visible,,"accessibility=Get Started"
+76.Click Get Started,tap,,"accessibility=Get Started"
+77.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+78.Click Next,tap,,"accessibility=Next"
+79.Click Mobile Number,tap,,"accessibility=Mobile Number"
+80.Click Close,tap,,"accessibility=Cancel"
+81.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
+82.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+83.Click Continue,tap,,"accessibility=Continue"
+84.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+85.Click Finish,tap,,"accessibility=Finish"
+86.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+87.Wait For Auto Ride,wait_until_visible,,"accessibility=Auto Ride"
+88.Click Auto Ride,tap,,"accessibility=Auto Ride"
+89.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
+90.Wait for Location,wait_until_visible,,"accessibility=Set location on the map"
+91.Select Destination,tap_coordinate,545:1299,
+92.Click Confirm,tap,,"accessibility=Confirm"
+93.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
+94.Ride Now,tap,,"accessibility=Ride Now"
+95.Load Driver App,switch_to,driver,
+96.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
+97.Accept Ride,tap_coordinate,784:2224,
+98.Wait for Arrived,wait_until_visible,,"accessibility=Arrived"
+99.Ride Arrived,tap,,"accessibility=Arrived"
+100.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+101.Yes Arrived,tap,,"accessibility=Yes"
+102.Wait for Start Ride,wait_until_visible,,"accessibility=Start Ride"
+103.Start Ride,tap,,"accessibility=Start Ride"
+104.Wait for OTP,wait_until_visible,,"automator=new UiSelector().className("android.view.View").instance(6)"
+105.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
+106.Wait for Start Ride,wait_until_visible,,"accessibility=Start"
+107.Start Ride,tap,,"accessibility=Start"
+108.Wait for Complete Ride,wait_until_visible,,"accessibility=Complete Ride"
+109.Complete Ride,tap,,"accessibility=Complete Ride"
+110.Wait for Collect Payment,wait_until_visible,,"accessibility=Collect Payment"
+111.Collect Payment,tap,,"accessibility=Collect Payment"
+112.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+113.Confirm Payment,tap,,"accessibility=Yes"
+114.Give Rating,tap_coordinate,444:1642,
+115.Submit Rating,tap,,"accessibility=Submit"
+116.Load User App,switch_to,user,
+117.Wait for Proceed Payment,wait_until_visible,,"accessibility=Proceed To Pay"
+118.Proceed Payment,tap,,"accessibility=Proceed To Pay"
+119.Wait for Proceed Pay,wait_until_visible,,"accessibility=Proceed To Pay"
+120.Pay Cash,tap,,"accessibility=Proceed To Pay"
+121.Wait for Review,wait_until_visible,,"accessibility=Give Review"
+122.Give Review,tap,,"accessibility=Give Review"
+123.Give Rating,tap_coordinate,444:1642,
+124.Submit Rating,tap,,"accessibility=Submit"
+125.Wait for Done,wait_until_visible,,"accessibility=Done"
+126.Trip Finished,tap,,"accessibility=Done"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+7.Wait for Auto Ride,wait_until_visible,,"//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+8.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+9. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+10. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+11. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
+12.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+13.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
+14.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+15.Select Source,click,,"//span[@aria-label='Select Source']"
+16.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
+17.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+19.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
+20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+21.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+22.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+23.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+24. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+25. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+26.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+27.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+28. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+29. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+30. Click Submit, click, , "//button[contains(.,'Submit')]"
+31. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+36.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+37.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+38.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+39.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+40.Add Driving License,click,,"//i[@title='Edit']"
+41.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+42.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+43.Click Submit, click, , "//button[normalize-space()='Submit']"
+44.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+45.Click Approve Driver,click,,"//i[@title='Approve']"
+46.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+47.Click Dashboard,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
+48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+49.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+50.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+51.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+</t>
   </si>
 </sst>
 </file>
@@ -2178,7 +2181,7 @@
         <v>50</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>37</v>
@@ -2553,7 +2556,7 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
@@ -2780,7 +2783,7 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
53th Commit : Test Case Upadated for Autor Ride Test
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BAF2AD2-2162-4A81-8E83-BE3C08508DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12531FF2-7D83-4478-B1FE-316E86BDB948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -1500,134 +1500,6 @@
 94.Click Driver Plan,tap,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"</t>
   </si>
   <si>
-    <t>1.Load Driver App,switch_to,driver,
-2.Wait For Notification,wait_until_visible,,"id=com.android.permissioncontroller:id/permission_allow_button"
-3.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
-4.Click Agree,tap,,"accessibility=Agree"
-5.Click Get Started,tap,,"accessibility=Get Started"
-6.Click Next,tap,,"accessibility=Next"
-7.Click Mobile Number,tap,,"accessibility=Mobile Number"
-8.Click Close,tap,,"accessibility=Cancel"
-9.Enter Mobile Number,type,{autoPhone},"automator=new UiSelector().className("android.widget.EditText")"
-10.Wait for Continue,wait_until_visible,,"accessibility=Continue"
-11.Click Continue,tap,,"accessibility=Continue"
-12.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-13.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
-14.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
-15.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
-16.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
-17.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
-18.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
-19.Drag Page Layout Upward,swipe,up,
-20.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
-21.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
-22.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
-23.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
-24.Wait for Agree,wait_until_visible,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
-25.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
-26.Wait For OTP,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
-27.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-28.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
-29.Click Hamburger,tap_coordinate ,75:209,COORDINATE_MODE
-30.Click Document,tap,,"accessibility=Documents"
-31.Wait For Document Page,wait_until_visible,,"accessibility=Add Documents"
-32.Wait For Upload,wait_until_visible,,"accessibility=Upload"
-33.Click Upload,tap,,"accessibility=Upload"
-34.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","accessibility=Upload Documents"
-35.Click Sort,tap_coordinate ,776:313,COORDINATE_MODE
-36.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
-37.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
-38.Click Crop,tap,,"accessibility=Crop"
-39.Click Calender,tap_coordinate ,121:1539,COORDINATE_MODE
-40.Click Month,tap,"accessibility=Next month"
-41.Click Date,tap_coordinate ,943:1290,COORDINATE_MODE
-42.Click Ok,tap,,"accessibility=OK"
-43.Click Upload,tap,,"accessibility=Upload Documents"
-44.Wait For Back,wait_until_visible,,"accessibility=Back"
-45.Click Back,tap,,"accessibility=Back"
-46.Wait For Back,wait_until_visible,,"accessibility=Back"
-47.Click Back,tap,,"accessibility=Back"
-48.Load Admin App,switch_to,web,
-49.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-50.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-51.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-52.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-53.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-54.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-55.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-56.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-57.Click Approve Driver,click,,"//i[@title='Approve']"
-58.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-59.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-60.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-61.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-62.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-63.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-64.Load Driver App,switch_to,driver,
-65.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
-66.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-67.Click Document,tap,,"accessibility=Documents"
-68.Wait For Back,wait_until_visible,,"accessibility=Back"
-69.Click Back,tap,,"accessibility=Back"
-70.Wait For Back,wait_until_visible,,"accessibility=Back"
-71.Click Back,tap,,"accessibility=Back"
-72.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
-73.Click Online,tap_coordinate,986:1936,
-74.Load User App,switch_to,user,
-75.Wait For Get Started,wait_until_visible,,"accessibility=Get Started"
-76.Click Get Started,tap,,"accessibility=Get Started"
-77.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
-78.Click Next,tap,,"accessibility=Next"
-79.Click Mobile Number,tap,,"accessibility=Mobile Number"
-80.Click Close,tap,,"accessibility=Cancel"
-81.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
-82.Wait for Continue,wait_until_visible,,"accessibility=Continue"
-83.Click Continue,tap,,"accessibility=Continue"
-84.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-85.Click Finish,tap,,"accessibility=Finish"
-86.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
-87.Wait For Auto Ride,wait_until_visible,,"accessibility=Auto Ride"
-88.Click Auto Ride,tap,,"accessibility=Auto Ride"
-89.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
-90.Wait for Location,wait_until_visible,,"accessibility=Set location on the map"
-91.Select Destination,tap_coordinate,545:1299,
-92.Click Confirm,tap,,"accessibility=Confirm"
-93.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
-94.Ride Now,tap,,"accessibility=Ride Now"
-95.Load Driver App,switch_to,driver,
-96.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
-97.Accept Ride,tap_coordinate,784:2224,
-98.Wait for Arrived,wait_until_visible,,"accessibility=Arrived"
-99.Ride Arrived,tap,,"accessibility=Arrived"
-100.Wait for Yes,wait_until_visible,,"accessibility=Yes"
-101.Yes Arrived,tap,,"accessibility=Yes"
-102.Wait for Start Ride,wait_until_visible,,"accessibility=Start Ride"
-103.Start Ride,tap,,"accessibility=Start Ride"
-104.Wait for OTP,wait_until_visible,,"automator=new UiSelector().className("android.view.View").instance(6)"
-105.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
-106.Wait for Start Ride,wait_until_visible,,"accessibility=Start"
-107.Start Ride,tap,,"accessibility=Start"
-108.Wait for Complete Ride,wait_until_visible,,"accessibility=Complete Ride"
-109.Complete Ride,tap,,"accessibility=Complete Ride"
-110.Wait for Collect Payment,wait_until_visible,,"accessibility=Collect Payment"
-111.Collect Payment,tap,,"accessibility=Collect Payment"
-112.Wait for Yes,wait_until_visible,,"accessibility=Yes"
-113.Confirm Payment,tap,,"accessibility=Yes"
-114.Give Rating,tap_coordinate,444:1642,
-115.Submit Rating,tap,,"accessibility=Submit"
-116.Load User App,switch_to,user,
-117.Wait for Proceed Payment,wait_until_visible,,"accessibility=Proceed To Pay"
-118.Proceed Payment,tap,,"accessibility=Proceed To Pay"
-119.Wait for Proceed Pay,wait_until_visible,,"accessibility=Proceed To Pay"
-120.Pay Cash,tap,,"accessibility=Proceed To Pay"
-121.Wait for Review,wait_until_visible,,"accessibility=Give Review"
-122.Give Review,tap,,"accessibility=Give Review"
-123.Give Rating,tap_coordinate,444:1642,
-124.Submit Rating,tap,,"accessibility=Submit"
-125.Wait for Done,wait_until_visible,,"accessibility=Done"
-126.Trip Finished,tap,,"accessibility=Done"</t>
-  </si>
-  <si>
     <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
 2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
 3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
@@ -1680,6 +1552,131 @@
 50.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
 51.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
 </t>
+  </si>
+  <si>
+    <t>1.Load Driver App,switch_to,driver,
+2.Wait For Notification,wait_until_visible,,"id=com.android.permissioncontroller:id/permission_allow_button"
+3.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+4.Click Agree,tap,,"accessibility=Agree"
+5.Click Get Started,tap,,"accessibility=Get Started"
+6.Click Next,tap,,"accessibility=Next"
+7.Click Mobile Number,tap,,"accessibility=Mobile Number"
+8.Click Close,tap,,"accessibility=Cancel"
+9.Enter Mobile Number,type,{autoPhone},"automator=new UiSelector().className("android.widget.EditText")"
+10.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+11.Click Continue,tap,,"accessibility=Continue"
+12.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+13.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+14.Wait For Popup,wait_until_visible,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+15.Click Independent Contractor,tap,,"//android.widget.CheckBox[contains(@content-desc,'Independent Contractor')]"
+16.Click Legal Document,tap,,"//android.widget.CheckBox[contains(@content-desc,'Legal &amp; Document')]"
+17.Click Safety Conduct,tap,,"//android.widget.CheckBox[contains(@content-desc,'Safety &amp; Code')]"
+18.Click Subscription Model,tap,,"//android.widget.CheckBox[contains(@content-desc,'Subscription Model')]"
+19.Drag Page Layout Upward,swipe,up,
+20.Click Liability,tap,,"//android.widget.CheckBox[contains(@content-desc,'Liability &amp; Indemnity')]"
+21.Click Data Protection,tap,,"//android.widget.CheckBox[contains(@content-desc,'Data Protection')]"
+22.Click Fitness Declaration,tap,,"//android.widget.CheckBox[contains(@content-desc,'Fitness Declaration')]"
+23.Click Confirmation,tap,,"//android.widget.CheckBox[contains(@content-desc,'Final Confirmation')]"
+24.Wait for Agree,wait_until_visible,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+25.Click Agree,tap,,"//android.widget.Button[@content-desc="AGREE &amp; CONTINUE"]"
+26.Wait For OTP,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
+27.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+28.Wait For Driver App,wait_until_visible,,"accessibility=Driver App"
+29.Click Hamburger,tap_coordinate ,75:209,COORDINATE_MODE
+30.Click Document,tap,,"accessibility=Documents"
+31.Wait For Document Page,wait_until_visible,,"accessibility=Add Documents"
+32.Wait For Upload,wait_until_visible,,"accessibility=Upload"
+33.Click Upload,tap,,"accessibility=Upload"
+34.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","accessibility=Upload Documents"
+35.Click Sort,tap_coordinate ,776:313,COORDINATE_MODE
+36.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
+37.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
+38.Click Crop,tap,,"accessibility=Crop"
+39.Click Calender,tap_coordinate ,121:1539,COORDINATE_MODE
+40.Click Month,tap,"accessibility=Next month"
+41.Click Date,tap_coordinate ,943:1290,COORDINATE_MODE
+42.Click Ok,tap,,"accessibility=OK"
+43.Click Upload,tap,,"accessibility=Upload Documents"
+44.Wait For Back,wait_until_visible,,"accessibility=Back"
+45.Click Back,tap,,"accessibility=Back"
+46.Load Admin App,switch_to,web,
+47.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+49.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+50.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+51.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+52.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+53.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+54.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+55.Click Approve Driver,click,,"//i[@title='Approve']"
+56.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+57.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+58.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+59.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+60.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+61.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+62.Load Driver App,switch_to,driver,
+63.Wait For Back,wait_until_visible,,"accessibility=Back"
+64.Click Document,tap,,"accessibility=Documents"
+65.Wait For Add Document,wait_until_visible,,"accessibility=Add Documents"
+66.Click Back,tap,,"accessibility=Back"
+67.Wait For Documents,wait_until_visible,,"accessibility=Documents"
+68.Drag Page Layout Upward,swipe,up,
+69.Click Back,tap_coordinate,135:113,
+70.Click Online,tap_coordinate,986:1936,
+71.Load User App,switch_to,user,
+72.Wait For Get Started,wait_until_visible,,"accessibility=Get Started"
+73.Click Get Started,tap,,"accessibility=Get Started"
+74.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+75.Click Next,tap,,"accessibility=Next"
+76.Click Mobile Number,tap,,"accessibility=Mobile Number"
+77.Click Close,tap,,"accessibility=Cancel"
+78.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
+79.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+80.Click Continue,tap,,"accessibility=Continue"
+81.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+82.Click Finish,tap,,"accessibility=Finish"
+83.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+84.Wait For Auto Ride,wait_until_visible,,"accessibility=Auto Ride"
+85.Click Auto Ride,tap,,"accessibility=Auto Ride"
+86.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
+87.Wait for Location,wait_until_visible,,"accessibility=Set location on the map"
+88.Select Destination,tap_coordinate,545:1299,
+89.Click Confirm,tap,,"accessibility=Confirm"
+90.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
+91.Ride Now,tap,,"accessibility=Ride Now"
+92.Load Driver App,switch_to,driver,
+93.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
+94.Accept Ride,tap_coordinate,784:2224,
+95.Wait for Arrived,wait_until_visible,,"accessibility=Arrived"
+96.Ride Arrived,tap,,"accessibility=Arrived"
+97.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+98.Yes Arrived,tap,,"accessibility=Yes"
+99.Wait for Start Ride,wait_until_visible,,"accessibility=Start Ride"
+100.Start Ride,tap,,"accessibility=Start Ride"
+101.Wait for OTP,wait_until_visible,,"automator=new UiSelector().className("android.view.View").instance(6)"
+102.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
+103.Wait for Start Ride,wait_until_visible,,"accessibility=Start"
+104.Start Ride,tap,,"accessibility=Start"
+105.Wait for Complete Ride,wait_until_visible,,"accessibility=Complete Ride"
+106.Complete Ride,tap,,"accessibility=Complete Ride"
+107.Wait for Collect Payment,wait_until_visible,,"accessibility=Collect Payment"
+108.Collect Payment,tap,,"accessibility=Collect Payment"
+109.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+110.Confirm Payment,tap,,"accessibility=Yes"
+111.Give Rating,tap_coordinate,444:1642,
+112.Submit Rating,tap,,"accessibility=Submit"
+113.Load User App,switch_to,user,
+114.Wait for Proceed Payment,wait_until_visible,,"accessibility=Proceed To Pay"
+115.Proceed Payment,tap,,"accessibility=Proceed To Pay"
+116.Wait for Proceed Pay,wait_until_visible,,"accessibility=Proceed To Pay"
+117.Pay Cash,tap,,"accessibility=Proceed To Pay"
+118.Wait for Review,wait_until_visible,,"accessibility=Give Review"
+119.Give Review,tap,,"accessibility=Give Review"
+120.Give Rating,tap_coordinate,444:1642,
+121.Submit Rating,tap,,"accessibility=Submit"
+122.Wait for Done,wait_until_visible,,"accessibility=Done"
+123.Trip Finished,tap,,"accessibility=Done"</t>
   </si>
 </sst>
 </file>
@@ -2556,7 +2553,7 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
@@ -2783,7 +2780,7 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
55th Commit : Mobile And Web Hybrid Framw Work Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12531FF2-7D83-4478-B1FE-316E86BDB948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F47539FC-5333-44AF-92CC-212E49C09453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -1588,95 +1588,115 @@
 32.Wait For Upload,wait_until_visible,,"accessibility=Upload"
 33.Click Upload,tap,,"accessibility=Upload"
 34.Upload License,uploadfile, "src/main/resources/test-data/license.JPG","accessibility=Upload Documents"
-35.Click Sort,tap_coordinate ,776:313,COORDINATE_MODE
-36.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
-37.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
-38.Click Crop,tap,,"accessibility=Crop"
-39.Click Calender,tap_coordinate ,121:1539,COORDINATE_MODE
-40.Click Month,tap,"accessibility=Next month"
-41.Click Date,tap_coordinate ,943:1290,COORDINATE_MODE
-42.Click Ok,tap,,"accessibility=OK"
-43.Click Upload,tap,,"accessibility=Upload Documents"
-44.Wait For Back,wait_until_visible,,"accessibility=Back"
-45.Click Back,tap,,"accessibility=Back"
-46.Load Admin App,switch_to,web,
-47.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-49.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-50.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-51.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-52.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-53.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-54.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-55.Click Approve Driver,click,,"//i[@title='Approve']"
-56.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-57.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-58.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-59.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-60.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-61.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-62.Load Driver App,switch_to,driver,
-63.Wait For Back,wait_until_visible,,"accessibility=Back"
-64.Click Document,tap,,"accessibility=Documents"
-65.Wait For Add Document,wait_until_visible,,"accessibility=Add Documents"
-66.Click Back,tap,,"accessibility=Back"
-67.Wait For Documents,wait_until_visible,,"accessibility=Documents"
-68.Drag Page Layout Upward,swipe,up,
-69.Click Back,tap_coordinate,135:113,
-70.Click Online,tap_coordinate,986:1936,
-71.Load User App,switch_to,user,
-72.Wait For Get Started,wait_until_visible,,"accessibility=Get Started"
-73.Click Get Started,tap,,"accessibility=Get Started"
-74.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
-75.Click Next,tap,,"accessibility=Next"
-76.Click Mobile Number,tap,,"accessibility=Mobile Number"
-77.Click Close,tap,,"accessibility=Cancel"
-78.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
-79.Wait for Continue,wait_until_visible,,"accessibility=Continue"
-80.Click Continue,tap,,"accessibility=Continue"
-81.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
-82.Click Finish,tap,,"accessibility=Finish"
-83.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
-84.Wait For Auto Ride,wait_until_visible,,"accessibility=Auto Ride"
-85.Click Auto Ride,tap,,"accessibility=Auto Ride"
-86.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
-87.Wait for Location,wait_until_visible,,"accessibility=Set location on the map"
-88.Select Destination,tap_coordinate,545:1299,
-89.Click Confirm,tap,,"accessibility=Confirm"
-90.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
-91.Ride Now,tap,,"accessibility=Ride Now"
-92.Load Driver App,switch_to,driver,
-93.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
-94.Accept Ride,tap_coordinate,784:2224,
-95.Wait for Arrived,wait_until_visible,,"accessibility=Arrived"
-96.Ride Arrived,tap,,"accessibility=Arrived"
-97.Wait for Yes,wait_until_visible,,"accessibility=Yes"
-98.Yes Arrived,tap,,"accessibility=Yes"
-99.Wait for Start Ride,wait_until_visible,,"accessibility=Start Ride"
-100.Start Ride,tap,,"accessibility=Start Ride"
-101.Wait for OTP,wait_until_visible,,"automator=new UiSelector().className("android.view.View").instance(6)"
-102.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
-103.Wait for Start Ride,wait_until_visible,,"accessibility=Start"
-104.Start Ride,tap,,"accessibility=Start"
-105.Wait for Complete Ride,wait_until_visible,,"accessibility=Complete Ride"
-106.Complete Ride,tap,,"accessibility=Complete Ride"
-107.Wait for Collect Payment,wait_until_visible,,"accessibility=Collect Payment"
-108.Collect Payment,tap,,"accessibility=Collect Payment"
-109.Wait for Yes,wait_until_visible,,"accessibility=Yes"
-110.Confirm Payment,tap,,"accessibility=Yes"
-111.Give Rating,tap_coordinate,444:1642,
-112.Submit Rating,tap,,"accessibility=Submit"
-113.Load User App,switch_to,user,
-114.Wait for Proceed Payment,wait_until_visible,,"accessibility=Proceed To Pay"
-115.Proceed Payment,tap,,"accessibility=Proceed To Pay"
-116.Wait for Proceed Pay,wait_until_visible,,"accessibility=Proceed To Pay"
-117.Pay Cash,tap,,"accessibility=Proceed To Pay"
-118.Wait for Review,wait_until_visible,,"accessibility=Give Review"
-119.Give Review,tap,,"accessibility=Give Review"
-120.Give Rating,tap_coordinate,444:1642,
-121.Submit Rating,tap,,"accessibility=Submit"
-122.Wait for Done,wait_until_visible,,"accessibility=Done"
-123.Trip Finished,tap,,"accessibility=Done"</t>
+35.Wait For Sort,wait_until_visible,,"automator=new UiSelector().resourceId("com.google.android.documentsui:id/content").instance(0)"
+36.Click Sort,tap,,"automator=new UiSelector().resourceId("com.google.android.documentsui:id/content").instance(0)"
+37.Wait For Modified,wait_until_visible,,"automator=new UiSelector().text("Modified (newest first)")"
+38.Click Modified,tap,,"automator=new UiSelector().text("Modified (newest first)")"
+39.Click License,tap,,"id=com.google.android.documentsui:id/icon_thumb"
+40.Wait For Crop,wait_until_visible,,"accessibility=Crop"
+41.Click Crop,tap,,"accessibility=Crop"
+42.Wait For  Add Document,wait_until_visible,,"accessibility=Add Documents"
+43.Click Calender,tap_coordinate ,121:1539,COORDINATE_MODE
+44.Click Month,tap,"accessibility=Next month"
+45.Click Date,tap_coordinate ,943:1290,COORDINATE_MODE
+46.Click Ok,tap,,"accessibility=OK"
+47.Click Upload,tap,,"accessibility=Upload Documents"
+48.Wait For Back,wait_until_visible,,"accessibility=Back"
+49.Click Back,tap,,"accessibility=Back"
+50.Load Admin App,switch_to,web,
+51.Wait For Driver Menu,wait_until_visible,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+52.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+53.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+54.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+55.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+56.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+57.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+58.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+59.Click Approve Driver,click,,"//i[@title='Approve']"
+60.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+61.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+62.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+63.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+64.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+65.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+66.Load Driver App,switch_to,driver,
+67.Wait For Back,wait_until_visible,,"accessibility=Back"
+68.Click Document,tap,,"accessibility=Documents"
+69.Wait For Add Document,wait_until_visible,,"accessibility=Add Documents"
+70.Click Back,tap,,"accessibility=Back"
+71.Wait For Documents,wait_until_visible,,"accessibility=Documents"
+72.Click Wallet,tap,,"accessibility=Wallet"
+73.Wait For Topup,wait_until_visible,,"accessibility=TopUp"
+74.Click Topup,tap,,"accessibility=TopUp"
+75.Wait For Topup Sum,wait_until_visible,,"accessibility=TopUp"
+76.Click Hundered,tap,,"accessibility=₹ 100.00"
+77.Click Proceed,tap,,"accessibility=Proceed"
+78.Wait For Contact No,wait_until_visible,,"automator=new UiSelector().className("android.widget.EditText")"
+79.Enter Driver Mobile,type,{autoPhone},"automator=new UiSelector().className("android.widget.EditText")"
+80.Wait For Payment Options,wait_until_visible,,"automator=new UiSelector().text("Payment Options")"
+81.Click Net Banking,tap,,"automator=new UiSelector().text("Netbanking")"
+82.Click Bob,tap_coordinate,277:1124,
+83.Wait For Success,wait_until_visible,,"automator=new UiSelector().text("Success")"
+84.Click Success,tap,,"automator=new UiSelector().text("Success")"
+85.Wait For Wallet  Back,wait_until_visible,,"accessibility=Wallet"
+86.Click Back,tap,,"accessibility=Back"
+87.Drag Page Layout Upward,swipe,up,
+88.Click Back,tap,,"accessibility=Back"
+89.Click Online,tap_coordinate,986:1936,
+90.Load User App,switch_to,user,
+91.Wait For Get Started,wait_until_visible,,"accessibility=Get Started"
+92.Click Get Started,tap,,"accessibility=Get Started"
+93.Click Allow Notification,tap,,"id=com.android.permissioncontroller:id/permission_allow_button"
+94.Click Next,tap,,"accessibility=Next"
+95.Click Mobile Number,tap,,"accessibility=Mobile Number"
+96.Click Close,tap,,"accessibility=Cancel"
+97.Enter Mobile Number,type,{userPhone},"automator=new UiSelector().className("android.widget.EditText")"
+98.Wait for Continue,wait_until_visible,,"accessibility=Continue"
+99.Click Continue,tap,,"accessibility=Continue"
+100.Enter OTP,type,123456,"automator=new UiSelector().className("android.widget.EditText")"
+101.Click Finish,tap,,"accessibility=Finish"
+102.Click Allow Location,tap,,"id=com.android.permissioncontroller:id/permission_allow_foreground_only_button"
+103.Wait For Auto Ride,wait_until_visible,,"accessibility=Auto Ride"
+104.Click Auto Ride,tap,,"accessibility=Auto Ride"
+105.Enter Destination, type, Parsn Manare, "automator=new UiSelector().className("android.widget.EditText").instance(1)"
+106.Wait for Location,wait_until_visible,,"accessibility=Set location on the map"
+107.Select Destination,tap_coordinate,545:1299,
+108.Click Confirm,tap,,"accessibility=Confirm"
+109.Wait for Ride,wait_until_visible,,"accessibility=Ride Now"
+110.Ride Now,tap,,"accessibility=Ride Now"
+111.Load Driver App,switch_to,driver,
+112.Wait for Accept,wait_until_visible,,"accessibility=Auto Ride"
+113.Accept Ride,tap_coordinate,801:2113,
+114.Wait for On My Way,wait_until_visible,,"accessibility=On My Way to Pickup"
+115.Wait for Arrived,wait_until_visible,,"accessibility=Arrived"
+116.Ride Arrived,tap,,"accessibility=Arrived"
+117.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+118.Yes Arrived,tap,,"accessibility=Yes"
+119.Wait for Start Ride,wait_until_visible,,"accessibility=Start Ride"
+120.Start Ride,tap,,"accessibility=Start Ride"
+121.Wait for OTP,wait_until_visible,,"automator=new UiSelector().className("android.view.View").instance(6)"
+122.Enter OTP,type,1234,"automator=new UiSelector().className("android.view.View").instance(6)"
+123.Wait for Start Ride,wait_until_visible,,"accessibility=Start"
+124.Start Ride,tap,,"accessibility=Start"
+125.Wait for Complete Ride,wait_until_visible,,"accessibility=Complete Ride"
+126.Complete Ride,tap,,"accessibility=Complete Ride"
+127.Wait for Collect Payment,wait_until_visible,,"accessibility=Collect Payment"
+128.Collect Payment,tap,,"accessibility=Collect Payment"
+129.Wait for Yes,wait_until_visible,,"accessibility=Yes"
+130.Confirm Payment,tap,,"accessibility=Yes"
+131.Give Rating,tap_coordinate,348:1545,
+132.Submit Rating,tap,,"accessibility=Submit"
+133.Load User App,switch_to,user,
+134.Wait for Proceed Payment,wait_until_visible,,"accessibility=Proceed To Pay"
+135.Proceed Payment,tap,,"accessibility=Proceed To Pay"
+136.Wait for Proceed Pay,wait_until_visible,,"accessibility=Proceed To Pay"
+137.Pay Cash,tap,,"accessibility=Proceed To Pay"
+138.Wait for Review,wait_until_visible,,"accessibility=Give Review"
+139.Give Review,tap,,"accessibility=Give Review"
+140.Give Rating,tap_coordinate,348:1619,
+141.Submit Rating,tap,,"accessibility=Submit"
+141.Wait for Done,wait_until_visible,,"accessibility=Done"
+142.Trip Finished,tap,,"accessibility=Done"</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
63th Commit : Global Locator For Web Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4383D7CB-E8BA-4909-A07B-FEDB535F41D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BAD3C24-384F-4833-901F-439CE2D469E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -1956,26 +1956,6 @@
     </r>
   </si>
   <si>
-    <t>1.Click Dashboard  Icon,click,,"admin.menu.dashboard"
-2. Click Customer  Icon,click,,"admin.menu.customer_icon"
-3.Click  Add Customers,click,,"admin.menu.add_customers"
-4. Verify Add Customer Heading,verify,,"admin.customer.add_heading"
-5.Enter Customer Name, type, customer{randomAlpha} &gt;&gt; customerName, "admin.customer.input_name"
-6.Enter Email, type, customer_{timestamp}@gmail.com&gt;&gt;customerEmail, "admin.customer.input_email"
-7.Enter Contact Number, type, {randomPhone}&gt;&gt;userPhone,"admin.customer.input_phone"
-8.Enter Video Call Limit, type, 60, "admin.customer.input_video_limit"
-9.Open Gender,click,,"admin.customer.dropdown_gender"
-10.Select Male,click,,"admin.customer.select_gender_male"
-11.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "admin.customer.upload_profile_img"
-12.Click Submit, click, , "admin.customer.submit_btn"
-13.Verify Added Succesfully, verify, , "admin.customer.toast_info"
-14. Click Customer  Icon,click,,"admin.menu.customer_icon"
-15. Click Customer  Icon,click,,"admin.menu.customer_icon"
-16.Click  Verified Customers,click,,"admin.menu.verified_customers"
-17. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading "
-18.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -2185,45 +2165,6 @@
     </r>
   </si>
   <si>
-    <t>1.Click drivers menu, click, , "admin.drivers.menu.icon"
-2.Click Add Driver menu, click, ,"admin.drivers.add_menu.link"
-3.Verify Add Driver page, verify, , "admin.drivers.add_page.header"
-4.Click Service Category Dropdown, click, , "admin.drivers.service_dropdown.select"
-5.Select Auto Ride Option, click, , "admin.drivers.autoride_option.span"
-6.Select Auto Ride Option, click, ,"admin.drivers.autoride_option.span"
-7.Wait for Auto Ride Checkbox, wait_until_visible, , "admin.drivers.autoride.checkbox"
-8.Click Auto Ride Checkbox, click, , "admin.drivers.autoride.checkbox"
-9.Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "admin.drivers.fullname.input"
-10.Enter Email, type, autodriver_{timestamp}@gmail.com &gt;&gt; autoEmail, "admin.drivers.email.input"
-11.Enter Contact Number, type, {randomPhone} &gt;&gt; autoPhone, "admin.drivers.phone.input"
-12.Click Whatsapp Checkbox, click, , "admin.drivers.whatsapp.checkbox"
-13.Enter Whatsapp Number, type, {autoPhone}, "admin.drivers.whatsapp_phone.input"
-14.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "admin.drivers.profile_image.file"
-15.Click Select Source Dropdown, click, ,"admin.drivers.source_dropdown.select"
-16.Select From Instagram Option, click, , "admin.drivers.instagram_option.span"
-17.Select Male Gender, click, ," admin.drivers.male_gender.div"
-18.Click Vehicle Type Dropdown, click, ,"admin.drivers.vehicle_dropdown.select"
-19.Select Pink Auto Option, click, ," admin.drivers.pink_auto_option.span"
-20.Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
-21.Enter Plate No, type, KL-01-AB-1234,"admin.drivers.plateno.input"
-22.Enter Model Name, type, petrol, "admin.drivers.modelname.input"
-23.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "admin.drivers.vehicle_image.file"
-24.Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
-25.Enter Bank Location, type, Chennai, "admin.drivers.banklocation.input"
-26.Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
-27.Enter Account Holder Name, type, {autoName}, "admin.drivers.accountholder.input"
-28.Enter Payment Email Address, type, {autoEmail}, "admin.drivers.paymentemail.input"
-29.Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
-30.Click Submit Button, click, , "admin.drivers.submit.button"
-31.Verify Driver Added Successfully, verify, , "admin.drivers.success_toast.div"
-32.Wait for Toast to Hide, wait, 1000, 
-33.Click drivers menu to refresh, click, , "admin.drivers.menu.icon"
-34.Click drivers menu to refresh, click, , "admin.drivers.menu.icon"
-35.Click Pending Documents Menu, click, , "admin.drivers.pending_docs.link"
-36.Filter Pending Docs by Name, type, {autoName}, "admin.drivers.name_filter.input"
-37.Click Dashboard Home Icon, click, , "admin.drivers.dashboard.icon"</t>
-  </si>
-  <si>
     <t>SA_TS_15</t>
   </si>
   <si>
@@ -2233,147 +2174,206 @@
     <t>TC_CA_15_Autoride_Locator_Test</t>
   </si>
   <si>
-    <t>1.Load User App, switch_to, user, 
-2.Wait For Get Started, wait_until_visible, ,"mobile.customer.get_started.btn"
-3.Load Driver App, switch_to, driver, 
-4.Wait For Notification, wait_until_visible, , "mobile.driver.permission_allow.btn"
-5.Load  Super Admin,switch_to,web,
-6.Wait For Admin, wait_until_visible, , "admin.login.email"
-7.Enter  Email , type , super_admin@gmail.com, "admin.login.email"
-8.Enter Password,type,R1mep@321, "admin.login.password"
-9.Click Login,click,,"admin.login.submit_btn"
-10.Verify Dashboard,verify,,"admin.dashboard.statistics_header"</t>
-  </si>
-  <si>
-    <t>1. Load Driver App, switch_to, driver, 
-2. Wait For Notification, wait_until_visible, , "mobile.driver.permission_allow.btn"
-3. Click Allow Notification, tap, , "mobile.driver.permission_allow.btn"
-4. Click Agree, tap, , "mobile.driver.agree.btn"
-5. Click Get Started, tap, , "mobile.driver.get_started.btn"
-6. Click Next, tap, ," mobile.driver.next.btn"
-7. Click Mobile Number, tap, , "mobile.driver.mobile_number_field.btn"
-8. Click Close, tap, , "mobile.driver.cancel.btn"
-9. Enter Mobile Number, type, {autoPhone}, "mobile.driver.edit_text.input"
-10. Wait for Continue, wait_until_visible, ,"mobile.driver.continue.btn"
-11. Click Continue, tap, ,"mobile.driver.continue.btn"
-12. Enter OTP, type, 123456, "mobile.driver.edit_text.input"
-13. Click Allow Location, tap, , "mobile.driver.location_allow.btn"
-14. Wait For Popup, wait_until_visible, , "mobile.driver.independent_contractor.checkbox"
-15. Click Independent Contractor, tap, , "mobile.driver.independent_contractor.checkbox"
-16. Click Legal Document, tap, , "mobile.driver.legal_document.checkbox"
-17. Click Safety Conduct, tap, ,"mobile.driver.safety_conduct.checkbox"
-18. Click Subscription Model, tap, , "mobile.driver.subscription_model.checkbox"
-19. Drag Page Layout Upward, swipe, up, 
-20. Click Liability, tap, , "mobile.driver.liability.checkbox"
-21. Click Data Protection, tap, , "mobile.driver.data_protection.checkbox"
-22. Click Fitness Declaration, tap, , "mobile.driver.fitness_declaration.checkbox"
-23. Click Confirmation, tap, , "mobile.driver.confirmation.checkbox"
-24. Wait for Agree, wait_until_visible, ,"mobile.driver.agree_continue.btn"
-25. Click Agree, tap, , "mobile.driver.agree_continue.btn"
-26. Wait For OTP, wait_until_visible, , "mobile.driver.edit_text.input"
-27. Enter OTP, type, 123456,"mobile.driver.edit_text.input"
-28. Wait For Driver App, wait_until_visible, , "mobile.driver.app_header.label"
-29. Click Hamburger, tap_coordinate, 75:209, COORDINATE_MODE
-30. Click Document, tap, , "mobile.driver.documents.menu"
-31. Wait For Document Page, wait_until_visible, , "mobile.driver.add_documents.header"
-32. Wait For Upload, wait_until_visible, ," mobile.driver.upload.btn"
-33. Click Upload, tap, ,"mobile.driver.upload.btn"
-34. Upload License, uploadfile, "src/main/resources/test-data/license.JPG", "mobile.driver.upload_docs.btn"
-35. Wait For Sort, wait_until_visible, ," mobile.driver.android_content.view"
-36. Click Sort, tap, , "mobile.driver.android_content.view"
-37. Wait For Modified, wait_until_visible, , "mobile.driver.sort_modified.btn"
-38. Click Modified, tap, ,"mobile.driver.sort_modified.btn"
-39. Click License, tap, , "mobile.driver.license_thumb.icon"
-40. Wait For Crop, wait_until_visible, ,"mobile.driver.crop.btn"
-41. Click Crop, tap, , "mobile.driver.crop.btn"
-42. Wait For Add Document, wait_until_visible, ,"mobile.driver.add_documents.header"
-43. Click Calendar, tap_coordinate, 121:1539, COORDINATE_MODE
-44. Click Month, tap, ,"mobile.driver.next_month.btn"
-45. Click Date, tap_coordinate, 943:1290, COORDINATE_MODE
-46. Click Ok, tap, , "mobile.driver.ok.btn"
-47. Click Upload Submission, tap, , "mobile.driver.upload_docs.btn"
-48. Wait For Back, wait_until_visible, , "mobile.driver.back.btn"
-49. Click Back, tap, , "mobile.driver.back.btn"
-50.Load Admin App,switch_to,web,
-51.Wait For Driver Menu,wait_until_visible,,"admin.drivers.menu.icon"
-52.Click drivers menu,click,,"admin.drivers.menu.icon"
-53.Click Pending Documents,click,,"admin.drivers.pending_docs.link"
-54.Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
-55.Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
-56.Click Doc Icon,click,,"admin.drivers.docs.icon"
-57.Driver Required Documents,verify,,"admin.drivers.required_docs.header"
-58.FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
-59.Click Approve Driver,click,,"admin.drivers.docs.approval"
-60.Verify Updated Succesfully, verify, , "admin.drivers.updated_toast.div"
-61.Click drivers menu,click,,"admin.drivers.menu.icon"
-62.Click drivers menu,click,,"admin.drivers.menu.icon"
-63.Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
-64.Approved Drivers List,verify,,"admin.drivers.approved_page.header"
-65.Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
-66.Load Driver App,switch_to,driver,
-67.Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
-68.Click Document,tap,,"mobile.driver.documents.menu"
-69.Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
-70.Click Back,tap,,"mobile.driver.back.btn"
-71.Wait For Documents,wait_until_visible,,"mobile.driver.documents.menu"
-72.Click Back,tap,,"mobile.driver.back.btn"
-73.Click Online,tap_coordinate,986:1936,
-74. Load User App, switch_to, user, 
-75. Wait For Get Started, wait_until_visible, ,"mobile.customer.get_started.btn"
-76. Click Get Started, tap, ,"mobile.customer.get_started.btn"
-77. Click Allow Notification, tap, ,"mobile.customer.permission_allow.btn"
-78. Click Next, tap, , "mobile.customer.next.btn"
-79. Click Mobile Number, tap, ,"mobile.customer.mobile_number_field.btn"
-80. Click Close, tap, , "mobile.customer.cancel.btn"
-81. Enter Mobile Number, type, {userPhone}, "mobile.customer.edit_text.input"
-82. Wait for Continue, wait_until_visible, , "mobile.customer.continue.btn"
-83. Click Continue, tap, ,"mobile.customer.continue.btn"
-84. Enter OTP, type, 123456, "mobile.customer.edit_text.input"
-85. Wait for Finish, wait_until_visible, ,"mobile.customer.finish.btn"
-86. Click Finish, tap, ,"mobile.customer.finish.btn"
-87. Click Allow Location, tap, ,"mobile.customer.location_allow.btn"
-88. Wait For Auto Ride, wait_until_visible, ,"mobile.customer.auto_ride.btn"
-89. Click Auto Ride, tap, ,"mobile.customer.auto_ride.btn"
-90. Enter Destination, type, Parsn Manare,"mobile.customer.destination.input"
-91. Wait for Location, wait_until_visible, ,"mobile.customer.set_location_map.btn"
-92. Select Destination, tap_coordinate, 545:1299, 
-93. Click Confirm, tap, ,"mobile.customer.confirm.btn"
-94. Wait for Ride, wait_until_visible, ,"mobile.customer.ride_now.btn"
-95. Ride Now, tap, , "mobile.customer.ride_now.btn"
-96. Load Driver App, switch_to, driver, 
-97. Wait for Accept, wait_until_visible, ,"mobile.driver.auto_ride_notification.label"
-98. Accept Ride, tap_coordinate, 801:2113, 
-99. Wait for On My Way, wait_until_visible, ,"mobile.driver.on_my_way.btn"
-100. Wait for Arrived, wait_until_visible, ,"mobile.driver.arrived.btn"
-101. Wait for Arrived, wait_until_visible, ,"mobile.driver.arrived.btn"
-102. Ride Arrived, tap, ,"mobile.driver.arrived.btn"
-103. Wait for Yes, wait_until_visible, ,"mobile.driver.yes.btn"
-104. Yes Arrived, tap, ,"mobile.driver.yes.btn"
-105. Wait for Start Ride, wait_until_visible, ,"mobile.driver.start_ride.btn"
-106. Start Ride, tap, ,"mobile.driver.start_ride.btn"
-107. Wait for OTP, wait_until_visible, ,"mobile.driver.otp_view.input"
-108. Enter OTP, type, 1234,"mobile.driver.otp_view.input"
-109. Wait for Start Ride Confirm, wait_until_visible, ,"mobile.driver.start.btn"
-110. Start Ride Confirm, tap, ,"mobile.driver.start.btn"
-111. Wait for Complete Ride, wait_until_visible, ,"mobile.driver.complete_ride.btn"
-112. Complete Ride, tap, ,"mobile.driver.complete_ride.btn"
-113. Wait for Collect Payment, wait_until_visible, ,"mobile.driver.collect_payment.btn"
-114. Collect Payment, tap, ,"mobile.driver.collect_payment.btn"
-115. Wait for Yes, wait_until_visible, ,"mobile.driver.yes.btn"
-116. Confirm Payment, tap, ,"mobile.driver.yes.btn"
-117. Give Rating, tap_coordinate, 348:1545, 
-118. Submit Rating, tap, ,"mobile.driver.submit_rating.btn"
-119. Load User App, switch_to, user, 
-120. Wait for Proceed Payment, wait_until_visible, , "mobile.customer.proceed_to_pay.btn"
-121. Proceed Payment, tap, ,"mobile.customer.proceed_to_pay.btn"
-122. Wait for Proceed Pay Confirm, wait_until_visible, , "mobile.customer.proceed_to_pay.btn"
-123. Pay Cash, tap, , "mobile.customer.proceed_to_pay.btn"
-124. Wait for Review, wait_until_visible, ,"mobile.customer.give_review.btn"
-125. Give Review, tap, ,"mobile.customer.give_review.btn"
-126. Give Rating, tap_coordinate, 348:1619, 
-127. Submit Rating, tap, , "mobile.customer.submit_rating.btn"
-128. Wait for Done, wait_until_visible, ,"mobile.customer.done.btn"
-129. Trip Finished, tap, , "mobile.customer.done.btn"</t>
+    <t>1. Load User App,switch_to,user,
+2. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+3. Load Driver App,switch_to,driver,
+4. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+5. Load Super Admin,switch_to,web,
+6. Wait For Admin,wait_until_visible,,"web.global.login.email"
+7. Enter Email,type,super_admin@gmail.com,"web.global.login.email"
+8. Enter Password,type,R1mep@321,"web.global.login.password"
+9. Click Login,click,,"web.global.login.submit_btn"
+10. Verify Dashboard,verify,,"web.global.dashboard.statistics_header"</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click Customer Icon,click,,"admin.menu.customer_icon"
+3. Click Add Customers,click,,"admin.menu.add_customers"
+4. Verify Add Customer Heading,verify,,"admin.customer.add_heading"
+5. Enter Customer Name,type,customer{randomAlpha} &gt;&gt; customerName,"admin.customer.input_name"
+6. Enter Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+7. Enter Contact Number,type,{randomPhone}&gt;&gt;userPhone,"admin.customer.input_phone"
+8. Enter Video Call Limit,type,60,"admin.customer.input_video_limit"
+9. Open Gender,click,,"admin.customer.dropdown_gender"
+10. Select Male,click,,"admin.customer.select_gender_male"
+11. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+12. Click Submit,click,,"web.global.action.submit"
+13. Verify Added Successfully,verify,,"web.global.toast.info"
+14. Click Customer Icon,click,,"admin.menu.customer_icon"
+15. Click Customer Icon,click,,"admin.menu.customer_icon"
+16. Click Verified Customers,click,,"admin.menu.verified_customers"
+17. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
+18. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
+  </si>
+  <si>
+    <t>1. Click drivers menu,click,,"admin.drivers.menu.icon"
+2. Click Add Driver menu,click,,"admin.drivers.add_menu.link"
+3. Verify Add Driver page,verify,,"admin.drivers.add_page.header"
+4. Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
+5. Select Auto Ride Option,click,,"admin.drivers.autoride_option.span"
+6. Select Auto Ride Option,click,,"admin.drivers.autoride_option.span"
+7. Wait for Auto Ride Checkbox,wait_until_visible,,"admin.drivers.autoride.checkbox"
+8. Click Auto Ride Checkbox,click,,"admin.drivers.autoride.checkbox"
+9. Enter Driver Name,type,autodriver{randomAlpha} &gt;&gt; autoName,"admin.drivers.fullname.input"
+10. Enter Email,type,autodriver_{timestamp}@gmail.com &gt;&gt; autoEmail,"admin.drivers.email.input"
+11. Enter Contact Number,type,{randomPhone} &gt;&gt; autoPhone,"admin.drivers.phone.input"
+12. Click Whatsapp Checkbox,click,,"admin.drivers.whatsapp.checkbox"
+13. Enter Whatsapp Number,type,{autoPhone},"admin.drivers.whatsapp_phone.input"
+14. Upload Profile Image,uploadfile,"src/main/resources/test-data/autodriver.jpg","admin.drivers.profile_image.file"
+15. Click Select Source Dropdown,click,,"admin.drivers.source_dropdown.select"
+16. Select From Instagram Option,click,,"admin.drivers.instagram_option.span"
+17. Select Male Gender,click,,"admin.drivers.male_gender.div"
+18. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
+19. Select Pink Auto Option,click,,"admin.drivers.pink_auto_option.span"
+20. Enter Model Year,type,2013,"admin.drivers.modelyear.input"
+21. Enter Plate No,type,KL-01-AB-1234,"admin.drivers.plateno.input"
+22. Enter Model Name,type,petrol,"admin.drivers.modelname.input"
+23. Upload Vehicle Image,uploadfile,"src/main/resources/test-data/vehicle.jpg","admin.drivers.vehicle_image.file"
+24. Enter Bank Name,type,HDFC Bank,"admin.drivers.bankname.input"
+25. Enter Bank Location,type,Chennai,"admin.drivers.banklocation.input"
+26. Enter Account Number,type,50100123456789,"admin.drivers.accountno.input"
+27. Enter Account Holder Name,type,{autoName},"admin.drivers.accountholder.input"
+28. Enter Payment Email Address,type,{autoEmail},"admin.drivers.paymentemail.input"
+29. Enter IFSC Code,type,HDFC0001234,"admin.drivers.ifsc.input"
+30. Click Submit Button,click,,"web.global.action.submit"
+31. Verify Driver Added Successfully,verify,,"web.global.toast.success"
+32. Wait for Toast to Hide,wait,1000,,
+33. Click drivers menu to refresh,click,,"admin.drivers.menu.icon"
+34. Click drivers menu to refresh,click,,"admin.drivers.menu.icon"
+35. Click Pending Documents Menu,click,,"admin.drivers.pending_docs.link"
+36. Filter Pending Docs by Name,type,{autoName},"admin.drivers.name_filter.input"
+37. Click Dashboard Home Icon,click,,"web.global.menu.dashboard"</t>
+  </si>
+  <si>
+    <t>1. Load Driver App,switch_to,driver,
+2. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+3. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+4. Click Agree,tap,,"mobile.driver.agree.btn"
+5. Click Get Started,tap,,"mobile.driver.get_started.btn"
+6. Click Next,tap,,"mobile.driver.next.btn"
+7. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+8. Click Close,tap,,"mobile.driver.cancel.btn"
+9. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+10. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+11. Click Continue,tap,,"mobile.driver.continue.btn"
+12. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+13. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+14. Wait For Popup,wait_until_visible,,"mobile.driver.independent_contractor.checkbox"
+15. Click Independent Contractor,tap,,"mobile.driver.independent_contractor.checkbox"
+16. Click Legal Document,tap,,"mobile.driver.legal_document.checkbox"
+17. Click Safety Conduct,tap,,"mobile.driver.safety_conduct.checkbox"
+18. Click Subscription Model,tap,,"mobile.driver.subscription_model.checkbox"
+19. Drag Page Layout Upward,swipe,up,
+20. Click Liability,tap,,"mobile.driver.liability.checkbox"
+21. Click Data Protection,tap,,"mobile.driver.data_protection.checkbox"
+22. Click Fitness Declaration,tap,,"mobile.driver.fitness_declaration.checkbox"
+23. Click Confirmation,tap,,"mobile.driver.confirmation.checkbox"
+24. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+25. Click Agree,tap,,"mobile.driver.agree_continue.btn"
+26. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+27. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+28. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+29. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+30. Click Document,tap,,"mobile.driver.documents.menu"
+31. Wait For Document Page,wait_until_visible,,"mobile.driver.add_documents.header"
+32. Wait For Upload,wait_until_visible,,"mobile.driver.upload.btn"
+33. Click Upload,tap,,"mobile.driver.upload.btn"
+34. Upload License,uploadfile,"src/main/resources/test-data/license.JPG","mobile.driver.upload_docs.btn"
+35. Wait For Sort,wait_until_visible,,"mobile.driver.android_content.view"
+36. Click Sort,tap,,"mobile.driver.android_content.view"
+37. Wait For Modified,wait_until_visible,,"mobile.driver.sort_modified.btn"
+38. Click Modified,tap,,"mobile.driver.sort_modified.btn"
+39. Click License,tap,,"mobile.driver.license_thumb.icon"
+40. Wait For Crop,wait_until_visible,,"mobile.driver.crop.btn"
+41. Click Crop,tap,,"mobile.driver.crop.btn"
+42. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+43. Click Calendar,tap_coordinate,121:1539,COORDINATE_MODE
+44. Click Month,tap,,"mobile.driver.next_month.btn"
+45. Click Date,tap_coordinate,943:1290,COORDINATE_MODE
+46. Click Ok,tap,,"mobile.driver.ok.btn"
+47. Click Upload Submission,tap,,"mobile.driver.upload_docs.btn"
+48. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+49. Click Back,tap,,"mobile.driver.back.btn"
+50. Load Admin App,switch_to,web,
+51. Wait For Driver Menu,wait_until_visible,,"admin.drivers.menu.icon"
+52. Click drivers menu,click,,"admin.drivers.menu.icon"
+53. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+54. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+55. Scroll Grid,tab,7,"admin.drivers.name_filter.input"
+56. Click Doc Icon,click,,"admin.drivers.docs.icon"
+57. Driver Required Documents,verify,,"admin.drivers.required_docs.header"
+58. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+59. Click Approve Driver,click,,"admin.drivers.docs.approval"
+60. Verify Updated Successfully,verify,,"web.global.toast.updated"
+61. Click drivers menu,click,,"admin.drivers.menu.icon"
+62. Click drivers menu,click,,"admin.drivers.menu.icon"
+63. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+64. Approved Drivers List,verify,,"admin.drivers.approved_page.header"
+65. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+66. Load Driver App,switch_to,driver,
+67. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+68. Click Document,tap,,"mobile.driver.documents.menu"
+69. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+70. Click Back,tap,,"mobile.driver.back.btn"
+71. Wait For Documents,wait_until_visible,,"mobile.driver.documents.menu"
+72. Click Back,tap,,"mobile.driver.back.btn"
+73. Click Online,tap_coordinate,986:1936,
+74. Load User App,switch_to,user,
+75. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+76. Click Get Started,tap,,"mobile.customer.get_started.btn"
+77. Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+78. Click Next,tap,,"mobile.customer.next.btn"
+79. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+80. Click Close,tap,,"mobile.customer.cancel.btn"
+81. Enter Mobile Number,type,{userPhone},"mobile.customer.edit_text.input"
+82. Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+83. Click Continue,tap,,"mobile.customer.continue.btn"
+84. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+85. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+86. Click Finish,tap,,"mobile.customer.finish.btn"
+87. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+88. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+89. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+90. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+91. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+92. Select Destination,tap_coordinate,545:1299,
+93. Click Confirm,tap,,"mobile.customer.confirm.btn"
+94. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+95. Ride Now,tap,,"mobile.customer.ride_now.btn"
+96. Load Driver App,switch_to,driver,
+97. Wait for Accept,wait_until_visible,,"mobile.driver.auto_ride_notification.label"
+98. Accept Ride,tap_coordinate,801:2113,
+99. Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
+100. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+101. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+102. Ride Arrived,tap,,"mobile.driver.arrived.btn"
+103. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+104. Yes Arrived,tap,,"mobile.driver.yes.btn"
+105. Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
+106. Start Ride,tap,,"mobile.driver.start_ride.btn"
+107. Wait for OTP,wait_until_visible,,"mobile.driver.otp_view.input"
+108. Enter OTP,type,1234,"mobile.driver.otp_view.input"
+109. Wait for Start Ride Confirm,wait_until_visible,,"mobile.driver.start.btn"
+110. Start Ride Confirm,tap,,"mobile.driver.start.btn"
+111. Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
+112. Complete Ride,tap,,"mobile.driver.complete_ride.btn"
+113. Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
+114. Collect Payment,tap,,"mobile.driver.collect_payment.btn"
+115. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+116. Confirm Payment,tap,,"mobile.driver.yes.btn"
+117. Give Rating,tap_coordinate,348:1545,
+118. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
+119. Load User App,switch_to,user,
+120. Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+121. Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
+122. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+123. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
+124. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
+125. Give Review,tap,,"mobile.customer.give_review.btn"
+126. Give Rating,tap_coordinate,348:1619,
+127. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
+128. Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
+129. Trip Finished,tap,,"mobile.customer.done.btn"</t>
   </si>
 </sst>
 </file>
@@ -3091,7 +3091,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>72</v>
       </c>
@@ -3105,7 +3105,7 @@
         <v>71</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>13</v>
@@ -3181,7 +3181,7 @@
         <v>77</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>78</v>
@@ -3244,22 +3244,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3317,13 +3317,13 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
@@ -3332,7 +3332,7 @@
         <v>89</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
67th Commit :Super Admin Driver  Locator Updated
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0DCBE08-EEA3-4235-8BB0-0C06C0716442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A45A3B-4D3E-411B-B8CB-5883BCC3FDCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rebooter" sheetId="34" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="92">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -1330,46 +1330,6 @@
 18.Filter Customer Name List,type,{customerName},"//input[@aria-label='Customer Name Filter Input']"</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-7.Wait for Auto Ride,wait_until_visible,,"//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-8.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-9. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-10. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-11. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
-12.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-13.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
-14.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-15.Select Source,click,,"//span[@aria-label='Select Source']"
-16.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
-17.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-19.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
-20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-21.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-22.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-23.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-24. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-25. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-26.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-27.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-28. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-29. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-30. Click Submit, click, , "//button[contains(.,'Submit')]"
-31. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-32. Wait for Toast to hide, wait, 1000,
-33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-34.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-35.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-36.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-37.Click  Dashboard Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
-</t>
-  </si>
-  <si>
     <t>1.Load User App,switch_to,user,
 2.Wait For Get Started,wait_until_visible,,"accessibility=Get Started"
 3.Click Get Started,tap,,"accessibility=Get Started"
@@ -1482,60 +1442,6 @@
 92.Click Subscription,tap,,"accessibility=Subscription"
 93.Wait Driver Plan,wait_until_visible,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"
 94.Click Driver Plan,tap,,"automator=new UiSelector().descriptionStartsWith("{driverSubscriptionName}")"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
-3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
-4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
-5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-6.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
-7.Wait for Auto Ride,wait_until_visible,,"//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-8.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
-9. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
-10. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
-11. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
-12.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
-13.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
-14.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
-15.Select Source,click,,"//span[@aria-label='Select Source']"
-16.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
-17.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
-18.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
-19.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
-20. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
-21.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
-22.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
-23.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
-24. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
-25. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
-26.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
-27.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
-28. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
-29. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
-30. Click Submit, click, , "//button[contains(.,'Submit')]"
-31. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-32.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-33.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-34.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
-35.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-36.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
-37.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
-38.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
-39.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
-40.Add Driving License,click,,"//i[@title='Edit']"
-41.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
-42.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
-43.Click Submit, click, , "//button[normalize-space()='Submit']"
-44.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-45.Click Approve Driver,click,,"//i[@title='Approve']"
-46.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-47.Click Dashboard,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
-48.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
-49.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
-50.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
-51.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
-</t>
   </si>
   <si>
     <t>1.Load Driver App,switch_to,driver,
@@ -2186,6 +2092,94 @@
 10. Verify Dashboard,verify,,"web.global.dashboard.statistics_header"</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+7. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+8. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
+9.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+10.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
+11.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+12.Select Source,click,,"//span[@aria-label='Select Source']"
+13.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
+14.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+15.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+16.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
+17. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+18.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+19.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+20.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+23.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+24.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+25. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+27. Click Submit, click, , "//button[contains(.,'Submit')]"
+28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+29. Wait for Toast to hide, wait, 1000,
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+32.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+33.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+34.Click  Dashboard Icon,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+2. Click Add Driver menu,click,,"//span[normalize-space()='Add Driver']"
+3. Verify Add Driver,verify,,"//div[contains(text(),'Add Driver')]"
+4.Click Service Category Dropdown,click,,"//span[@aria-label='Select Service category']"
+5.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+6. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "//label[contains(.,'Full Name')]/following::input[1]"
+7. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "//label[contains(.,'Email')]/following::input[1]"
+8. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "//input[@type='tel']"
+9.Click Whatspp, click, , "//div[contains(@class, 'mdc-checkbox')][1]"
+10.Enter Whatspp Number, type, {autoPhone}, "//span[normalize-space()='WhatsApp Number']/ancestor::div[contains(@class,'flex-col')]//input[@type='tel']"
+11.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "//input[@type='file']"
+12.Select Source,click,,"//span[@aria-label='Select Source']"
+13.Select Instagram,click,,"//span[normalize-space()='From Instagram']"
+14.Select Male Gender, click, , "//div[contains(@class, 'genlabel') and text()='Male']"
+15.Click Vehicle Type Dropdown,click,,"//span[contains(@aria-label,'vehicle type')]"
+16.Select  Auto Option,click,,"//span[normalize-space()='Pink Auto']"
+17. Enter Model Year, type, 2013, "//label[contains(.,'Model Year')]/following::input[1]"
+18.Enter Plate No, type, KL-01-AB-1234, "//label[contains(.,'Plate No')]/following::input[1]"
+19.Enter Model Name, type, petrol, "//label[contains(.,'Model Name')]/following::input[1]"
+20.Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "(//input[@type='file'])[2]"
+21. Enter Bank Name, type, HDFC Bank, "//label[contains(.,'Bank Name')]/following::input[1]"
+22. Enter Bank Location, type, Chennai, "//label[contains(.,'Bank Location')]/following::input[1]"
+23.Enter Account Number, type, 50100123456789, "//label[contains(.,'Account Number')]/following::input[1]"
+24.Enter Account Holder Name, type,{autoName}, "//label[contains(.,'Account Holder Name')]/following::input[1]"
+25. Enter Payment Email Address, type, {autoEmail}, "//label[contains(.,'Payment Email Address')]/following::input[1]"
+26. Enter IFSC Code, type, HDFC0001234, "//label[contains(.,'IFSC Code')]/following::input[1]"
+27. Click Submit, click, , "//button[contains(.,'Submit')]"
+28. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
+29.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+30.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+31.Click Pending Documents,click,,"//span[normalize-space()='Pending Documents']"
+32.Filter by Name,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+33.Scroll Grid, tab, 7, "//input[@aria-label='Driver Name Filter Input']"
+34.Click Doc Icon,click,,"//i[@class='bi bi-file-earmark-text cursor-pointer gridIcon Navigate']"
+35.Driver Required Documents,verify,,"//div[contains(text(),'Driver Required Documents')]"
+36.FilterDocumet List,type,Driving Licence,"//input[@aria-label='Document Name Filter Input']"
+37.Add Driving License,click,,"//i[@title='Edit']"
+38.Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "//input[@type='file']"
+39.Enter Expiry Date,type,12-12-2026,"//input[@placeholder='DD/MM/YYYY']"
+40.Click Submit, click, , "//button[normalize-space()='Submit']"
+41.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+42.Click Approve Driver,click,,"//i[@title='Approve']"
+43.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
+44.Click Dashboard,click,,"//i[@class='fa-house-chimney fa-solid iconstyle']"
+45.Click drivers menu,click,,"//i[contains(@class,'fa-motorcycle fa-solid iconstyle')]"
+46.Click Approved Drivers,click,,"//span[normalize-space()='Approved Drivers']"
+47.Approved Drivers List,verify,,"//div[contains(text(),'Approved Drivers List')]"
+48.Filter Approved Driver,type,{autoName},"//input[@aria-label='Driver Name Filter Input']"
+</t>
+  </si>
+  <si>
     <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
 2. Click Customer Icon,click,,"admin.menu.customer_icon"
 3. Click Add Customers,click,,"admin.menu.add_customers"
@@ -2193,56 +2187,54 @@
 5. Enter Customer Name,type,customer{randomAlpha} &gt;&gt; customerName,"admin.customer.input_name"
 6. Enter Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
 7. Enter Contact Number,type,{randomPhone}&gt;&gt;userPhone,"admin.customer.input_phone"
-8. Enter Video Call Limit,type,60,"admin.customer.input_video_limit"
+8.Enter Video Call Limit,type,50,"admin.customer.input_video_limit"
 9. Open Gender,click,,"admin.customer.dropdown_gender"
 10. Select Male,click,,"admin.customer.select_gender_male"
-11. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
-12. Click Submit,click,,"web.global.action.submit"
+11.Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+12.Click Submit,click,,"web.global.action.submit"
 13. Verify Added Successfully,verify,,"web.global.toast.info"
-14. Click Customer Icon,click,,"admin.menu.customer_icon"
-15. Click Customer Icon,click,,"admin.menu.customer_icon"
-16. Click Verified Customers,click,,"admin.menu.verified_customers"
+14.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+15.Click Customer Icon,click,,"admin.menu.customer_icon"
+16.Click Verified Customers,click,,"admin.menu.verified_customers"
 17. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
-18. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
-  </si>
-  <si>
-    <t>1. Click drivers menu,click,,"admin.drivers.menu.icon"
-2. Click Add Driver menu,click,,"admin.drivers.add_menu.link"
-3. Verify Add Driver page,verify,,"admin.drivers.add_page.header"
-4. Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
-5. Select Auto Ride Option,click,,"admin.drivers.autoride_option.span"
-6. Select Auto Ride Option,click,,"admin.drivers.autoride_option.span"
-7. Wait for Auto Ride Checkbox,wait_until_visible,,"admin.drivers.autoride.checkbox"
-8. Click Auto Ride Checkbox,click,,"admin.drivers.autoride.checkbox"
-9. Enter Driver Name,type,autodriver{randomAlpha} &gt;&gt; autoName,"admin.drivers.fullname.input"
-10. Enter Email,type,autodriver_{timestamp}@gmail.com &gt;&gt; autoEmail,"admin.drivers.email.input"
-11. Enter Contact Number,type,{randomPhone} &gt;&gt; autoPhone,"admin.drivers.phone.input"
-12. Click Whatsapp Checkbox,click,,"admin.drivers.whatsapp.checkbox"
-13. Enter Whatsapp Number,type,{autoPhone},"admin.drivers.whatsapp_phone.input"
-14. Upload Profile Image,uploadfile,"src/main/resources/test-data/autodriver.jpg","admin.drivers.profile_image.file"
-15. Click Select Source Dropdown,click,,"admin.drivers.source_dropdown.select"
-16. Select From Instagram Option,click,,"admin.drivers.instagram_option.span"
-17. Select Male Gender,click,,"admin.drivers.male_gender.div"
-18. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
-19. Select Pink Auto Option,click,,"admin.drivers.pink_auto_option.span"
-20. Enter Model Year,type,2013,"admin.drivers.modelyear.input"
-21. Enter Plate No,type,KL-01-AB-1234,"admin.drivers.plateno.input"
-22. Enter Model Name,type,petrol,"admin.drivers.modelname.input"
-23. Upload Vehicle Image,uploadfile,"src/main/resources/test-data/vehicle.jpg","admin.drivers.vehicle_image.file"
-24. Enter Bank Name,type,HDFC Bank,"admin.drivers.bankname.input"
-25. Enter Bank Location,type,Chennai,"admin.drivers.banklocation.input"
-26. Enter Account Number,type,50100123456789,"admin.drivers.accountno.input"
-27. Enter Account Holder Name,type,{autoName},"admin.drivers.accountholder.input"
-28. Enter Payment Email Address,type,{autoEmail},"admin.drivers.paymentemail.input"
-29. Enter IFSC Code,type,HDFC0001234,"admin.drivers.ifsc.input"
-30. Click Submit Button,click,,"web.global.action.submit"
-31. Verify Driver Added Successfully,verify,,"web.global.toast.success"
-32. Wait for Toast to Hide,wait,1000,,
-33. Click drivers menu to refresh,click,,"admin.drivers.menu.icon"
-34. Click drivers menu to refresh,click,,"admin.drivers.menu.icon"
-35. Click Pending Documents Menu,click,,"admin.drivers.pending_docs.link"
-36. Filter Pending Docs by Name,type,{autoName},"admin.drivers.name_filter.input"
-37. Click Dashboard Home Icon,click,,"web.global.menu.dashboard"</t>
+18.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click drivers menu,click,,"admin.drivers.menu.icon"
+3. Click Add Driver menu,click,,"admin.drivers.add_menu.link"
+4. Verify Add Driver page,verify,,"admin.drivers.add_page.header"
+5. Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
+6. Select Auto Ride Option,click,,"admin.drivers.service_option.autoride"
+7. Enter Driver Name,type,autodriver{randomAlpha} &gt;&gt; autoName,"admin.drivers.fullname.input"
+8. Enter Email,type,autodriver_{timestamp}@gmail.com &gt;&gt; autoEmail,"admin.drivers.email.input"
+9. Enter Contact Number,type,{randomPhone} &gt;&gt; autoPhone,"admin.drivers.phone.input"
+10. Click Whatsapp Checkbox,click,,"admin.drivers.whatsapp.checkbox"
+11. Enter Whatsapp Number,type,{autoPhone},"admin.drivers.whatsapp_phone.input"
+12. Upload Profile Image,uploadfile,"src/main/resources/test-data/autodriver.jpg","admin.drivers.profile_image.file"
+13. Click Select Source Dropdown,click,,"admin.drivers.source_dropdown.select"
+14. Select From Instagram Option,click,,"admin.drivers.instagram_option.span"
+15. Select Male Gender,click,,"admin.drivers.male_gender.div"
+16. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
+17. Select Pink Auto Option,click,,"admin.drivers.vehicle_option.pinkauto"
+18. Enter Model Year,type,2013,"admin.drivers.modelyear.input"
+19. Enter Plate No,type,KL-01-AB-1234,"admin.drivers.plateno.input"
+20. Enter Model Name,type,petrol,"admin.drivers.modelname.input"
+21. Upload Vehicle Image,uploadfile,"src/main/resources/test-data/vehicle.jpg","admin.drivers.vehicle_image.file"
+22. Enter Bank Name,type,HDFC Bank,"admin.drivers.bankname.input"
+23. Enter Bank Location,type,Chennai,"admin.drivers.banklocation.input"
+24. Enter Account Number,type,50100123456789,"admin.drivers.accountno.input"
+25. Enter Account Holder Name,type,{autoName},"admin.drivers.accountholder.input"
+26. Enter Payment Email Address,type,{autoEmail},"admin.drivers.paymentemail.input"
+27. Enter IFSC Code,type,HDFC0001234,"admin.drivers.ifsc.input"
+28. Click Submit Button,click,,"web.global.action.submit"
+29. Verify Driver Added Successfully,verify,,"web.global.toast.success"
+30. Wait for Toast to Hide,wait,1000,,
+31.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+32. Click drivers menu to refresh,click,,"admin.drivers.menu.icon"
+33. Click Pending Documents Menu,click,,"admin.drivers.pending_docs.link"
+34. Filter Pending Docs by Name,type,{autoName},"admin.drivers.name_filter.input"
+35. Click Dashboard Home Icon,click,,"web.global.menu.dashboard"</t>
   </si>
   <si>
     <t>1. Load Driver App,switch_to,driver,
@@ -2293,87 +2285,97 @@
 46. Click Ok,tap,,"mobile.driver.ok.btn"
 47. Click Upload Submission,tap,,"mobile.driver.upload_docs.btn"
 48. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
-49. Click Back,tap,,"mobile.driver.back.btn"
-50. Load Admin App,switch_to,web,
-51. Wait For Driver Menu,wait_until_visible,,"admin.drivers.menu.icon"
-52. Click drivers menu,click,,"admin.drivers.menu.icon"
-53. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
-54. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
-55. Scroll Grid,tab,7,"admin.drivers.name_filter.input"
-56. Click Doc Icon,click,,"admin.drivers.docs.icon"
-57. Driver Required Documents,verify,,"admin.drivers.required_docs.header"
-58. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
-59. Click Approve Driver,click,,"admin.drivers.docs.approval"
-60. Verify Updated Successfully,verify,,"web.global.toast.updated"
-61. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-62. Click drivers menu,click,,"admin.drivers.menu.icon"
-63. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
-64. Approved Drivers List,verify,,"admin.drivers.approved_page.header"
-65. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
-66. Load Driver App,switch_to,driver,
-67. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
-68. Click Document,tap,,"mobile.driver.documents.menu"
-69. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
-70. Click Back,tap,,"mobile.driver.back.btn"
-71. Wait For Documents,wait_until_visible,,"mobile.driver.documents.menu"
+49. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+50. Click Back,tap,,"mobile.driver.back.btn"
+51. Load Admin App,switch_to,web,
+52. Wait For Dashboard,wait_until_visible,,"web.global.menu.dashboard"
+53. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+54. Click drivers menu,click,,"admin.drivers.menu.icon"
+55. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+56. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+57. Scroll Grid,tab,7,"admin.drivers.name_filter.input"
+58. Click Doc Icon,click,,"admin.drivers.docs.icon"
+59. Driver Required Documents,verify,,"admin.drivers.required_docs.header"
+60. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+61. Click Approve Driver,click,,"admin.drivers.docs.approval"
+62. Verify Updated Successfully,verify,,"web.global.toast.updated"
+63. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+64. Click drivers menu,click,,"admin.drivers.menu.icon"
+65. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+66. Approved Drivers List,verify,,"admin.drivers.approved_page.header"
+67. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+68. Load Driver App,switch_to,driver,
+69. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+70. Click Document,tap,,"mobile.driver.documents.menu"
+71. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
 72. Click Back,tap,,"mobile.driver.back.btn"
-73. Click Online,tap_coordinate,986:1936,
-74. Load User App,switch_to,user,
-75. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-76. Click Get Started,tap,,"mobile.customer.get_started.btn"
-77. Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-78. Click Next,tap,,"mobile.customer.next.btn"
-79. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-80. Click Close,tap,,"mobile.customer.cancel.btn"
-81. Enter Mobile Number,type,{userPhone},"mobile.customer.edit_text.input"
-82. Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-83. Click Continue,tap,,"mobile.customer.continue.btn"
-84. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-85. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
-86. Click Finish,tap,,"mobile.customer.finish.btn"
-87. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-88. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
-89. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
-90. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
-91. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
-92. Select Destination,tap_coordinate,545:1299,
-93. Click Confirm,tap,,"mobile.customer.confirm.btn"
-94. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
-95. Ride Now,tap,,"mobile.customer.ride_now.btn"
-96. Load Driver App,switch_to,driver,
-97. Wait for Accept,wait_until_visible,,"mobile.driver.auto_ride_notification.label"
-98. Accept Ride,tap_coordinate,801:2113,
-99. Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
-100. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
-101. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
-102. Ride Arrived,tap,,"mobile.driver.arrived.btn"
-103. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
-104. Yes Arrived,tap,,"mobile.driver.yes.btn"
-105. Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
-106. Start Ride,tap,,"mobile.driver.start_ride.btn"
-107. Wait for OTP,wait_until_visible,,"mobile.driver.otp_view.input"
-108. Enter OTP,type,1234,"mobile.driver.otp_view.input"
-109. Wait for Start Ride Confirm,wait_until_visible,,"mobile.driver.start.btn"
-110. Start Ride Confirm,tap,,"mobile.driver.start.btn"
-111. Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
-112. Complete Ride,tap,,"mobile.driver.complete_ride.btn"
-113. Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
-114. Collect Payment,tap,,"mobile.driver.collect_payment.btn"
-115. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
-116. Confirm Payment,tap,,"mobile.driver.yes.btn"
-117. Give Rating,tap_coordinate,348:1545,
-118. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
-119. Load User App,switch_to,user,
-120. Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
-121. Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
-122. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
-123. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
-124. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
-125. Give Review,tap,,"mobile.customer.give_review.btn"
-126. Give Rating,tap_coordinate,348:1619,
-127. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
-128. Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
-129. Trip Finished,tap,,"mobile.customer.done.btn"</t>
+73. Wait For Documents,wait_until_visible,,"mobile.driver.documents.menu"
+74. Click Back,tap,,"mobile.driver.back.btn"
+75. Click Online,tap_coordinate,986:1936,
+76. Load User App,switch_to,user,
+77. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+78. Click Get Started,tap,,"mobile.customer.get_started.btn"
+79. Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+80. Click Next,tap,,"mobile.customer.next.btn"
+81. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+82. Click Close,tap,,"mobile.customer.cancel.btn"
+83. Enter Mobile Number,type,{userPhone},"mobile.customer.edit_text.input"
+84. Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+85. Click Continue,tap,,"mobile.customer.continue.btn"
+86. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+87. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+88. Click Finish,tap,,"mobile.customer.finish.btn"
+89. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+90. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+91. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+92. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+93. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+94. Select Destination,tap_coordinate,545:1299,
+95. Click Confirm,tap,,"mobile.customer.confirm.btn"
+96. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+97. Ride Now,tap,,"mobile.customer.ride_now.btn"
+98. Load Driver App,switch_to,driver,
+99. Wait for Accept,wait_until_visible,,"mobile.driver.auto_ride_notification.label"
+100. Accept Ride,tap_coordinate,801:2113,
+101. Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
+102. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+103. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+104. Ride Arrived,tap,,"mobile.driver.arrived.btn"
+105. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+106. Yes Arrived,tap,,"mobile.driver.yes.btn"
+107. Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
+108. Start Ride,tap,,"mobile.driver.start_ride.btn"
+109. Wait for OTP,wait_until_visible,,"mobile.driver.otp_view.input"
+110. Enter OTP,type,1234,"mobile.driver.otp_view.input"
+111. Wait for Start Ride Confirm,wait_until_visible,,"mobile.driver.start.btn"
+112. Start Ride Confirm,tap,,"mobile.driver.start.btn"
+113. Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
+114. Complete Ride,tap,,"mobile.driver.complete_ride.btn"
+115. Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
+116. Collect Payment,tap,,"mobile.driver.collect_payment.btn"
+117. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+118. Confirm Payment,tap,,"mobile.driver.yes.btn"
+119. Give Rating,tap_coordinate,348:1545,
+120. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
+121. Load User App,switch_to,user,
+122. Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+123. Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
+124. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+125. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
+126. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
+127. Give Review,tap,,"mobile.customer.give_review.btn"
+128. Give Rating,tap_coordinate,348:1619,
+129. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
+130. Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
+131. Trip Finished,tap,,"mobile.customer.done.btn"</t>
+  </si>
+  <si>
+    <t>Removed Steps</t>
+  </si>
+  <si>
+    <t>7.Select Auto Ride Option,click,,"//span[normalize-space()='Auto Ride']"
+8.Wait for Auto Ride,wait_until_visible,,"//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"
+9.Click Auto Ride, click, , "//label[contains(.,'Driver Services')]/following-sibling::mat-checkbox"</t>
   </si>
 </sst>
 </file>
@@ -2869,7 +2871,7 @@
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>36</v>
@@ -2947,13 +2949,13 @@
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>49</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>37</v>
@@ -3018,13 +3020,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>15</v>
@@ -3093,19 +3095,19 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>13</v>
@@ -3169,22 +3171,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>77</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>87</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3213,7 +3215,7 @@
     <col min="4" max="4" width="35.5546875" customWidth="1"/>
     <col min="5" max="5" width="71.44140625" customWidth="1"/>
     <col min="6" max="6" width="29.6640625" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="7" max="7" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -3236,7 +3238,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>6</v>
@@ -3244,13 +3246,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
@@ -3259,7 +3261,10 @@
         <v>88</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3317,13 +3322,13 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
@@ -3332,7 +3337,7 @@
         <v>89</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3407,7 +3412,7 @@
         <v>44</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>30</v>
@@ -3558,7 +3563,7 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>54</v>
+        <v>85</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
@@ -3624,13 +3629,13 @@
         <v>19</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
@@ -3697,7 +3702,7 @@
         <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>32</v>
@@ -3773,7 +3778,7 @@
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
@@ -3851,13 +3856,13 @@
         <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>52</v>
@@ -3926,16 +3931,16 @@
         <v>48</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
70th Commit: Tranport Admin Locator File Created
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEECFB57-3AE6-43A9-8664-6F945368A9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFF04D7-0A0A-4ABD-8B02-B335DB125DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="94">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -2188,63 +2188,6 @@
 10.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"</t>
   </si>
   <si>
-    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-2. Click Customer Icon,click,,"admin.menu.customer_icon"
-3. Click Add Customers,click,,"admin.menu.add_customers"
-4. Wait For Customer Heading,wait_until_visible,,"admin.customer.add_heading"
-5. Enter Customer Name,type,customer{randomAlpha} &gt;&gt; customerName,"admin.customer.input_name"
-6. Enter Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
-7. Enter Contact Number,type,{randomPhone}&gt;&gt;userPhone,"admin.customer.input_phone"
-8.Enter Video Call Limit,type,50,"admin.customer.input_video_limit"
-9. Open Gender,click,,"admin.customer.dropdown_gender"
-10. Select Male,click,,"admin.customer.select_gender_male"
-11.Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
-12.Click Submit,click,,"web.global.action.submit"
-13. Wait For Added Successfully,wait_until_visible,,"web.global.toast.info"
-14.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-15.Click Customer Icon,click,,"admin.menu.customer_icon"
-16.Click Verified Customers,click,,"admin.menu.verified_customers"
-17. Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
-18.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
-  </si>
-  <si>
-    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-2. Click drivers menu,click,,"admin.drivers.menu.icon"
-3. Click Add Driver menu,click,,"admin.drivers.add_menu.link"
-4. Wait For Add Driver page,wait_until_visible,,"admin.drivers.add_page.header"
-5. Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
-6. Select Auto Ride Option,click,,"admin.drivers.service_option.autoride"
-7. Enter Driver Name,type,autodriver{randomAlpha} &gt;&gt; autoName,"admin.drivers.fullname.input"
-8. Enter Email,type,autodriver_{timestamp}@gmail.com &gt;&gt; autoEmail,"admin.drivers.email.input"
-9. Enter Contact Number,type,{randomPhone} &gt;&gt; autoPhone,"admin.drivers.phone.input"
-10. Click Whatsapp Checkbox,click,,"admin.drivers.whatsapp.checkbox"
-11. Enter Whatsapp Number,type,{autoPhone},"admin.drivers.whatsapp_phone.input"
-12. Upload Profile Image,uploadfile,"src/main/resources/test-data/autodriver.jpg","admin.drivers.profile_image.file"
-13. Click Select Source Dropdown,click,,"admin.drivers.source_dropdown.select"
-14. Select From Instagram Option,click,,"admin.drivers.instagram_option.span"
-15. Select Male Gender,click,,"admin.drivers.male_gender.div"
-16. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
-17. Select Pink Auto Option,click,,"admin.drivers.vehicle_option.pinkauto"
-18. Enter Model Year,type,2013,"admin.drivers.modelyear.input"
-19. Enter Plate No,type,KL-01-AB-1234,"admin.drivers.plateno.input"
-20. Enter Model Name,type,petrol,"admin.drivers.modelname.input"
-21. Upload Vehicle Image,uploadfile,"src/main/resources/test-data/vehicle.jpg","admin.drivers.vehicle_image.file"
-22. Enter Bank Name,type,HDFC Bank,"admin.drivers.bankname.input"
-23. Enter Bank Location,type,Chennai,"admin.drivers.banklocation.input"
-24. Enter Account Number,type,50100123456789,"admin.drivers.accountno.input"
-25. Enter Account Holder Name,type,{autoName},"admin.drivers.accountholder.input"
-26. Enter Payment Email Address,type,{autoEmail},"admin.drivers.paymentemail.input"
-27. Enter IFSC Code,type,HDFC0001234,"admin.drivers.ifsc.input"
-28. Click Submit Button,click,,"web.global.action.submit"
-29. Wait For Driver Added Successfully,wait_until_visible,,"web.global.toast.success"
-30. Wait for Toast to Hide,wait,1000,,
-31.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-32. Click drivers menu to refresh,click,,"admin.drivers.menu.icon"
-33. Click Pending Documents Menu,click,,"admin.drivers.pending_docs.link"
-34. Filter Pending Docs by Name,type,{autoName},"admin.drivers.name_filter.input"
-35. Click Dashboard Home Icon,click,,"web.global.menu.dashboard"</t>
-  </si>
-  <si>
     <t>1. Load Driver App,switch_to,driver,
 2. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
 3. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
@@ -2376,6 +2319,68 @@
 129. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
 130. Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
 131. Trip Finished,tap,,"mobile.customer.done.btn"</t>
+  </si>
+  <si>
+    <t>Deleted Test Case</t>
+  </si>
+  <si>
+    <t>8.Enter Video Call Limit,type,50,"admin.customer.input_video_limit"</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click Customer Icon,click,,"admin.menu.customer_icon"
+3. Click Add Customers,click,,"admin.menu.add_customers"
+4. Wait For Customer Heading,wait_until_visible,,"admin.customer.add_heading"
+5. Enter Customer Name,type,customer{randomAlpha} &gt;&gt; customerName,"admin.customer.input_name"
+6. Enter Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+7. Enter Contact Number,type,{randomPhone}&gt;&gt;userPhone,"admin.customer.input_phone"
+8. Open Gender,click,,"admin.customer.dropdown_gender"
+9. Select Male,click,,"admin.customer.select_gender_male"
+10.Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+11.Click Submit,click,,"web.global.action.submit"
+12. Wait For Added Successfully,wait_until_visible,,"web.global.toast.info"
+13.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+14.Click Customer Icon,click,,"admin.menu.customer_icon"
+15.Click Verified Customers,click,,"admin.menu.verified_customers"
+16. Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
+17.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click drivers menu,click,,"admin.drivers.menu.icon"
+3. Click Add Driver menu,click,,"admin.drivers.add_menu.link"
+4. Wait For Add Driver page,wait_until_visible,,"admin.drivers.add_page.header"
+5. Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
+6. Select Auto Ride Option,click,,"admin.drivers.service_dropdown.auto_ride"
+7. Enter Driver Name,type,autodriver{randomAlpha} &gt;&gt; autoName,"admin.drivers.fullname.input"
+8. Enter Email,type,autodriver_{timestamp}@gmail.com &gt;&gt; autoEmail,"admin.drivers.email.input"
+9. Enter Contact Number,type,{randomPhone} &gt;&gt; autoPhone,"admin.drivers.phone.input"
+10. Click Whatsapp Checkbox,click,,"admin.drivers.whatsapp.checkbox"
+11. Enter Whatsapp Number,type,{autoPhone},"admin.drivers.whatsapp_phone.input"
+12. Upload Profile Image,uploadfile,"src/main/resources/test-data/autodriver.jpg","admin.drivers.profile_image.file"
+13. Click Select Source Dropdown,click,,"admin.drivers.source_dropdown.select"
+14. Select From Instagram Option,click,,"admin.drivers.instagram_option.span"
+15. Select Male Gender,click,,"admin.drivers.male_gender.div"
+16. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
+17. Select Pink Auto Option,click,,"admin.drivers.vehicle_option.pinkauto"
+18. Enter Model Year,type,2013,"admin.drivers.modelyear.input"
+19. Enter Plate No,type,KL-01-AB-1234,"admin.drivers.plateno.input"
+20. Enter Model Name,type,petrol,"admin.drivers.modelname.input"
+21. Upload Vehicle Image,uploadfile,"src/main/resources/test-data/vehicle.jpg","admin.drivers.vehicle_image.file"
+22. Enter Bank Name,type,HDFC Bank,"admin.drivers.bankname.input"
+23. Enter Bank Location,type,Chennai,"admin.drivers.banklocation.input"
+24. Enter Account Number,type,50100123456789,"admin.drivers.accountno.input"
+25. Enter Account Holder Name,type,{autoName},"admin.drivers.accountholder.input"
+26. Enter Payment Email Address,type,{autoEmail},"admin.drivers.paymentemail.input"
+27. Enter IFSC Code,type,HDFC0001234,"admin.drivers.ifsc.input"
+28. Click Submit Button,click,,"web.global.action.submit"
+29. Wait For Driver Added Successfully,wait_until_visible,,"web.global.toast.success"
+30. Wait for Toast to Hide,wait,1000,,
+31.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+32. Click drivers menu to refresh,click,,"admin.drivers.menu.icon"
+33. Click Pending Documents Menu,click,,"admin.drivers.pending_docs.link"
+34. Filter Pending Docs by Name,type,{autoName},"admin.drivers.name_filter.input"
+35. Click Dashboard Home Icon,click,,"web.global.menu.dashboard"</t>
   </si>
 </sst>
 </file>
@@ -3139,7 +3144,7 @@
     <col min="4" max="4" width="31.6640625" customWidth="1"/>
     <col min="5" max="5" width="53.21875" customWidth="1"/>
     <col min="6" max="6" width="29" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+    <col min="7" max="7" width="42.44140625" customWidth="1"/>
     <col min="8" max="8" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3163,7 +3168,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>6</v>
@@ -3183,10 +3188,13 @@
         <v>75</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>76</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3258,7 +3266,7 @@
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>77</v>
@@ -3334,7 +3342,7 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
81th Commit: Regression Database Test Data File Created
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43545072-72FC-4B5E-B0C7-65ABABDE62D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2BAE396-E242-411B-94F7-B8A56ED8C1D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -19,7 +19,8 @@
     <sheet name="HybridApprovedAutoDriver" sheetId="38" r:id="rId4"/>
     <sheet name="HybridSubscriptionPlanTest" sheetId="40" r:id="rId5"/>
     <sheet name="AutoRideCompleteTest" sheetId="47" r:id="rId6"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId7"/>
+    <sheet name="DriverAppWalletVerificaton" sheetId="48" r:id="rId7"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="63">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -1101,277 +1102,6 @@
 49.Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"</t>
   </si>
   <si>
-    <t>1.Click badge,click,,"admin.subscription.badge.icon"
-2.Click Subscription Plan,click,,"admin.subscription.menu_link"
-3.Click Subscription Plan,click,,"admin.subscription.menu_link"
-4.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
-5.Verify Driver Subscription Plan Lists ,verify,,"admin.subscription.driver.header"
-6.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_add"
-7.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
-8.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
-9.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "admin.subscription.common.name.input"
-10.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
-11.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.input"
-12.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.input"
-13.Enter Number Of Days, type,100, "admin.subscription.common.days.alt_input"
-14.Enter Number Of Free Rides, type,2, "admin.subscription.driver.free_rides.input"
-15.Enter Price, type,5000, "admin.subscription.common.price.input"
-16.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.driver.desc_english.textarea"
-17.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.driver.desc_arabic.textarea"
-18.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.driver.desc_tamil.textarea"
-19.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.driver.desc_hindi.textarea"
-20.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
-21.Select On,click,,"admin.subscription.common.status.option_on"
-22.Click Submit ,click,,"web.global.action.submit"
-23.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
-24.Click badge,click,,"admin.subscription.badge.icon"
-25.Click Subscription Plan,click,,"admin.subscription.menu_link"
-26.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
-27.Verify Customer Subscription Plan Lists ,verify,,"admin.subscription.customer.header"
-28.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
-29.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
-30.Select Pest Control,click,,"admin.subscription.common.category.option_pest"
-31.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "admin.subscription.common.name.input"
-32.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
-33.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
-34.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
-35.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
-36.Enter Number Of Free Rides, type,2, "admin.subscription.customer.free_rides.input"
-37.Enter Price, type,5000, "admin.subscription.common.price.input"
-38.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.customer.desc_english.textarea"
-39.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.customer.desc_arabic.textarea"
-40.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.customer.desc_tamil.textarea"
-41.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.customer.desc_hindi.textarea"
-42.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
-43.Select On,click,,"admin.subscription.common.status.option_on"
-44.Click Submit ,click,,"web.global.action.submit"
-45.Filter Services List,type,{custometSubscriptionName},"admin.subscription.common.filter.input"
-46.Load User App,switch_to,user,
-47.Wait for Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-48.Click Get Started,tap,,"mobile.customer.get_started.btn"
-49.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-50.Click Next,tap,,"mobile.customer.next.btn"
-51.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-52.Click Close,tap,,"mobile.customer.cancel.btn"
-53.Enter Mobile Number,type,{userPhone},"mobile.customer.edit_text.input"
-54.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-55.Click Continue,tap,,"mobile.customer.continue.btn"
-56.Enter OTP,type,123456,"mobile.customer.edit_text.input"
-57.Click Finish,tap,,"mobile.customer.finish.btn"
-58.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-59.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
-60.Click Subscription,tap,,"mobile.customer.subscription.btn"
-61.Wait Customer Plan,wait_until_visible,,"mobile.customer.dynamic_subscription.plan"
-62.Click Customer Plan,tap,,"mobile.customer.dynamic_subscription.plan"
-63.Load Driver App,switch_to,driver,
-64.Wait for Popup,wait_until_visible,,"mobile.driver.permission_allow.btn"
-65.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-66.Click Agree,tap,,"mobile.driver.agree.btn"
-67.Click Get Started,tap,,"mobile.driver.get_started.btn"
-68.Click Next,tap,,"mobile.driver.next.btn"
-69.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-70.Click Close,tap,,"mobile.driver.cancel.btn"
-71.Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
-72.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-73.Click Continue,tap,,"mobile.driver.continue.btn"
-74.Enter OTP,type,123456,"mobile.driver.edit_text.input"
-75.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-76.Wait for Popup,wait_until_visible,,"mobile.driver.independent_contractor.checkbox"
-77.Click Independent Contractor,tap,,"mobile.driver.independent_contractor.checkbox"
-78.Click Legal Document,tap,,"mobile.driver.legal_document.checkbox"
-79.Click Safety Conduct,tap,,"mobile.driver.safety_conduct.checkbox"
-80.Click Subscription Model,tap,,"mobile.driver.subscription_model.checkbox"
-81.Drag Page Layout Upward,swipe,up,
-82.Click Liability,tap,,"mobile.driver.liability.checkbox"
-83.Click Data Protection,tap,,"mobile.driver.data_protection.checkbox"
-84.Click Fitness Declaration,tap,,"mobile.driver.fitness_declaration.checkbox"
-85.Click Confirmation,tap,,"mobile.driver.confirmation.checkbox"
-86.Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
-87.Click Agree,tap,,"mobile.driver.agree_continue.btn"
-88.Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
-89.Enter OTP,type,123456,"mobile.driver.edit_text.input"
-90.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-91.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-92.Click Subscription,tap,,"mobile.driver.subscription.btn"
-93.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
-94.Click Driver Plan,tap,,"mobile.driver.dynamic_subscription.plan"
-95.Click Back,tap,,"mobile.driver.back.btn"
-96.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
-97.Drag Page Layout Upward,swipe,up,
-98.Wait For Manage Account,wait_until_visible,,"mobile.driver.manage_account.btn"
-99.Click Manage Account,tap,,"mobile.driver.manage_account.btn"
-100.Wait For Logout,wait_until_visible,,"mobile.driver.logout.btn"
-101.Click Logout,tap,,"mobile.driver.logout.btn"
-102.Wait For Logout Popup,wait_until_visible,,"mobile.driver.logout.popup_btn"
-103.Click Logout Popup,tap,,"mobile.driver.logout.popup_btn"
-104.Load User App,switch_to,user,
-105.Click Back,tap,,"mobile.driver.back.btn"
-106.Wait For Profile Details,wait_until_visible,,"mobile.customer.account.heading"
-107.Drag Page Layout Upward,swipe,up,
-108.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
-109.Click Manage Account,tap,,"mobile.customer.manage_account.btn"
-110.Wait For Logout,wait_until_visible,,"mobile.customer.logout.btn"
-111.Click Logout,tap,,"mobile.customer.logout.btn"
-112.Wait For Logout Popup,wait_until_visible,,"mobile.customer.logout.popup_btn"
-113.Click Logout Popup,tap,,"mobile.customer.logout.popup_btn"
-114.Reload User App Completely,reload_app,user,
-115.Reload Driver App Completely,reload_app,driver,</t>
-  </si>
-  <si>
-    <t>1. Load Driver App,switch_to,driver,
-2. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-3. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-4. Click Agree,tap,,"mobile.driver.agree.btn"
-5. Click Get Started,tap,,"mobile.driver.get_started.btn"
-6. Click Next,tap,,"mobile.driver.next.btn"
-7. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-8. Click Close,tap,,"mobile.driver.cancel.btn"
-9. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
-10. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-11. Click Continue,tap,,"mobile.driver.continue.btn"
-12. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-13. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-14. Wait For Popup,wait_until_visible,,"mobile.driver.independent_contractor.checkbox"
-15. Click Independent Contractor,tap,,"mobile.driver.independent_contractor.checkbox"
-16. Click Legal Document,tap,,"mobile.driver.legal_document.checkbox"
-17. Click Safety Conduct,tap,,"mobile.driver.safety_conduct.checkbox"
-18. Click Subscription Model,tap,,"mobile.driver.subscription_model.checkbox"
-19. Drag Page Layout Upward,swipe,up,
-20. Click Liability,tap,,"mobile.driver.liability.checkbox"
-21. Click Data Protection,tap,,"mobile.driver.data_protection.checkbox"
-22. Click Fitness Declaration,tap,,"mobile.driver.fitness_declaration.checkbox"
-23. Click Confirmation,tap,,"mobile.driver.confirmation.checkbox"
-24. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
-25. Click Agree,tap,,"mobile.driver.agree_continue.btn"
-26. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
-27. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-28. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-29. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-30. Click Document,tap,,"mobile.driver.documents.menu"
-31. Wait For Document Page,wait_until_visible,,"mobile.driver.add_documents.header"
-32. Wait For Upload,wait_until_visible,,"mobile.driver.upload.btn"
-33. Click Upload,tap,,"mobile.driver.upload.btn"
-34. Upload License,uploadfile,"src/main/resources/test-data/license.JPG","mobile.driver.upload_docs.btn"
-35. Wait For Sort,wait_until_visible,,"mobile.driver.android_content.view"
-36. Click Sort,tap,,"mobile.driver.android_content.view"
-37. Wait For Modified,wait_until_visible,,"mobile.driver.sort_modified.btn"
-38. Click Modified,tap,,"mobile.driver.sort_modified.btn"
-39. Click License,tap,,"mobile.driver.license_thumb.icon"
-40. Wait For Crop,wait_until_visible,,"mobile.driver.crop.btn"
-41. Click Crop,tap,,"mobile.driver.crop.btn"
-42. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
-43. Click Calendar,tap_coordinate,121:1539,COORDINATE_MODE
-44. Click Month,tap,,"mobile.driver.next_month.btn"
-45. Click Date,tap_coordinate,943:1290,COORDINATE_MODE
-46. Click Ok,tap,,"mobile.driver.ok.btn"
-47. Click Upload Submission,tap,,"mobile.driver.upload_docs.btn"
-48. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
-49. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
-50. Click Back,tap,,"mobile.driver.back.btn"
-51. Load Admin App,switch_to,web,
-52. Wait For Dashboard,wait_until_visible,,"web.global.menu.dashboard"
-53. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-54. Click drivers menu,click,,"admin.drivers.menu.icon"
-55. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
-56. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
-57. Scroll Grid,tab,7,"admin.drivers.name_filter.input"
-58. Click Doc Icon,click,,"admin.drivers.docs.icon"
-59. Wait For Required Documents,wait_until_visible,,"admin.drivers.required_docs.header"
-60. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
-61. Click Approve Driver,click,,"admin.drivers.docs.approval"
-62. Wait For Updated Successfully,wait_until_visible,,"web.global.toast.updated"
-63. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-64. Click drivers menu,click,,"admin.drivers.menu.icon"
-65. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
-66.Wait For Approved Drivers List,wait_until_visible,,"admin.drivers.approved_page.header"
-67. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
-68. Load Driver App,switch_to,driver,
-69. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
-70. Click Document,tap,,"mobile.driver.documents.menu"
-71. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
-72. Click Back,tap,,"mobile.driver.back.btn"
-73. Wait For Documents,wait_until_visible,,"mobile.driver.documents.menu"
-74. Click Back,tap,,"mobile.driver.back.btn"
-75. Click Online,tap_coordinate,986:1936,
-76. Load User App,switch_to,user,
-77. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-78. Click Get Started,tap,,"mobile.customer.get_started.btn"
-79. Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-80. Click Next,tap,,"mobile.customer.next.btn"
-81. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-82. Click Close,tap,,"mobile.customer.cancel.btn"
-83. Enter Mobile Number,type,{userPhone},"mobile.customer.edit_text.input"
-84. Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-85. Click Continue,tap,,"mobile.customer.continue.btn"
-86. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-87. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
-88. Click Finish,tap,,"mobile.customer.finish.btn"
-89. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-90. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
-91. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
-92. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
-93. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
-94. Select Destination,tap_coordinate,545:1299,
-95. Click Confirm,tap,,"mobile.customer.confirm.btn"
-96. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
-97. Ride Now,tap,,"mobile.customer.ride_now.btn"
-98. Load Driver App,switch_to,driver,
-99. Wait for Accept,wait_until_visible,,"mobile.driver.auto_ride_notification.label"
-100. Accept Ride,tap_coordinate,801:2113,
-101. Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
-102. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
-103. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
-104. Ride Arrived,tap,,"mobile.driver.arrived.btn"
-105. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
-106. Yes Arrived,tap,,"mobile.driver.yes.btn"
-107. Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
-108. Start Ride,tap,,"mobile.driver.start_ride.btn"
-109. Wait for OTP,wait_until_visible,,"mobile.driver.otp_view.input"
-110. Enter OTP,type,1234,"mobile.driver.otp_view.input"
-111. Wait for Start Ride Confirm,wait_until_visible,,"mobile.driver.start.btn"
-112. Start Ride Confirm,tap,,"mobile.driver.start.btn"
-113. Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
-114. Complete Ride,tap,,"mobile.driver.complete_ride.btn"
-115. Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
-116. Collect Payment,tap,,"mobile.driver.collect_payment.btn"
-117. Load User App,switch_to,user,
-118. Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
-119. Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
-120. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
-121. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
-122. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
-123. Give Review,tap,,"mobile.customer.give_review.btn"
-124. Give Rating,tap_coordinate,348:1619,
-125. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
-126. Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
-127. Trip Finished,tap,,"mobile.customer.done.btn"
-128.Wait for Back,wait_until_visible,,"mobile.driver.back.btn"
-129.Click Back,tap,,"mobile.driver.back.btn"
-130.Wait for Profile Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
-130.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
-131.Wait For Profile Details,wait_until_visible,,"mobile.customer.account.heading"
-132.Drag Page Layout Upward,swipe,up,
-133.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
-134.Click Manage Account,tap,,"mobile.customer.manage_account.btn"
-135.Wait For Logout,wait_until_visible,,"mobile.customer.logout.btn"
-136.Click Logout,tap,,"mobile.customer.logout.btn"
-137.Wait For Logout Popup,wait_until_visible,,"mobile.customer.logout.popup_btn"
-138.Click Logout Popup,tap,,"mobile.customer.logout.popup_btn"
-139.Load Driver App,switch_to,driver,
-140 Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-141.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-142.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
-143.Drag Page Layout Upward,swipe,up,
-144.Wait For Manage Account,wait_until_visible,,"mobile.driver.manage_account.btn"
-145.Click Manage Account,tap,,"mobile.driver.manage_account.btn"
-146.Wait For Logout,wait_until_visible,,"mobile.driver.logout.btn"
-147.Click Logout,tap,,"mobile.driver.logout.btn"
-148.Wait For Logout Popup,wait_until_visible,,"mobile.driver.logout.popup_btn"
-149.Click Logout Popup,tap,,"mobile.driver.logout.popup_btn"
-150.Reload User App Completely,reload_app,user,
-151.Reload Driver App Completely,reload_app,driver,</t>
-  </si>
-  <si>
     <t xml:space="preserve">1. Load User App,switch_to,user,
 2. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
 3. Load Driver App,switch_to,driver,
@@ -1382,6 +1112,476 @@
 8. Enter Password,type,R1mep@321,"web.global.login.password"
 9. Click Login,click,,"web.global.login.submit_btn"
 10.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
+</t>
+  </si>
+  <si>
+    <t>TC_CA_06_Driver_App_Wallet_Verification</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The UserDriverWebIntialilzer,HybridAddCustomer and  HybridUnApprovedAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>UserDriverWebIntialilzer</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
+    <t>This end-to-end hybrid regression test verifies the runtime visibility and functionality of the mobile Driver Wallet module based on configurations managed within the Super Admin Web Portal. The execution workflow first activates the wallet feature via the admin portal's site settings, logs into the driver application, and executes a full simulated wallet top-up transaction using Net Banking to confirm operational stability. It then reverts to the web panel to toggle the wallet status to "OFF," restarts the mobile application context to clear active sessions, re-authenticates the driver, and explicitly asserts that the Wallet option is completely absent from the side menu hierarchy.</t>
+  </si>
+  <si>
+    <t>Driver App Wallet Verification</t>
+  </si>
+  <si>
+    <t>1. Load Driver App,switch_to,driver,
+2.Reload Driver App Completely,reload_app,driver,
+3. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+4. Load Super Admin,switch_to,web,
+5.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
+6. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+7. Click Settings Menu,click,,"web.global.menu.settings"
+8. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+9. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+10.Wait For On,wait,2000,
+11. Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+12. Click Submit Button,click,,"web.global.action.submit"
+13. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+14. Load Driver App,switch_to,driver,
+15. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+16. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+17. Click Agree,tap,,"mobile.driver.agree.btn"
+18. Click Get Started,tap,,"mobile.driver.get_started.btn"
+19. Click Next,tap,,"mobile.driver.next.btn"
+20. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+21. Click Close,tap,,"mobile.driver.cancel.btn"
+22. Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+23. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+24. Click Continue,tap,,"mobile.driver.continue.btn"
+25. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+26. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+27. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+28. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+29.wait for Wallet,wait_until_visible,"mobile.driver.wallet.btn"
+30.Click Wallet,tap,,"mobile.driver.wallet.btn"
+31.Wait For Topup,wait_until_visible,,"mobile.driver.top_up.btn"
+32.Click Topup,tap,,"mobile.driver.top_up.btn"
+33.Wait For Topup Sum,wait_until_visible,,"mobile.driver.top_up.btn"
+34.Click Hundered,tap,,"mobile.driver.top_up_amount.hundred"
+35.Click Proceed,tap,,"mobile.driver.top_up.proceed"
+36.Wait For Contact No,wait_until_visible,,"mobile.driver.top_up.contact_no_box"
+37.Enter Driver Mobile,type,regression.approved_driver.phone,"mobile.driver.top_up.contact_no_box"
+38.Wait For Payment Options,wait_until_visible,,"mobile.driver.top_up.payment_option"
+39.Wait For Net Banking,wait,3000,
+40.Click Net Banking,tap,,"mobile.driver.top_up.net_banking"
+41.Click Bob,tap_coordinate,277:1124,
+42.Wait For Success,wait_until_visible,,"mobile.driver.top_up.succes_popup"
+43.Click Success,tap,,"mobile.driver.top_up.succes_popup"
+44.Wait For Wallet  Back,wait_until_visible,,"mobile.driver.wallet.btn"
+45.Click Back,tap,,"mobile.driver.back.btn"
+46.Drag Page Layout Upward,swipe,up,
+47.Click Back,tap,,"mobile.driver.back.btn"
+48.Reload Driver App Completely,reload_app,driver,
+49. Switch To Web Session,switch_to,web,
+50.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+51. Click Settings Menu,click,,"admin.setting.sidebar.menu"
+52. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+53. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+54.Wait For off,wait,2000,
+55. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
+56. Click Submit Button,click,,"web.global.action.submit"
+57. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+58. Switch To Driver Session,switch_to,driver,
+59. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+60. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+61. Click Agree,tap,,"mobile.driver.agree.btn"
+62. Click Get Started,tap,,"mobile.driver.get_started.btn"
+63. Click Next,tap,,"mobile.driver.next.btn"
+64. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+65. Click Close,tap,,"mobile.driver.cancel.btn"
+66. Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+67. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+68. Click Continue,tap,,"mobile.driver.continue.btn"
+69. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+70. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+71. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+72.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+73.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
+74.Check Wallet absent,element_absent,,"accessibility=Wallet"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3. Load Driver App,switch_to,driver,
+4. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+5. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+6. Click Agree,tap,,"mobile.driver.agree.btn"
+7. Click Get Started,tap,,"mobile.driver.get_started.btn"
+8. Click Next,tap,,"mobile.driver.next.btn"
+9. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+10. Click Close,tap,,"mobile.driver.cancel.btn"
+11. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+12. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+13. Click Continue,tap,,"mobile.driver.continue.btn"
+14. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+15. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+16. Wait For Popup,wait_until_visible,,"mobile.driver.independent_contractor.checkbox"
+17. Click Independent Contractor,tap,,"mobile.driver.independent_contractor.checkbox"
+18. Click Legal Document,tap,,"mobile.driver.legal_document.checkbox"
+19. Click Safety Conduct,tap,,"mobile.driver.safety_conduct.checkbox"
+20. Click Subscription Model,tap,,"mobile.driver.subscription_model.checkbox"
+21. Drag Page Layout Upward,swipe,up,
+22. Click Liability,tap,,"mobile.driver.liability.checkbox"
+23. Click Data Protection,tap,,"mobile.driver.data_protection.checkbox"
+24. Click Fitness Declaration,tap,,"mobile.driver.fitness_declaration.checkbox"
+25. Click Confirmation,tap,,"mobile.driver.confirmation.checkbox"
+26. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+27. Click Agree,tap,,"mobile.driver.agree_continue.btn"
+28. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+29. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+30. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+31. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+32. Click Document,tap,,"mobile.driver.documents.menu"
+33. Wait For Document Page,wait_until_visible,,"mobile.driver.add_documents.header"
+34. Wait For Upload,wait_until_visible,,"mobile.driver.upload.btn"
+35. Click Upload,tap,,"mobile.driver.upload.btn"
+36. Upload License,uploadfile,"src/main/resources/test-data/license.JPG","mobile.driver.upload_docs.btn"
+37. Wait For Sort,wait_until_visible,,"mobile.driver.android_content.view"
+38. Click Sort,tap,,"mobile.driver.android_content.view"
+39. Wait For Modified,wait_until_visible,,"mobile.driver.sort_modified.btn"
+40. Click Modified,tap,,"mobile.driver.sort_modified.btn"
+41. Click License,tap,,"mobile.driver.license_thumb.icon"
+42. Wait For Crop,wait_until_visible,,"mobile.driver.crop.btn"
+43. Click Crop,tap,,"mobile.driver.crop.btn"
+44. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+45. Click Calendar,tap_coordinate,121:1539,COORDINATE_MODE
+46. Click Month,tap,,"mobile.driver.next_month.btn"
+47. Click Date,tap_coordinate,943:1290,COORDINATE_MODE
+48. Click Ok,tap,,"mobile.driver.ok.btn"
+49. Click Upload Submission,tap,,"mobile.driver.upload_docs.btn"
+50. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+51. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+52. Click Back,tap,,"mobile.driver.back.btn"
+53. Load Admin App,switch_to,web,
+54. Wait For Dashboard,wait_until_visible,,"web.global.menu.dashboard"
+55. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+56. Click drivers menu,click,,"admin.drivers.menu.icon"
+57. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+58. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+59. Scroll Grid,tab,7,"admin.drivers.name_filter.input"
+60. Click Doc Icon,click,,"admin.drivers.docs.icon"
+61. Wait For Required Documents,wait_until_visible,,"admin.drivers.required_docs.header"
+62. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+63. Click Approve Driver,click,,"admin.drivers.docs.approval"
+64. Wait For Updated Successfully,wait_until_visible,,"web.global.toast.updated"
+65. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+66. Click drivers menu,click,,"admin.drivers.menu.icon"
+67. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+68.Wait For Approved Drivers List,wait_until_visible,,"admin.drivers.approved_page.header"
+69. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+70. Load Driver App,switch_to,driver,
+71. Wait For Back,wait_until_visible,,"mobile.driver.back.btn"
+72. Click Document,tap,,"mobile.driver.documents.menu"
+73. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+74. Click Back,tap,,"mobile.driver.back.btn"
+75. Wait For Documents,wait_until_visible,,"mobile.driver.documents.menu"
+76. Click Back,tap,,"mobile.driver.back.btn"
+77. Click Online,tap_coordinate,986:1936,
+78. Load User App,switch_to,user,
+79. Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+80. Click Get Started,tap,,"mobile.customer.get_started.btn"
+81. Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+82. Click Next,tap,,"mobile.customer.next.btn"
+83. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+84. Click Close,tap,,"mobile.customer.cancel.btn"
+85. Enter Mobile Number,type,{userPhone},"mobile.customer.edit_text.input"
+86. Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+87. Click Continue,tap,,"mobile.customer.continue.btn"
+88. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+89. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+90. Click Finish,tap,,"mobile.customer.finish.btn"
+91. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+92. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+93. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+94. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+95. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+96. Select Destination,tap_coordinate,545:1299,
+97. Click Confirm,tap,,"mobile.customer.confirm.btn"
+98. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+99. Ride Now,tap,,"mobile.customer.ride_now.btn"
+100. Load Driver App,switch_to,driver,
+101. Wait for Accept,wait_until_visible,,"mobile.driver.auto_ride_notification.label"
+102. Accept Ride,tap_coordinate,801:2113,
+103. Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
+104. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+105. Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+106. Ride Arrived,tap,,"mobile.driver.arrived.btn"
+107. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+108. Yes Arrived,tap,,"mobile.driver.yes.btn"
+109. Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
+110. Start Ride,tap,,"mobile.driver.start_ride.btn"
+111. Wait for OTP,wait_until_visible,,"mobile.driver.otp_view.input"
+112. Enter OTP,type,1234,"mobile.driver.otp_view.input"
+113. Wait for Start Ride Confirm,wait_until_visible,,"mobile.driver.start.btn"
+114. Start Ride Confirm,tap,,"mobile.driver.start.btn"
+115. Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
+116. Complete Ride,tap,,"mobile.driver.complete_ride.btn"
+117. Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
+118. Collect Payment,tap,,"mobile.driver.collect_payment.btn"
+119. Load User App,switch_to,user,
+120. Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+121. Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
+122. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+123. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
+124. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
+125. Give Review,tap,,"mobile.customer.give_review.btn"
+126. Give Rating,tap_coordinate,348:1619,
+127. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
+128. Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
+129. Trip Finished,tap,,"mobile.customer.done.btn"
+130.Wait for Back,wait_until_visible,,"mobile.driver.back.btn"
+131.Click Back,tap,,"mobile.driver.back.btn"
+132.Wait for Profile Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
+133.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
+134.Wait For Profile Details,wait_until_visible,,"mobile.customer.account.heading"
+135.Drag Page Layout Upward,swipe,up,
+136.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
+137.Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+138.Wait For Logout,wait_until_visible,,"mobile.customer.logout.btn"
+139.Click Logout,tap,,"mobile.customer.logout.btn"
+140.Wait For Logout Popup,wait_until_visible,,"mobile.customer.logout.popup_btn"
+141.Click Logout Popup,tap,,"mobile.customer.logout.popup_btn"
+142.Load Driver App,switch_to,driver,
+143. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+144.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+145.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
+146.Drag Page Layout Upward,swipe,up,
+147.Wait For Manage Account,wait_until_visible,,"mobile.driver.manage_account.btn"
+148.Click Manage Account,tap,,"mobile.driver.manage_account.btn"
+149.Wait For Logout,wait_until_visible,,"mobile.driver.logout.btn"
+150.Click Logout,tap,,"mobile.driver.logout.btn"
+151.Wait For Logout Popup,wait_until_visible,,"mobile.driver.logout.popup_btn"
+152.Click Logout Popup,tap,,"mobile.driver.logout.popup_btn"
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3.Load Super Admin,switch_to,web,
+4.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+5.Click Subscription Plan,click,,"admin.subscription.menu_link"
+6.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
+7.Verify Driver Subscription Plan Lists ,verify,,"admin.subscription.driver.header"
+8.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_add"
+9.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+10.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
+11.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "admin.subscription.common.name.input"
+12.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+13.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.input"
+14.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.input"
+15.Enter Number Of Days, type,100, "admin.subscription.common.days.alt_input"
+16.Enter Number Of Free Rides, type,2, "admin.subscription.driver.free_rides.input"
+17.Enter Price, type,5000, "admin.subscription.common.price.input"
+18.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.driver.desc_english.textarea"
+19.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.driver.desc_arabic.textarea"
+20.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.driver.desc_tamil.textarea"
+21.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.driver.desc_hindi.textarea"
+22.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+23.Select On,click,,"admin.subscription.common.status.option_on"
+24.Click Submit ,click,,"web.global.action.submit"
+25.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
+26.Click badge,click,,"admin.subscription.badge.icon"
+27.Click Subscription Plan,click,,"admin.subscription.menu_link"
+28.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
+29.Verify Customer Subscription Plan Lists ,verify,,"admin.subscription.customer.header"
+30.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
+31.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+32.Select Pest Control,click,,"admin.subscription.common.category.option_pest"
+33.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "admin.subscription.common.name.input"
+34.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+35.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
+36.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
+37.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
+38.Enter Number Of Free Rides, type,2, "admin.subscription.customer.free_rides.input"
+39.Enter Price, type,5000, "admin.subscription.common.price.input"
+40.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.customer.desc_english.textarea"
+41.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.customer.desc_arabic.textarea"
+42.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.customer.desc_tamil.textarea"
+43.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.customer.desc_hindi.textarea"
+44.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+45.Select On,click,,"admin.subscription.common.status.option_on"
+46.Click Submit ,click,,"web.global.action.submit"
+47.Filter Services List,type,{custometSubscriptionName},"admin.subscription.common.filter.input"
+48.Load User App,switch_to,user,
+49.Wait for Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+50.Click Get Started,tap,,"mobile.customer.get_started.btn"
+51.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+52.Click Next,tap,,"mobile.customer.next.btn"
+53.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+54.Click Close,tap,,"mobile.customer.cancel.btn"
+55.Enter Mobile Number,type,{userPhone},"mobile.customer.edit_text.input"
+56.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+57.Click Continue,tap,,"mobile.customer.continue.btn"
+58.Enter OTP,type,123456,"mobile.customer.edit_text.input"
+59.Click Finish,tap,,"mobile.customer.finish.btn"
+60.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+61.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
+62.Click Subscription,tap,,"mobile.customer.subscription.btn"
+63.Wait Customer Plan,wait_until_visible,,"mobile.customer.dynamic_subscription.plan"
+64.Click Customer Plan,tap,,"mobile.customer.dynamic_subscription.plan"
+65.Load Driver App,switch_to,driver,
+66.Wait for Popup,wait_until_visible,,"mobile.driver.permission_allow.btn"
+67.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+68.Click Agree,tap,,"mobile.driver.agree.btn"
+69.Click Get Started,tap,,"mobile.driver.get_started.btn"
+70.Click Next,tap,,"mobile.driver.next.btn"
+71.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+72.Click Close,tap,,"mobile.driver.cancel.btn"
+73.Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+74.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+75.Click Continue,tap,,"mobile.driver.continue.btn"
+76.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+77.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+78.Wait for Popup,wait_until_visible,,"mobile.driver.independent_contractor.checkbox"
+79.Click Independent Contractor,tap,,"mobile.driver.independent_contractor.checkbox"
+80.Click Legal Document,tap,,"mobile.driver.legal_document.checkbox"
+81.Click Safety Conduct,tap,,"mobile.driver.safety_conduct.checkbox"
+82.Click Subscription Model,tap,,"mobile.driver.subscription_model.checkbox"
+83.Drag Page Layout Upward,swipe,up,
+84.Click Liability,tap,,"mobile.driver.liability.checkbox"
+85.Click Data Protection,tap,,"mobile.driver.data_protection.checkbox"
+86.Click Fitness Declaration,tap,,"mobile.driver.fitness_declaration.checkbox"
+87.Click Confirmation,tap,,"mobile.driver.confirmation.checkbox"
+88.Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+89.Click Agree,tap,,"mobile.driver.agree_continue.btn"
+90.Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+91.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+92.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+93.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+94.Click Subscription,tap,,"mobile.driver.subscription.btn"
+95.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
+96.Click Driver Plan,tap,,"mobile.driver.dynamic_subscription.plan"
+97.Click Back,tap,,"mobile.driver.back.btn"
+98.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
+99.Drag Page Layout Upward,swipe,up,
+100.Wait For Manage Account,wait_until_visible,,"mobile.driver.manage_account.btn"
+101.Click Manage Account,tap,,"mobile.driver.manage_account.btn"
+102.Wait For Logout,wait_until_visible,,"mobile.driver.logout.btn"
+103.Click Logout,tap,,"mobile.driver.logout.btn"
+104.Wait For Logout Popup,wait_until_visible,,"mobile.driver.logout.popup_btn"
+105.Click Logout Popup,tap,,"mobile.driver.logout.popup_btn"
+106.Load User App,switch_to,user,
+107.Click Back,tap,,"mobile.driver.back.btn"
+108.Wait For Profile Details,wait_until_visible,,"mobile.customer.account.heading"
+109.Drag Page Layout Upward,swipe,up,
+110.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
+111.Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+112.Wait For Logout,wait_until_visible,,"mobile.customer.logout.btn"
+113.Click Logout,tap,,"mobile.customer.logout.btn"
+114.Wait For Logout Popup,wait_until_visible,,"mobile.customer.logout.popup_btn"
+115.Click Logout Popup,tap,,"mobile.customer.logout.popup_btn"
 </t>
   </si>
 </sst>
@@ -1808,7 +2008,7 @@
         <v>32</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>33</v>
@@ -2110,7 +2310,7 @@
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>46</v>
@@ -2188,7 +2388,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>51</v>
@@ -2218,6 +2418,90 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD2DD3E8-3167-4AD5-B95A-26FB801D55E0}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
85th Commit: Transport Tests Grouped
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3F198C7-8137-4687-9FE2-30D186D66542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F080529-5D24-4920-8028-5C96D944EE91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -18,9 +18,9 @@
     <sheet name="HybridUnApprovedAutoDriver" sheetId="46" r:id="rId3"/>
     <sheet name="HybridApprovedAutoDriver" sheetId="38" r:id="rId4"/>
     <sheet name="HybridSubscriptionPlanTest" sheetId="40" r:id="rId5"/>
-    <sheet name="AutoRideCompleteTest" sheetId="47" r:id="rId6"/>
-    <sheet name="DriverAppWalletVerificaton" sheetId="48" r:id="rId7"/>
-    <sheet name="NonVerifiedAndDeletedCustomer" sheetId="50" r:id="rId8"/>
+    <sheet name="DriverAppWalletVerificaton" sheetId="48" r:id="rId6"/>
+    <sheet name="NonVerifiedAndDeletedCustomer" sheetId="50" r:id="rId7"/>
+    <sheet name="AutoRideCompleteTest" sheetId="47" r:id="rId8"/>
     <sheet name="CustomerLanguageCheck" sheetId="52" r:id="rId9"/>
     <sheet name="DriverLanguageCheck" sheetId="53" r:id="rId10"/>
     <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId11"/>
@@ -2040,15 +2040,6 @@
     <t>Subscriptin Plan Complete Test</t>
   </si>
   <si>
-    <t>TC_CA_02_Autoride_Complete_Test</t>
-  </si>
-  <si>
-    <t>TC_CA_03_Driver_App_Wallet_Verification</t>
-  </si>
-  <si>
-    <t>TC_CA_04_Non_Verified_And_Deleted_Customer</t>
-  </si>
-  <si>
     <t>This comprehensive, cross-platform regression test suite validates the entire lifecycle of a customer account by seamlessly orchestrating actions between native mobile applications and the centralized web administration portal. The test sequence begins by initializing a fresh mobile session using the reload_app utility, executing a new user registration flow via dynamic device permissions, randomized phone generation, and OTP simulation. The execution then seamlessly switches context to the web portal to locate the newly created profile under the Non-Verified Customers matrix, populates missing metadata (including automated profile image uploads and randomized alpha naming strings), and submits the profile to trigger status escalation. After confirming the user's migration into the Verified Customers data grid, the execution switches back to the mobile application instance to verify verified account access. Finally, the test validates data-compliance workflows by triggering a native Delete Account chain from the mobile device settings and cross-verifying that the user profile is immediately and correctly relocated to the web admin’s Deleted Customers repository.</t>
   </si>
   <si>
@@ -2166,6 +2157,15 @@
 97.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
 98.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
 99.Wait For Deletion,wait,2000,</t>
+  </si>
+  <si>
+    <t>TC_CA_02_Driver_App_Wallet_Verification</t>
+  </si>
+  <si>
+    <t>TC_CA_03_Non_Verified_And_Deleted_Customer</t>
+  </si>
+  <si>
+    <t>TC_CA_04_Autoride_Complete_Test</t>
   </si>
 </sst>
 </file>
@@ -2661,10 +2661,10 @@
         <v>61</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>65</v>
@@ -2742,7 +2742,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>9</v>
@@ -3049,7 +3049,7 @@
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>52</v>
@@ -3079,6 +3079,174 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD2DD3E8-3167-4AD5-B95A-26FB801D55E0}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{437C624E-95B4-48EB-A315-8931C834404A}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1895CC0E-D326-49C3-B5DA-E3C80EEAE5A9}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3121,13 +3289,13 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>14</v>
@@ -3143,174 +3311,6 @@
       </c>
       <c r="H2" s="2" t="s">
         <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD2DD3E8-3167-4AD5-B95A-26FB801D55E0}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{437C624E-95B4-48EB-A315-8931C834404A}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3379,10 +3379,10 @@
         <v>60</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>63</v>

</xml_diff>

<commit_message>
87th Commit: Data Base Run Time Value Fetching Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F080529-5D24-4920-8028-5C96D944EE91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59D0F3CD-37E1-4054-B8E3-45FFC72A06DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="HybridSubscriptionPlanTest" sheetId="40" r:id="rId5"/>
     <sheet name="DriverAppWalletVerificaton" sheetId="48" r:id="rId6"/>
     <sheet name="NonVerifiedAndDeletedCustomer" sheetId="50" r:id="rId7"/>
-    <sheet name="AutoRideCompleteTest" sheetId="47" r:id="rId8"/>
+    <sheet name="AutoRideCompleteTest" sheetId="54" r:id="rId8"/>
     <sheet name="CustomerLanguageCheck" sheetId="52" r:id="rId9"/>
     <sheet name="DriverLanguageCheck" sheetId="53" r:id="rId10"/>
     <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId11"/>
@@ -1559,92 +1559,6 @@
 18.Click Online Toggle Button,tap,,"mobile.driver.online_toggle.btn"</t>
   </si>
   <si>
-    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
-2.Reload Driver App Completely,reload_app,driver,
-3.Load Driver App,switch_to,driver,
-4.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-5.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-6.Click Agree,tap,,"mobile.driver.agree.btn"
-7.Click Get Started,tap,,"mobile.driver.get_started.btn"
-8.Click Next,tap,,"mobile.driver.next.btn"
-9.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-10.Click Close,tap,,"mobile.driver.cancel.btn"
-11.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
-12.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-13 Click Continue,tap,,"mobile.driver.continue.btn"
-14. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-15.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-16.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-17.Wait For Pageload,wait,3000,
-18.Load User App,switch_to,user,
-19.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-20.Click Get Started,tap,,"mobile.customer.get_started.btn"
-21.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-22.Click Next,tap,,"mobile.customer.next.btn"
-23.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-24.Click Close,tap,,"mobile.customer.cancel.btn"
-25.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
-26.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-27. Click Continue,tap,,"mobile.customer.continue.btn"
-28. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-29. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
-30. Click Finish,tap,,"mobile.customer.finish.btn"
-31. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-32. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
-33. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
-34. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
-35. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
-36. Select Destination,tap_coordinate,545:1299,
-37. Click Confirm,tap,,"mobile.customer.confirm.btn"
-38. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
-39. Ride Now,tap,,"mobile.customer.ride_now.btn"
-40. Load Driver App,switch_to,driver,
-41.Wait for Accept,wait_until_visible,,"mobie.driver.auto_ride_accept.button"
-42.Click  Accept Ride,tap,,"mobie.driver.auto_ride_accept.button"
-43.Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
-44.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
-45.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
-46.Ride Arrived,tap,,"mobile.driver.arrived.btn"
-47.Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
-48.Yes Arrived,tap,,"mobile.driver.yes.btn"
-49.Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
-50.Start Ride,tap,,"mobile.driver.start_ride.btn"
-51.wait for Otp,wait_until_visible,,"mobile.driver.otp_view.input"
-52.Enter OTP,type,1234,"mobile.driver.otp_view.input"
-53.Wait for Start Button,wait_until_visible,,"mobile.driver.start.btn"
-54.Start Ride Button,tap,,"mobile.driver.start.btn"
-55.Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
-56.Complete Ride,tap,,"mobile.driver.complete_ride.btn"
-57.Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
-58.Collect Payment,tap,,"mobile.driver.collect_payment.btn"
-59.Load User App,switch_to,user,
-60.Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
-61.Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
-62. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
-63. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
-64. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
-65. Give Review,tap,,"mobile.customer.give_review.btn"
-66. Give Rating,tap_coordinate,348:1619,
-67. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
-68.Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
-69.Trip Finished,tap,,"mobile.customer.done.btn"
-70. Load Driver App,switch_to,driver,
-71.Wait  For Proceed,wait_until_visible,,"mobile.driver.payment.proceed_btn"
-72.Click For Proceed,tap,,"mobile.driver.payment.proceed_btn"
-73. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
-74. Confirm Payment,tap,,"mobile.driver.yes.btn"
-75.Wait For Give Review Button,wait_until_visible,,"mobile.driver.give_review.btn"
-76.Click Give Review Button,tap,,"mobile.driver.give_review.btn"
-77.Wait For Rating,wait,2000,
-78. Give Rating,tap_coordinate,348:1545,
-79. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
-80.Wait for Complete Button,wait_until_visible,,"mobile.driver.complete.btn"
-81.Click Complete Button,tap,,"mobile.driver.complete.btn"
-82.Wait For  ride complete submit button,wait_until_visible,,"mobile.driver.ride_complete_submit.btn"
-83.Click Ride Complete Submit Button,tap,,"mobile.driver.ride_complete_submit.btn"
-</t>
-  </si>
-  <si>
     <t>1. Load Driver App,switch_to,driver,
 2.Reload Driver App Completely,reload_app,driver,
 3. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
@@ -1732,167 +1646,6 @@
   </si>
   <si>
     <t>Driver Language Check</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
-2.Reload Driver App Completely,reload_app,driver,
-3. Load User App,switch_to,user,
-4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-5. Click Get Started,tap,,"mobile.customer.get_started.btn"
-6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
-7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
-8. Click Next,tap,,"mobile.customer.next.btn"
-9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-10. Click Close,tap,,"mobile.customer.cancel.btn"
-11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
-12. Click Continue,tap,,"mobile.customer.continue.btn"
-13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
-14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
-16. Switch To Web Session,switch_to,web,
-17. Click Customer Menu,click,,"admin.menu.customer_icon"
-18. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
-19. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
-20. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
-21. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
-22. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
-23.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
-24. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
-25. Select Male Gender,click,,"admin.customer.select_gender_male"
-26. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
-27. Wait for Toast to Hide,wait,3000,,
-28. Click Submit Button,click,,"web.global.action.submit"
-29. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
-30. Click Customer Menu,click,,"admin.menu.customer_icon"
-31. Click Customer Menu,click,,"admin.menu.customer_icon"
-32. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
-33.Wait For Customer Filter,wait,3000,
-34. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-35.Wait For Customer,wait,2000,
-36. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
-37. Load User App,switch_to,user,
-38. Reload User App Completely,reload_app,user,
-39. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-40.Click Get Started,tap,,"mobile.customer.get_started.btn" 
-41.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
-42. Click Next,tap,,"mobile.customer.next.btn"
-43. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-44. Click Close,tap,,"mobile.customer.cancel.btn"
-45. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
-46. Click Continue,tap,,"mobile.customer.continue.btn"
-47. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-48. Click Finish,tap,,"mobile.customer.finish.btn"
-49. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-50. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
-51. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
-52.Wait For Profile,wait,5000,
-53. Click Profile,tap_coordinate,558:405,COORDINATE_MODE
-54. Wait For Profile Details,wait_until_visible,,"mobile.customer.edit_account.heading"
-55.Click Back,tap,,"mobile.customer.back.btn"
-56.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
-57. Drag Page Layout Upward,swipe,up,
-58.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
-59. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
-60. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
-61. Click Manage Account,tap,,"mobile.customer.delete.btn"
-62. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
-63. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
-64. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
-65. Switch To Web Session,switch_to,web,
-66. Click Customer Menu,click,,"admin.menu.customer_icon"
-67. Click Customer DropDown,click,,"admin.menu.customer_icon"
-68. Click Delete Customer,click,,"admin.menu.customer_deleted"
-69. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-70. Wait For Delete Customer,wait_until_visible,,"admin.customer.filter_name"
-</t>
-  </si>
-  <si>
-    <t>1.Reload User App Completely,reload_app,user,
-2.Reload Driver App Completely,reload_app,driver,
-3. Load User App,switch_to,user,
-4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-5. Click Get Started,tap,,"mobile.customer.get_started.btn"
-6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
-7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
-8. Click Next,tap,,"mobile.customer.next.btn"
-9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-10. Click Close,tap,,"mobile.customer.cancel.btn"
-11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
-12. Click Continue,tap,,"mobile.customer.continue.btn"
-13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
-14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
-16. Switch To Web Session,switch_to,web,
-17. Click Customer Menu,click,,"admin.menu.customer_icon"
-18. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
-19. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
-20. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
-21. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
-22. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
-23.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
-24. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
-25. Select Male Gender,click,,"admin.customer.select_gender_male"
-26. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
-27. Wait for Toast to Hide,wait,3000,,
-28. Click Submit Button,click,,"web.global.action.submit"
-29. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
-30. Click Customer Menu,click,,"admin.menu.customer_icon"
-31. Click Customer Menu,click,,"admin.menu.customer_icon"
-32. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
-33.Wait For Customer Filter,wait,3000,
-34. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-35.Wait For Customer,wait,2000,
-36. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
-37. Load User App,switch_to,user,
-38. Reload User App Completely,reload_app,user,
-39. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-40.Click Get Started,tap,,"mobile.customer.get_started.btn" 
-41.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
-42. Click Next,tap,,"mobile.customer.next.btn"
-43. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-44. Click Close,tap,,"mobile.customer.cancel.btn"
-45. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
-46. Click Continue,tap,,"mobile.customer.continue.btn"
-47. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-48. Click Finish,tap,,"mobile.customer.finish.btn"
-49. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-50. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
-51. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
-52.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
-53. Drag Page Layout Upward,swipe,up,
-54. Click Select Language,tap,,"mobile.customer.Language.btn"
-55. Wait for Language Setting option,wait,3000,,
-56. Click Select Tamil Language,tap,,"mobile.customer.Language.Tamil.button"
-57. Click Select english Language Update,tap,,"mobile.customer.menu.Language.save_changes.btn"
-58. Wait for Language Setting option,wait,3000,,
-59. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
-60. Wait For Page Load,wait,3000,
-61. Click Select Language,tap,,"mobile.customer.Language_menu.Tamil.btn"
-62. Wait for Language Setting option,wait,3000,,
-63. Click Select hindi Language,tap,,"mobile.customer.Language.Hindi.button"
-64. Click Select Tamil Language Update,tap,,"mobile.customer.menu.Language_Tamil.save_changes.btn"
-65. Wait for Profile,wait,3000,,
-66. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
-67. Wait For Page Load,wait,3000
-68. Click Select Language,tap,,"mobile.customer.Language_menu.Hindi.btn"
-69. Wait for Language Setting option,wait,3000,,
-70. Click Select english Language,tap,,"mobile.customer.Language.English.button"
-71. Click Select hindi Language Update,tap,,"mobile.customer.menu.Language_Hindi.save_changes.btn"
-72. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
-73. Drag Page Layout Upward,swipe,up,
-74. Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
-75. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
-76. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
-77. Click Manage Account,tap,,"mobile.customer.delete.btn"
-78. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
-79. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
-80. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
-81. Switch To Web Session,switch_to,web,
-82. Click Customer Menu,click,,"admin.menu.customer_icon"
-83. Click Customer DropDown,click,,"admin.menu.customer_icon"
-84. Click Delete Customer,click,,"admin.menu.customer_deleted"
-85. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-86. Wait For Delete Customer,wait_until_visible,,"admin.customer.filter_name"</t>
   </si>
   <si>
     <t>79.Click Language menu,tap,,"mobile.driver.Language.btn"
@@ -2058,6 +1811,15 @@
     <t>TC_CA_07_test_data_cleanup</t>
   </si>
   <si>
+    <t>TC_CA_02_Driver_App_Wallet_Verification</t>
+  </si>
+  <si>
+    <t>TC_CA_03_Non_Verified_And_Deleted_Customer</t>
+  </si>
+  <si>
+    <t>TC_CA_04_Autoride_Complete_Test</t>
+  </si>
+  <si>
     <t>1.Reload User App Completely,reload_app,user,
 2.Reload Driver App Completely,reload_app,driver,
 3.Load Super Admin,switch_to,web,
@@ -2083,7 +1845,7 @@
 23.Select On,click,,"admin.subscription.common.status.option_on"
 24.Click Submit ,click,,"web.global.action.submit"
 25.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
-26.Click badge,click,,"admin.subscription.badge.icon"
+26.Click Dashboard Icon,click,,"web.global.menu.dashboard"
 27.Click Subscription Plan,click,,"admin.subscription.menu_link"
 28.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
 29.Verify Customer Subscription Plan Lists ,verify,,"admin.subscription.customer.header"
@@ -2091,9 +1853,9 @@
 31.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
 32.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
 33.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "admin.subscription.common.name.input"
-34.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
-35.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
-36.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
+34.Enter Customer Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+35.Enter Customer Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
+36.Enter Customer Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
 37.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
 38.Enter Number Of Free Rides, type,2, "admin.subscription.customer.free_rides.input"
 39.Enter Price, type,5000, "admin.subscription.common.price.input"
@@ -2159,13 +1921,255 @@
 99.Wait For Deletion,wait,2000,</t>
   </si>
   <si>
-    <t>TC_CA_02_Driver_App_Wallet_Verification</t>
-  </si>
-  <si>
-    <t>TC_CA_03_Non_Verified_And_Deleted_Customer</t>
-  </si>
-  <si>
-    <t>TC_CA_04_Autoride_Complete_Test</t>
+    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3.Load Driver App,switch_to,driver,
+4.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+5.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+6.Click Agree,tap,,"mobile.driver.agree.btn"
+7.Click Get Started,tap,,"mobile.driver.get_started.btn"
+8.Click Next,tap,,"mobile.driver.next.btn"
+9.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+10.Click Close,tap,,"mobile.driver.cancel.btn"
+11.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+12.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+13 Click Continue,tap,,"mobile.driver.continue.btn"
+14. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+15.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+16.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+17.Wait For Pageload,wait,3000,
+18.Load User App,switch_to,user,
+19.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+20.Click Get Started,tap,,"mobile.customer.get_started.btn"
+21.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+22.Click Next,tap,,"mobile.customer.next.btn"
+23.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+24.Click Close,tap,,"mobile.customer.cancel.btn"
+25.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+26.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+27. Click Continue,tap,,"mobile.customer.continue.btn"
+28. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+29. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+30. Click Finish,tap,,"mobile.customer.finish.btn"
+31. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+32. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+33. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+34. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+35. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+36. Select Destination,tap_coordinate,545:1299,
+37. Click Confirm,tap,,"mobile.customer.confirm.btn"
+38. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+39. Ride Now,tap,,"mobile.customer.ride_now.btn"
+40. Load Driver App,switch_to,driver,
+41.Wait for Accept,wait_until_visible,,"mobie.driver.auto_ride_accept.button"
+42.Click  Accept Ride,tap,,"mobie.driver.auto_ride_accept.button"
+43.Fetch Ride Code from DB,fetch_db_value,ride_otp,"SELECT otp FROM we1.user_ride_booking ORDER BY id DESC LIMIT 1"
+44.Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
+45.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+46.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+47.Ride Arrived,tap,,"mobile.driver.arrived.btn"
+48.Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+49.Yes Arrived,tap,,"mobile.driver.yes.btn"
+50.Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
+51.Start Ride,tap,,"mobile.driver.start_ride.btn"
+52.wait for Otp,wait_until_visible,,"mobile.driver.otp_view.input"
+53.Enter OTP,type,{ride_otp},"mobile.driver.otp_view.input"
+54.Wait for Start Button,wait_until_visible,,"mobile.driver.start.btn"
+55.Start Ride Button,tap,,"mobile.driver.start.btn"
+56.Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
+57.Complete Ride,tap,,"mobile.driver.complete_ride.btn"
+58.Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
+59.Collect Payment,tap,,"mobile.driver.collect_payment.btn"
+60.Load User App,switch_to,user,
+61.Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+62.Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
+63. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+64. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
+65. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
+66. Give Review,tap,,"mobile.customer.give_review.btn"
+67. Give Rating,tap_coordinate,348:1619,
+68. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
+69.Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
+70.Trip Finished,tap,,"mobile.customer.done.btn"
+71. Load Driver App,switch_to,driver,
+72.Wait  For Proceed,wait_until_visible,,"mobile.driver.payment.proceed_btn"
+73.Click For Proceed,tap,,"mobile.driver.payment.proceed_btn"
+74. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+75. Confirm Payment,tap,,"mobile.driver.yes.btn"
+76.Wait For Give Review Button,wait_until_visible,,"mobile.driver.give_review.btn"
+77.Click Give Review Button,tap,,"mobile.driver.give_review.btn"
+78.Wait For Rating,wait,2000,
+79. Give Rating,tap_coordinate,348:1545,
+80. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
+81.Wait for Complete Button,wait_until_visible,,"mobile.driver.complete.btn"
+82.Click Complete Button,tap,,"mobile.driver.complete.btn"
+83.Wait For  ride complete submit button,wait_until_visible,,"mobile.driver.ride_complete_submit.btn"
+84.Click Ride Complete Submit Button,tap,,"mobile.driver.ride_complete_submit.btn"
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3. Load User App,switch_to,user,
+4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+5. Click Get Started,tap,,"mobile.customer.get_started.btn"
+6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
+7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
+8. Click Next,tap,,"mobile.customer.next.btn"
+9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap,,"mobile.customer.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
+12. Click Continue,tap,,"mobile.customer.continue.btn"
+13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
+14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
+16. Switch To Web Session,switch_to,web,
+17. Click Customer Menu,click,,"admin.menu.customer_icon"
+18. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
+19. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
+20. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
+21. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
+22. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+23.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
+24. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
+25. Select Male Gender,click,,"admin.customer.select_gender_male"
+26. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+27. Wait for Toast to Hide,wait,3000,,
+28. Click Submit Button,click,,"web.global.action.submit"
+29. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
+30. Click Customer Menu,click,,"admin.menu.customer_icon"
+31. Click Customer Menu,click,,"admin.menu.customer_icon"
+32. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
+33.Wait For Customer Filter,wait,3000,
+34. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+35.Wait For Customer,wait,2000,
+36. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
+37. Load User App,switch_to,user,
+38. Reload User App Completely,reload_app,user,
+39. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+40.Click Get Started,tap,,"mobile.customer.get_started.btn" 
+41.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
+42. Click Next,tap,,"mobile.customer.next.btn"
+43. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+44. Click Close,tap,,"mobile.customer.cancel.btn"
+45. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+46. Click Continue,tap,,"mobile.customer.continue.btn"
+47. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+48. Click Finish,tap,,"mobile.customer.finish.btn"
+49. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+50. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
+51. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
+52.Wait For Profile,wait,5000,
+53. Click Profile,tap_coordinate,558:405,COORDINATE_MODE
+54. Wait For Profile Details,wait_until_visible,,"mobile.customer.edit_account.heading"
+55.Click Back,tap,,"mobile.customer.back.btn"
+56.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+57. Drag Page Layout Upward,swipe,up,
+58.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
+59. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+60. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
+61. Click Manage Account,tap,,"mobile.customer.delete.btn"
+62. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
+63. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
+64. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
+65. Switch To Web Session,switch_to,web,
+66. Click Customer Menu,click,,"admin.menu.customer_icon"
+67. Click Customer DropDown,click,,"admin.menu.customer_icon"
+68. Click Delete Customer,click,,"admin.menu.customer_deleted"
+69.Wait For Delted Customer,wait,3000, 
+69. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+70.Wait For Delted Customer,wait,3000, 
+</t>
+  </si>
+  <si>
+    <t>1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3. Load User App,switch_to,user,
+4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+5. Click Get Started,tap,,"mobile.customer.get_started.btn"
+6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
+7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
+8. Click Next,tap,,"mobile.customer.next.btn"
+9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap,,"mobile.customer.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
+12. Click Continue,tap,,"mobile.customer.continue.btn"
+13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
+14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
+16. Switch To Web Session,switch_to,web,
+17.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+18. Click Customer Menu,click,,"admin.menu.customer_icon"
+19. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
+20. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
+21. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
+22. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
+23. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+24.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
+25. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
+26. Select Male Gender,click,,"admin.customer.select_gender_male"
+27. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+28. Wait for Toast to Hide,wait,3000,,
+29. Click Submit Button,click,,"web.global.action.submit"
+30. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
+31. Click Customer Menu,click,,"admin.menu.customer_icon"
+32. Click Customer Menu,click,,"admin.menu.customer_icon"
+33. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
+34.Wait For Customer Filter,wait,3000,
+35. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+36.Wait For Customer,wait,2000,
+37. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
+38. Load User App,switch_to,user,
+39. Reload User App Completely,reload_app,user,
+40. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+41.Click Get Started,tap,,"mobile.customer.get_started.btn" 
+42.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
+43. Click Next,tap,,"mobile.customer.next.btn"
+44. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+45. Click Close,tap,,"mobile.customer.cancel.btn"
+46. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+47. Click Continue,tap,,"mobile.customer.continue.btn"
+48. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+49. Click Finish,tap,,"mobile.customer.finish.btn"
+50. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+51. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
+52. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
+53.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+54. Drag Page Layout Upward,swipe,up,
+55. Click Select Language,tap,,"mobile.customer.Language.btn"
+56. Wait for Language Setting option,wait,3000,,
+57. Click Select Tamil Language,tap,,"mobile.customer.Language.Tamil.button"
+58. Click Select english Language Update,tap,,"mobile.customer.menu.Language.save_changes.btn"
+59. Wait for Language Setting option,wait,3000,,
+60. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
+61. Wait For Page Load,wait,3000,
+62. Click Select Language,tap,,"mobile.customer.Language_menu.Tamil.btn"
+63. Wait for Language Setting option,wait,3000,,
+64. Click Select hindi Language,tap,,"mobile.customer.Language.Hindi.button"
+65. Click Select Tamil Language Update,tap,,"mobile.customer.menu.Language_Tamil.save_changes.btn"
+66. Wait for Profile,wait,3000,,
+67. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
+68. Wait For Page Load,wait,3000
+69. Click Select Language,tap,,"mobile.customer.Language_menu.Hindi.btn"
+70. Wait for Language Setting option,wait,3000,,
+71. Click Select english Language,tap,,"mobile.customer.Language.English.button"
+72. Click Select hindi Language Update,tap,,"mobile.customer.menu.Language_Hindi.save_changes.btn"
+73. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
+74. Drag Page Layout Upward,swipe,up,
+75. Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
+76. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+77. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
+78. Click Manage Account,tap,,"mobile.customer.delete.btn"
+79. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
+80. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
+81. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
+82. Switch To Web Session,switch_to,web,
+83. Click Customer Menu,click,,"admin.menu.customer_icon"
+84. Click Customer DropDown,click,,"admin.menu.customer_icon"
+85. Click Delete Customer,click,,"admin.menu.customer_deleted"
+86.Wait For Delete Cusotmer,wait,3000,
+86. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+87. Wait For Delete Cusotmer,wait,3000,</t>
   </si>
 </sst>
 </file>
@@ -2658,22 +2662,22 @@
         <v>44</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="H2" s="2"/>
     </row>
@@ -2736,13 +2740,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>9</v>
@@ -2811,13 +2815,13 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>34</v>
@@ -2889,13 +2893,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>37</v>
@@ -2964,13 +2968,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>13</v>
@@ -3040,10 +3044,10 @@
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
@@ -3127,13 +3131,13 @@
         <v>49</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>48</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>
@@ -3208,16 +3212,16 @@
         <v>35</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>
@@ -3247,7 +3251,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1895CC0E-D326-49C3-B5DA-E3C80EEAE5A9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A659562-16FE-472A-9348-C2754F8B87F9}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3295,13 +3299,13 @@
         <v>43</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>
@@ -3376,16 +3380,16 @@
         <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>47</v>

</xml_diff>

<commit_message>
89th Commit: Set Date Keyword Implemted
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F20D60A-A21C-4341-8B9F-43BDF7D103B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C632D79D-468E-42B6-9882-3EAA534403F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -18,12 +18,14 @@
     <sheet name="HybridUnApprovedAutoDriver" sheetId="46" r:id="rId3"/>
     <sheet name="HybridApprovedAutoDriver" sheetId="38" r:id="rId4"/>
     <sheet name="HybridSubscriptionPlanTest" sheetId="40" r:id="rId5"/>
-    <sheet name="DriverAppWalletVerificaton" sheetId="48" r:id="rId6"/>
-    <sheet name="NonVerifiedAndDeletedCustomer" sheetId="50" r:id="rId7"/>
-    <sheet name="AutoRideCompleteTest" sheetId="54" r:id="rId8"/>
-    <sheet name="CustomerLanguageCheck" sheetId="52" r:id="rId9"/>
-    <sheet name="DriverLanguageCheck" sheetId="53" r:id="rId10"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId11"/>
+    <sheet name="DriverAppWalletVerification" sheetId="48" r:id="rId6"/>
+    <sheet name="CustomerAppWalletCheck" sheetId="55" r:id="rId7"/>
+    <sheet name="NonVerifiedAndDeletedCustomer" sheetId="50" r:id="rId8"/>
+    <sheet name="CustomerAppEmergencyNumber" sheetId="56" r:id="rId9"/>
+    <sheet name="CustomerLanguageCheck" sheetId="52" r:id="rId10"/>
+    <sheet name="DriverLanguageCheck" sheetId="53" r:id="rId11"/>
+    <sheet name="AutoRideCompleteTest" sheetId="54" r:id="rId12"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId13"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="97">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -872,118 +874,6 @@
 </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The UserDriverWebIntialilzer,HybridAddCustomer and  HybridUnApprovedAutoDriver test sheets must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RunSheet:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>UserDriverWebIntialilzer</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
-    </r>
-  </si>
-  <si>
     <t>This end-to-end hybrid regression test verifies the runtime visibility and functionality of the mobile Driver Wallet module based on configurations managed within the Super Admin Web Portal. The execution workflow first activates the wallet feature via the admin portal's site settings, logs into the driver application, and executes a full simulated wallet top-up transaction using Net Banking to confirm operational stability. It then reverts to the web panel to toggle the wallet status to "OFF," restarts the mobile application context to clear active sessions, re-authenticates the driver, and explicitly asserts that the Wallet option is completely absent from the side menu hierarchy.</t>
   </si>
   <si>
@@ -1115,119 +1005,6 @@
   </si>
   <si>
     <t>Orginal Test Steps Old Apk</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Data Dependency:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The UserDriverWebIntialilzer, HybridAddCustomer and HybridApprovedAutoDriver test sheets must always be executed prior to running this  test
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>RunSheet:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">UserDriverWebIntialilzer
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-System State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Access Rights:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> A valid Super Admin account exists in the database.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Data Availability:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
-    </r>
   </si>
   <si>
     <t>1.Reload User App Completely,reload_app,user,
@@ -1639,9 +1416,6 @@
     <t>SA_TS_07</t>
   </si>
   <si>
-    <t>Non Verified Customer</t>
-  </si>
-  <si>
     <t>Customer Language Check</t>
   </si>
   <si>
@@ -1653,122 +1427,6 @@
 92. Click Language menu,tap,,"mobile.driver.Language_menu.Hindi.btn"</t>
   </si>
   <si>
-    <t>1. Reload User App Completely,reload_app,user,
-2. Reload Driver App Completely,reload_app,driver,
-3.  Switch To Web Session,switch_to,web,
-4. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-5. Click drivers menu,click,,"admin.drivers.menu.icon"
-6. Click Add Driver menu,click,,"admin.drivers.add_menu.link"
-7. Verify Add Driver,verify,,"admin.drivers.add_page.header"
-8. Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
-9. Select Auto Ride Option,click,,"admin.drivers.service_dropdown.auto_ride"
-10. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "admin.drivers.fullname.input"
-11. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "admin.drivers.email.input"
-12. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "admin.drivers.phone.input"
-13. Click Whatspp, click, , "admin.drivers.whatsapp.checkbox"
-14. Enter Whatspp Number, type, {autoPhone}, "admin.drivers.whatsapp_phone.input"
-15. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "admin.drivers.profile_image.file"
-16. Select Source,click,,"admin.drivers.source_dropdown.select"
-17. Select Instagram,click,,"admin.drivers.instagram_option.span"
-18. Select Male Gender, click, , "admin.drivers.male_gender.div"
-19. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
-20. Select  Auto Option,click,,"admin.drivers.vehicle_option.pinkauto"
-21. Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
-22. Enter Plate No, type, KL-01-AB-1234, "admin.drivers.plateno.input"
-23. Enter Model Name, type, petrol, "admin.drivers.modelname.input"
-24. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "admin.drivers.vehicle_image.file"
-25. Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
-26. Enter Bank Location, type, Chennai, "admin.drivers.banklocation.input"
-27. Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
-28. Enter Account Holder Name, type,{autoName}, "admin.drivers.accountholder.input"
-29. Enter Payment Email Address, type, {autoEmail}, "admin.drivers.paymentemail.input"
-30. Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
-31. Click Submit, click, , "web.global.action.submit"
-32. Verify Driver Added, verify, , "web.global.toast.success"
-33. Click drivers menu,click,,"admin.drivers.menu.icon"
-34. Click drivers menu,click,,"admin.drivers.menu.icon"
-35. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
-36. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
-37. Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
-38. Click Doc Icon,click,,"admin.drivers.docs.icon"
-39. Driver Required Documents,verify,,"admin.drivers.required_docs.header"
-40. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
-41. Add Driving License,click,,"admin.drivers.docs.edit_icon"
-42. Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "admin.drivers.profile_image.file"
-43. Enter Expiry Date,type,12-12-2026,"admin.drivers.doc_expiry.input"
-44. Click Submit, click, , "web.global.action.submit"
-45. Verify Updated Succesfully, verify, , "web.global.toast.updated"
-46. Click Approve Driver,click,,"admin.drivers.docs.approval"
-47. Verify Updated Succesfully, verify, , "web.global.toast.updated"
-48. Click Dashboard,click,,"web.global.menu.dashboard"
-49. Click drivers menu,click,,"admin.drivers.menu.icon"
-50. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
-51. Approved Drivers List,verify,,"admin.drivers.approved_page.header"
-52. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
-53. Wait For Get_Started,wait_until_visible,,"admin.drivers.name_filter.input"
-54. Load Driver App,switch_to,driver,
-55. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-56. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-57. Click Agree,tap,,"mobile.driver.agree.btn"
-58. Click Get Started,tap,,"mobile.driver.get_started.btn"
-59. Click Next,tap,,"mobile.driver.next.btn"
-60. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-61. Click Close,tap,,"mobile.driver.cancel.btn"
-62. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
-63. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-64. Click Continue,tap,,"mobile.driver.continue.btn"
-65. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-66. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-67. Wait for Toast to Hide,wait,3000,,
-68. Click Select All Agree,tap,,"mobile.driver.independent_contractor.checkbox_Select_All"
-69. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
-70. Click Agree,tap,,"mobile.driver.agree_continue.btn"
-71. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
-72. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-73. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-74.Wait For Hamburger Menu,wait,3000
-75. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-76.Wait For Driver Profile Load,wait,3000,
-77. Drag Page Layout Upward,swipe,up,
-78.Wait For Language Menu,wait,3000,
-79. Click Language menu,tap_coordinate,394:1631,COORDINATE_MODE
-80. Wait for Language Setting option,wait,3000,,
-81. Click Select Tamil Language,tap,,"mobile.driver.Language.Tamil.button"
-82. Click Select Tamil Language Update,tap,,"mobile.driver.menu.Language.save_changes.btn"
-83. Wait for Language Setting option,wait,3000,,
-84. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-85. Drag Page Layout Upward,swipe,up,
-86.Wait For Page Load,wait,3000,
-87. Click Language menu,tap_coordinate,394:1631,COORDINATE_MODE
-88. Wait for Language Setting option,wait,3000,,
-89. Click Select Hindi Language,tap,,"mobile.driver.Language.Hindi.button"
-90. Click Select Hindi Language Update,tap,,"mobile.driver.menu.Language_Tamil.save_changes.btn"
-91. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-92. Drag Page Layout Upward,swipe,up,
-93.Wait For Page Load,wait,3000,
-94. Click Language menu,tap_coordinate,394:1631,COORDINATE_MODE
-95. Wait for Language Setting option,wait,3000,,
-96. Click Select English Language,tap,,"mobile.driver.Language.English.button"
-97. Click Select English Language Update,tap,,"mobile.driver.menu.Language_Hindi.save_changes.btn"
-98. Wait for Language Setting option,wait,3000,,
-99. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-100. Drag Page Layout Upward,swipe,up,
-101. Wait for Manage Account Loading,wait,3000,,
-102. Click Manage Account,tap,,"mobile.driver.manage_account.btn"
-103. Click Delete Account,tap,,"mobile.driver.delete.btn"
-104. Click Delete Account Sure,tap,,"mobile.driver.delete_sure.btn"
-105. Switch To Web Session,switch_to,web,
-106. Wait for Menu,wait_until_visible,,"admin.drivers.menu.icon"
-107. Click Driver Menu,click,,"admin.drivers.menu.icon"
-108. Click Driver DropDown,click,,"admin.drivers.menu.icon"
-109. Wait for Agree,wait_until_visible,,"Global.menu.driver_deleted"
-110. Click Delete Driver,click,,"Global.menu.driver_deleted"
-111. Enter Driver Vehicele,type,Pink Auto,"Global.menu.Delete_Driver.Vehicle_Type_Filter" 
-112. scroll grid,tab,4,,”Global.menu.Delete_Driver.Contact_Type_Filter"
-113. Enter Driver Name,type,{autoName},"Global.menu.Delete_Driver.Contact_Type_Filter"
-114. Wait For Delete Driver,wait_until_visible,,"Global.menu.Delete_Driver.Contact_Type_Filter"</t>
-  </si>
-  <si>
     <t>SA_TS_0A</t>
   </si>
   <si>
@@ -1781,294 +1439,498 @@
     <t>TC_CA_0B_Hybrid_Unapproved_Auto_Driver</t>
   </si>
   <si>
-    <t>SA_TS_0D</t>
-  </si>
-  <si>
-    <t>TC_CA_0D_Hybrid_Approved_Auto_Driver</t>
-  </si>
-  <si>
     <t>TC_CA_01_Hybrid_Subscription_Plan_Test</t>
   </si>
   <si>
-    <t>Subscriptin Plan Complete Test</t>
-  </si>
-  <si>
     <t>This comprehensive, cross-platform regression test suite validates the entire lifecycle of a customer account by seamlessly orchestrating actions between native mobile applications and the centralized web administration portal. The test sequence begins by initializing a fresh mobile session using the reload_app utility, executing a new user registration flow via dynamic device permissions, randomized phone generation, and OTP simulation. The execution then seamlessly switches context to the web portal to locate the newly created profile under the Non-Verified Customers matrix, populates missing metadata (including automated profile image uploads and randomized alpha naming strings), and submits the profile to trigger status escalation. After confirming the user's migration into the Verified Customers data grid, the execution switches back to the mobile application instance to verify verified account access. Finally, the test validates data-compliance workflows by triggering a native Delete Account chain from the mobile device settings and cross-verifying that the user profile is immediately and correctly relocated to the web admin’s Deleted Customers repository.</t>
   </si>
   <si>
-    <t>TC_CA_05_Customer_Language_Check</t>
-  </si>
-  <si>
     <t>This comprehensive, cross-platform regression test suite validates the customer onboarding lifecycle, profile verification, and dynamic UI localization capabilities across both native mobile environments and the centralized web admin portal. The script begins by orchestrating an initial mobile registration and OTP verification sequence, shifts context to the web portal to escalate the profile from the Non-Verified Customers grid to the Verified Customers list via metadata injection and profile image uploads, and logs back into the mobile app to verify access. It then comprehensively audits the localization subsystem by performing sequential runtime dialect switches—transitioning the interface dynamically from English to Tamil, Tamil to Hindi, and back to English—while verifying that language save triggers update the UI element bounds properly without memory leaks. Finally, the suite executes a clean teardown flow by triggering a native Delete Account action from the mobile settings drawer and cross-verifying that the profile records are accurately reassigned to the web admin's Deleted Customers master repository.</t>
   </si>
   <si>
-    <t>TC_CA_06_Driver_Language_Check</t>
-  </si>
-  <si>
     <t>This end-to-end, cross-platform regression test suite orchestrates a complex testing lifecycle for driver management by coordinating operations between the central web administration portal and native mobile driver application runtimes. The execution flow begins by initializing clean device environments using the reload_app keyword and shifts context to the web portal to register a new driver profile with comprehensive metadata mapping—including automated profile picture uploads, customized vehicle specifications ("Pink Auto"), and corporate banking infrastructure parameters. The test then executes a multi-tiered regulatory validation pipeline by locating the profile in the Pending Documents grid, uploading a simulated driving license file with an active expiry date, and escalating the profile to the official Approved Drivers registry. Transitioning into the native mobile engine environment, the suite authenticates the newly approved driver using dynamic OTP routing, processes specialized compliance checkboxes, and thoroughly audits the application's localization subsystem by executing dynamic runtime language shifts—transitioning the interface seamlessly from English to Tamil, Tamil to Hindi, and back to English. Finally, the suite tests legal compliance and lifecycle termination rules by triggering a native Delete Account flow from the driver app interface and verifying that the record instantly relocates to the web admin's Deleted Drivers repository under localized filtering conditions.</t>
   </si>
   <si>
-    <t>TC_CA_07_test_data_cleanup</t>
-  </si>
-  <si>
     <t>TC_CA_02_Driver_App_Wallet_Verification</t>
   </si>
   <si>
-    <t>TC_CA_03_Non_Verified_And_Deleted_Customer</t>
-  </si>
-  <si>
-    <t>TC_CA_04_Autoride_Complete_Test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
-2.Reload Driver App Completely,reload_app,driver,
-3.Load Driver App,switch_to,driver,
-4.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-5.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-6.Click Agree,tap,,"mobile.driver.agree.btn"
-7.Click Get Started,tap,,"mobile.driver.get_started.btn"
-8.Click Next,tap,,"mobile.driver.next.btn"
-9.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-10.Click Close,tap,,"mobile.driver.cancel.btn"
-11.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
-12.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-13 Click Continue,tap,,"mobile.driver.continue.btn"
-14. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-15.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-16.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-17.Wait For Pageload,wait,3000,
-18.Load User App,switch_to,user,
-19.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-20.Click Get Started,tap,,"mobile.customer.get_started.btn"
-21.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-22.Click Next,tap,,"mobile.customer.next.btn"
-23.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-24.Click Close,tap,,"mobile.customer.cancel.btn"
-25.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
-26.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-27. Click Continue,tap,,"mobile.customer.continue.btn"
-28. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-29. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
-30. Click Finish,tap,,"mobile.customer.finish.btn"
-31. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-32. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
-33. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
-34. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
-35. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
-36. Select Destination,tap_coordinate,545:1299,
-37. Click Confirm,tap,,"mobile.customer.confirm.btn"
-38. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
-39. Ride Now,tap,,"mobile.customer.ride_now.btn"
-40. Load Driver App,switch_to,driver,
-41.Wait for Accept,wait_until_visible,,"mobie.driver.auto_ride_accept.button"
-42.Click  Accept Ride,tap,,"mobie.driver.auto_ride_accept.button"
-43.Fetch Ride Code from DB,fetch_db_value,ride_otp,"SELECT otp FROM we1.user_ride_booking ORDER BY id DESC LIMIT 1"
-44.Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
-45.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
-46.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
-47.Ride Arrived,tap,,"mobile.driver.arrived.btn"
-48.Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
-49.Yes Arrived,tap,,"mobile.driver.yes.btn"
-50.Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
-51.Start Ride,tap,,"mobile.driver.start_ride.btn"
-52.wait for Otp,wait_until_visible,,"mobile.driver.otp_view.input"
-53.Enter OTP,type,{ride_otp},"mobile.driver.otp_view.input"
-54.Wait for Start Button,wait_until_visible,,"mobile.driver.start.btn"
-55.Start Ride Button,tap,,"mobile.driver.start.btn"
-56.Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
-57.Complete Ride,tap,,"mobile.driver.complete_ride.btn"
-58.Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
-59.Collect Payment,tap,,"mobile.driver.collect_payment.btn"
-60.Load User App,switch_to,user,
-61.Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
-62.Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
-63. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
-64. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
-65. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
-66. Give Review,tap,,"mobile.customer.give_review.btn"
-67. Give Rating,tap_coordinate,348:1619,
-68. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
-69.Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
-70.Trip Finished,tap,,"mobile.customer.done.btn"
-71. Load Driver App,switch_to,driver,
-72.Wait  For Proceed,wait_until_visible,,"mobile.driver.payment.proceed_btn"
-73.Click For Proceed,tap,,"mobile.driver.payment.proceed_btn"
-74. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
-75. Confirm Payment,tap,,"mobile.driver.yes.btn"
-76.Wait For Give Review Button,wait_until_visible,,"mobile.driver.give_review.btn"
-77.Click Give Review Button,tap,,"mobile.driver.give_review.btn"
-78.Wait For Rating,wait,2000,
-79. Give Rating,tap_coordinate,348:1545,
-80. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
-81.Wait for Complete Button,wait_until_visible,,"mobile.driver.complete.btn"
-82.Click Complete Button,tap,,"mobile.driver.complete.btn"
-83.Wait For  ride complete submit button,wait_until_visible,,"mobile.driver.ride_complete_submit.btn"
-84.Click Ride Complete Submit Button,tap,,"mobile.driver.ride_complete_submit.btn"
+    <t>Customer App Wallet Check</t>
+  </si>
+  <si>
+    <t>TC_CA_03_Customer_App_Wallet_Check</t>
+  </si>
+  <si>
+    <t>This end-to-end hybrid regression test verifies the runtime visibility and functionality of the mobile Customer Wallet module based on configurations managed within the Super Admin Web Portal. The execution workflow first activates the wallet feature via the admin portal's site settings, logs into the customer application, and executes a full simulated wallet top-up transaction using Net Banking to confirm operational stability. It then reverts to the web panel to toggle the wallet status to "OFF," restarts the mobile application context to clear active sessions, re-authenticates the customer, and explicitly asserts that the Wallet option is completely absent from the side menu hierarchy.</t>
+  </si>
+  <si>
+    <t>SA_TS_0C</t>
+  </si>
+  <si>
+    <t>TC_CA_0C_Hybrid_Approved_Auto_Driver</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The UserDriverWebIntialilzer  sheet must always be executed prior to running this  test
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
-2.Reload Driver App Completely,reload_app,driver,
-3. Load User App,switch_to,user,
-4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-5. Click Get Started,tap,,"mobile.customer.get_started.btn"
-6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
-7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
-8. Click Next,tap,,"mobile.customer.next.btn"
-9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-10. Click Close,tap,,"mobile.customer.cancel.btn"
-11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
-12. Click Continue,tap,,"mobile.customer.continue.btn"
-13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
-14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
-16. Switch To Web Session,switch_to,web,
-17. Click Customer Menu,click,,"admin.menu.customer_icon"
-18. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
-19. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
-20. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
-21. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
-22. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
-23.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
-24. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
-25. Select Male Gender,click,,"admin.customer.select_gender_male"
-26. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
-27. Wait for Toast to Hide,wait,3000,,
-28. Click Submit Button,click,,"web.global.action.submit"
-29. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
-30. Click Customer Menu,click,,"admin.menu.customer_icon"
-31. Click Customer Menu,click,,"admin.menu.customer_icon"
-32. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
-33.Wait For Customer Filter,wait,3000,
-34. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-35.Wait For Customer,wait,2000,
-36. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
-37. Load User App,switch_to,user,
-38. Reload User App Completely,reload_app,user,
-39. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-40.Click Get Started,tap,,"mobile.customer.get_started.btn" 
-41.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
-42. Click Next,tap,,"mobile.customer.next.btn"
-43. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-44. Click Close,tap,,"mobile.customer.cancel.btn"
-45. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
-46. Click Continue,tap,,"mobile.customer.continue.btn"
-47. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-48. Click Finish,tap,,"mobile.customer.finish.btn"
-49. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-50. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
-51. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
-52.Wait For Profile,wait,5000,
-53. Click Profile,tap_coordinate,558:405,COORDINATE_MODE
-54. Wait For Profile Details,wait_until_visible,,"mobile.customer.edit_account.heading"
-55.Click Back,tap,,"mobile.customer.back.btn"
-56.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
-57. Drag Page Layout Upward,swipe,up,
-58.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
-59. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
-60. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
-61. Click Manage Account,tap,,"mobile.customer.delete.btn"
-62. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
-63. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
-64. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
-65. Switch To Web Session,switch_to,web,
-66. Click Customer Menu,click,,"admin.menu.customer_icon"
-67. Click Customer DropDown,click,,"admin.menu.customer_icon"
-68. Click Delete Customer,click,,"admin.menu.customer_deleted"
-69.Wait For Delted Customer,wait,3000, 
-69. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-70.Wait For Delted Customer,wait,3000, 
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">UserDriverWebIntialilzer
 </t>
-  </si>
-  <si>
-    <t>1.Reload User App Completely,reload_app,user,
-2.Reload Driver App Completely,reload_app,driver,
-3. Load User App,switch_to,user,
-4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-5. Click Get Started,tap,,"mobile.customer.get_started.btn"
-6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
-7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
-8. Click Next,tap,,"mobile.customer.next.btn"
-9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-10. Click Close,tap,,"mobile.customer.cancel.btn"
-11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
-12. Click Continue,tap,,"mobile.customer.continue.btn"
-13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
-14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
-16. Switch To Web Session,switch_to,web,
-17.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-18. Click Customer Menu,click,,"admin.menu.customer_icon"
-19. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
-20. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
-21. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
-22. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
-23. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
-24.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
-25. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
-26. Select Male Gender,click,,"admin.customer.select_gender_male"
-27. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
-28. Wait for Toast to Hide,wait,3000,,
-29. Click Submit Button,click,,"web.global.action.submit"
-30. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
-31. Click Customer Menu,click,,"admin.menu.customer_icon"
-32. Click Customer Menu,click,,"admin.menu.customer_icon"
-33. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
-34.Wait For Customer Filter,wait,3000,
-35. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-36.Wait For Customer,wait,2000,
-37. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
-38. Load User App,switch_to,user,
-39. Reload User App Completely,reload_app,user,
-40. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
-41.Click Get Started,tap,,"mobile.customer.get_started.btn" 
-42.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
-43. Click Next,tap,,"mobile.customer.next.btn"
-44. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-45. Click Close,tap,,"mobile.customer.cancel.btn"
-46. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
-47. Click Continue,tap,,"mobile.customer.continue.btn"
-48. Enter OTP,type,123456,"mobile.customer.edit_text.input"
-49. Click Finish,tap,,"mobile.customer.finish.btn"
-50. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-51. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
-52. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
-53.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
-54. Drag Page Layout Upward,swipe,up,
-55. Click Select Language,tap,,"mobile.customer.Language.btn"
-56. Wait for Language Setting option,wait,3000,,
-57. Click Select Tamil Language,tap,,"mobile.customer.Language.Tamil.button"
-58. Click Select english Language Update,tap,,"mobile.customer.menu.Language.save_changes.btn"
-59. Wait for Language Setting option,wait,3000,,
-60. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
-61. Wait For Page Load,wait,3000,
-62. Click Select Language,tap,,"mobile.customer.Language_menu.Tamil.btn"
-63. Wait for Language Setting option,wait,3000,,
-64. Click Select hindi Language,tap,,"mobile.customer.Language.Hindi.button"
-65. Click Select Tamil Language Update,tap,,"mobile.customer.menu.Language_Tamil.save_changes.btn"
-66. Wait for Profile,wait,3000,,
-67. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
-68. Wait For Page Load,wait,3000
-69. Click Select Language,tap,,"mobile.customer.Language_menu.Hindi.btn"
-70. Wait for Language Setting option,wait,3000,,
-71. Click Select english Language,tap,,"mobile.customer.Language.English.button"
-72. Click Select hindi Language Update,tap,,"mobile.customer.menu.Language_Hindi.save_changes.btn"
-73. Click Profile_Menu,tap_coordinate,979:2106,COORDINATE_MODE
-74. Drag Page Layout Upward,swipe,up,
-75. Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
-76. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
-77. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
-78. Click Manage Account,tap,,"mobile.customer.delete.btn"
-79. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
-80. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
-81. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
-82. Switch To Web Session,switch_to,web,
-83. Click Customer Menu,click,,"admin.menu.customer_icon"
-84. Click Customer DropDown,click,,"admin.menu.customer_icon"
-85. Click Delete Customer,click,,"admin.menu.customer_deleted"
-86.Wait For Delete Cusotmer,wait,3000,
-86. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-87. Wait For Delete Cusotmer,wait,3000,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The UserDriverWebIntialilzer test sheet must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>UserDriverWebIntialilzer</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Data Dependency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The UserDriverWebIntialilzer sheet must always be executed prior to running this lifecycle test. This pre-execution sequence ensures that an active, authenticated Super Admin web session is established and that a valid, unassigned driver identity exists within the system pool. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>RunSheet:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>UserDriverWebIntialilzer</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+System State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Before running the test suite, ensure the target environments are active and properly connected by verifying that the WE1 Web Application is live at https://dev.we1.co/#/login (matched to base.url in config.properties), the Appium Server is up and listening on port 4723, and the necessary Android Emulators (e.g., for User, Driver, or Store modules) are fully booted via Android Studio with their USB debugging configurations ready to receive automated sessions.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Access Rights:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> A valid Super Admin account exists in the database.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Data Availability:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> All essential test configurations and structural variables are completely consolidated within the config.properties file. This includes the Web Admin and dashboard URLs, centralized Super Admin login credentials, and the necessary database connection strings (jdbc:postgresql) for backend verification and cleanup routines. For the mobile infrastructure, the local execution data is fully detailed with precise Appium server links, specific Android Emulator device IDs (emulator-5554 and emulator-5556), verified application package/activity details, and secure, absolute local directory paths for the User and Driver APKs. This centralizes your test-run parameters, ensuring the automation engine can dynamically fetch data inputs, framework timeouts, and target Excel regression sheets (we1_hybrid_regression.xlsx) natively before runtime.</t>
+    </r>
+  </si>
+  <si>
+    <t>Non Verified And Delete Customer</t>
+  </si>
+  <si>
+    <t>TC_CA_04_Non_Verified_And_Deleted_Customer</t>
+  </si>
+  <si>
+    <t>SA_TS_08</t>
+  </si>
+  <si>
+    <t>1.Load User App,switch_to,user,
+2.Reload User App Completely,reload_app,user,
+3.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+4. Load Super Admin,switch_to,web,
+5.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
+6. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+7. Click Settings Menu,click,,"web.global.menu.settings"
+8. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+9. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+10.Wait For On,wait,2000,
+11. Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+12. Click Submit Button,click,,"web.global.action.submit"
+13. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+14. Load User App,switch_to,user,
+15.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+16.Click Get Started,tap,,"mobile.customer.get_started.btn"
+17.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+18.Click Next,tap,,"mobile.customer.next.btn"
+19.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+20.Click Close,tap,,"mobile.customer.cancel.btn"
+21.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+22.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+23.Click Continue,tap,,"mobile.customer.continue.btn"
+24.Enter OTP,type,123456,"mobile.customer.edit_text.input"
+25.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+26.Click Finish,tap,,"mobile.customer.finish.btn"
+27.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+28. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
+29. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
+30.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+31.wait for Wallet,wait_until_visible,"mobile.customer.wallet.btn"
+32.Click Wallet,tap,,"mobile.customer.wallet.btn"
+33.Wait For Topup,wait_until_visible,,"mobile.customer.top_up.btn"
+34.Click Topup,tap,,"mobile.customer.top_up.btn"
+35.Wait For Topup Sum,wait_until_visible,,"mobile.customer.top_up.btn"
+36.Click Hundered,tap,,"mobile.customer.top_up_amount.hundred"
+37.Click Proceed,tap,,"mobile.customer.top_up.proceed"
+38.Wait For Contact No,wait_until_visible,,"mobile.customer.top_up.contact_no_box"
+39.Enter Customer Mobile,type,regression.customer.phone,"mobile.customer.top_up.contact_no_box"
+40.Wait For Payment Options,wait_until_visible,,"mobile.customer.top_up.payment_option"
+41.Wait For Net Banking,wait,5000,
+42.Click Net Banking,tap,,"mobile.customer.top_up.net_banking"
+43.Wait For Bob,wait,5000,
+44.Click Bob,tap_coordinate,288:1325,
+45.Wait For Success,wait_until_visible,,"mobile.customer.top_up.succes_popup"
+46.Click Success,tap,,"mobile.customer.top_up.succes_popup"
+47.Wait For Wallet  Back,wait_until_visible,,"mobile.customer.wallet.btn"
+48.Click Back,tap,,"mobile.customer.back.btn"
+49.Drag Page Layout Upward,swipe,up,
+48.Click Back,tap,,"mobile.customer.back.btn"
+50.Reload User App Completely,reload_app,user,
+51. Switch To Web Session,switch_to,web,
+52.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+53. Click Settings Menu,click,,"admin.setting.sidebar.menu"
+54. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+55. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+56.Wait For off,wait,2000,
+57. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
+58. Click Submit Button,click,,"web.global.action.submit"
+59. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+60. Load User App,switch_to,user,
+61.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+62.Click Get Started,tap,,"mobile.customer.get_started.btn"
+63.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+64.Click Next,tap,,"mobile.customer.next.btn"
+65.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+66.Click Close,tap,,"mobile.customer.cancel.btn"
+67.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+68.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+69.Click Continue,tap,,"mobile.customer.continue.btn"
+70.Enter OTP,type,123456,"mobile.customer.edit_text.input"
+71.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+72.Click Finish,tap,,"mobile.customer.finish.btn"
+73.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+74. Wait For Landing Page,wait_until_visible,,"mobile.customer.Landing_page.search_bar"
+75. Click Profile_Menu,tap_coordinate,972:2119,COORDINATE_MODE
+76.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+77.Check Wallet absent,element_absent,,"mobile.customer.wallet.btn"</t>
+  </si>
+  <si>
+    <t>33.Wait For Topup,wait_until_visible,,"mobile.customer.top_up.btn"
+34.Click Topup,tap,,"mobile.customer.top_up.btn"
+35.Wait For Topup Sum,wait_until_visible,,"mobile.customer.top_up.btn"
+36.Click Hundered,tap,,"mobile.customer.top_up_amount.hundred"
+37.Click Proceed,tap,,"mobile.customer.top_up.proceed"
+38.Wait For Contact No,wait_until_visible,,"mobile.customer.top_up.contact_no_box"
+39.Enter Customer Mobile,type,regression.customer.phone,"mobile.customer.top_up.contact_no_box"
+40.Wait For Payment Options,wait_until_visible,,"mobile.customer.top_up.payment_option"
+41.Wait For Net Banking,wait,5000,
+42.Click Net Banking,tap,,"mobile.customer.top_up.net_banking"
+43.Wait For Bob,wait,5000,
+44.Click Bob,tap_coordinate,288:1325,
+45.Wait For Success,wait_until_visible,,"mobile.customer.top_up.succes_popup"
+46.Click Success,tap,,"mobile.customer.top_up.succes_popup"
+47.Wait For Wallet  Back,wait_until_visible,,"mobile.customer.wallet.btn"
+48.Click Back,tap,,"mobile.customer.back.btn"
+49.Drag Page Layout Upward,swipe,up,
+48.Click Back,tap,,"mobile.customer.back.btn"</t>
+  </si>
+  <si>
+    <t>Add Customer App Emergency Number</t>
+  </si>
+  <si>
+    <t>TC_CA_05_Add_Customer_App_Emergency_Number</t>
+  </si>
+  <si>
+    <t>This end-to-end regression test suite validates native customer onboarding workflows and profile property mutations across mobile and web runtime interfaces. The test sequence begins by executing a clean app initialization loop, walking through device access configuration, and utilizing dynamic runtime token generation to process mobile OTP verification steps. It then completes native in-app self-registration by populating customer metadata fields (name strings, email structures, gender flags, and legal checklists) before interacting with coordinate boundaries to locate the account drawer profiles. Crucially, the script provisions an active fallback record inside the native Emergency Contact subsystem, saves the payload, and tests intent handling by triggering the emergency alert call mechanism. Finally, the test switches to the web administration platform to locate the freshly synchronized account record inside the Verified Customers data matrix, opening the admin's inline panel to execute data-integrity lookups against the updated emergency phone element bounds.</t>
+  </si>
+  <si>
+    <t>SA_TS_09</t>
+  </si>
+  <si>
+    <t>TC_CA_09_test_data_cleanup</t>
+  </si>
+  <si>
+    <t>Subscription Plan Complete Test</t>
   </si>
   <si>
     <t>1.Reload User App Completely,reload_app,user,
@@ -2131,7 +1993,7 @@
 58.Enter OTP,type,123456,"mobile.customer.edit_text.input"
 59.Click Finish,tap,,"mobile.customer.finish.btn"
 60.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-61.Profile, tap_coordinate ,971:2102,COORDINATE_MODE
+61.Profile, tap,,"mobile.customer.home_page.profile_icon"
 62.Click Subscription,tap_if_present,,"mobile.customer.subscription.btn"
 63.Wait Customer Plan,wait_if_present,,"mobile.customer.dynamic_subscription.plan"
 64.Click Customer Plan,tap_if_present,,"mobile.customer.dynamic_subscription.plan"
@@ -2170,6 +2032,497 @@
 97.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
 98.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
 99.Wait For Deletion,wait,2000,</t>
+  </si>
+  <si>
+    <t>1.Load User App,switch_to,user,
+2.Reload User App Completely,reload_app,user,
+3.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+4. Load Super Admin,switch_to,web,
+5.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
+6. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+7. Click Settings Menu,click,,"web.global.menu.settings"
+8. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+9. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+10.Wait For On,wait,2000,
+11. Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+12. Click Submit Button,click,,"web.global.action.submit"
+13. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+14. Load User App,switch_to,user,
+15.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+16.Click Get Started,tap,,"mobile.customer.get_started.btn"
+17.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+18.Click Next,tap,,"mobile.customer.next.btn"
+19.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+20.Click Close,tap,,"mobile.customer.cancel.btn"
+21.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+22.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+23.Click Continue,tap,,"mobile.customer.continue.btn"
+24.Enter OTP,type,123456,"mobile.customer.edit_text.input"
+25.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+26.Click Finish,tap,,"mobile.customer.finish.btn"
+27.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+28. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
+29. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+30.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+31.wait for Wallet,wait_until_visible,"mobile.customer.wallet.btn"
+32.Check Wallet Present,element_present,,"mobile.customer.wallet.btn"
+33.Reload User App Completely,reload_app,user,
+34. Switch To Web Session,switch_to,web,
+35.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+36. Click Settings Menu,click,,"admin.setting.sidebar.menu"
+37. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+38. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+39.Wait For off,wait,2000,
+40. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
+41. Click Submit Button,click,,"web.global.action.submit"
+42. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+43. Load User App,switch_to,user,
+44.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+45.Click Get Started,tap,,"mobile.customer.get_started.btn"
+46.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+47.Click Next,tap,,"mobile.customer.next.btn"
+48.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+49.Click Close,tap,,"mobile.customer.cancel.btn"
+50.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+51.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+52.Click Continue,tap,,"mobile.customer.continue.btn"
+53.Enter OTP,type,123456,"mobile.customer.edit_text.input"
+54.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+55.Click Finish,tap,,"mobile.customer.finish.btn"
+56.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+57. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
+58. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+59.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+60.Check Wallet absent,element_absent,,"mobile.customer.wallet.btn"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3. Load User App,switch_to,user,
+4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+5. Click Get Started,tap,,"mobile.customer.get_started.btn"
+6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
+7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
+8. Click Next,tap,,"mobile.customer.next.btn"
+9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap,,"mobile.customer.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
+12. Click Continue,tap,,"mobile.customer.continue.btn"
+13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
+14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
+16. Switch To Web Session,switch_to,web,
+17. Click Customer Menu,click,,"admin.menu.customer_icon"
+18. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
+19. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
+20. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
+21. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
+22. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+23.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
+24. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
+25. Select Male Gender,click,,"admin.customer.select_gender_male"
+26. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+27. Wait for Toast to Hide,wait,3000,,
+28. Click Submit Button,click,,"web.global.action.submit"
+29. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
+30. Click Customer Menu,click,,"admin.menu.customer_icon"
+31. Click Customer Menu,click,,"admin.menu.customer_icon"
+32. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
+33.Wait For Customer Filter,wait,3000,
+34. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+35.Wait For Customer,wait,2000,
+36. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
+37. Load User App,switch_to,user,
+38. Reload User App Completely,reload_app,user,
+39. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+40.Click Get Started,tap,,"mobile.customer.get_started.btn" 
+41.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
+42. Click Next,tap,,"mobile.customer.next.btn"
+43. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+44. Click Close,tap,,"mobile.customer.cancel.btn"
+45. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+46. Click Continue,tap,,"mobile.customer.continue.btn"
+47. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+48. Click Finish,tap,,"mobile.customer.finish.btn"
+49. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+50. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
+51. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+52.Wait For Profile,wait,5000,
+53. Click  Edit Profile,tap,,"mobile.customer.profile_Details.edit_profile_icon"
+54. Wait For Profile Details,wait_until_visible,,"mobile.customer.edit_account.heading"
+55.Click Back,tap,,"mobile.customer.back.btn"
+56.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+57. Drag Page Layout Upward,swipe,up,
+58.Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
+59. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+60. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
+61. Click Manage Account,tap,,"mobile.customer.delete.btn"
+62. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
+63. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
+64. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
+65. Switch To Web Session,switch_to,web,
+66. Click Customer Menu,click,,"admin.menu.customer_icon"
+67. Click Customer DropDown,click,,"admin.menu.customer_icon"
+68. Click Delete Customer,click,,"admin.menu.customer_deleted"
+69.Wait For Delted Customer,wait,3000, 
+70. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+71.Wait For Delted Customer,wait,3000, 
+</t>
+  </si>
+  <si>
+    <t>1. Reload User App Completely,reload_app,user,
+2. Reload Driver App Completely,reload_app,driver,
+3. Load User App,switch_to,user,
+4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+5. Click Get Started,tap,,"mobile.customer.get_started.btn"
+6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
+7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
+8. Click Next,tap,,"mobile.customer.next.btn"
+9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap,,"mobile.customer.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
+12. Click Continue,tap,,"mobile.customer.continue.btn"
+13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input"
+14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+15. Wait For Landing Page,wait_until_visible,,"mobile.customer.register_customer.name"
+16. Enter Customer Name,type,customer{randomAlpha}&gt;&gt;customerName,"mobile.customer.register_customer.name"
+17. Enter Customer Email,type,customer{timestamp}@gmail.com&gt;&gt;customerEmail,"mobile.customer.register_customer.email"
+18. Select gender male,tap,,"mobile.customer.register_customer.gender.female"
+19. Click the checkbox,tap,,"mobile.customer.register_customer.checkbox"
+20. Click sign_up button,tap,,"mobile.customer.register_customer.sign_up"
+21 Click the while using the app,tap,,"mobile.customer.location_allow.btn"
+22. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+23. Click Emergency Contact,tap,,"mobile.customer.menu.Emergency"
+24. Click Add Emergency Contact,tap,,"mobile.customer.menu.Emergency.Emergency_Add_Number"
+25. Enter Emergency Number,type,{randomPhone}&gt;&gt;emergencyPhone,"mobile.customer.menu.Emergency.Emergency_Number_Field"
+26. Click update button in profile,tap,,"mobile.customer.menu.profile_edit.update"
+27. Click Back button in profile,tap,,"mobile.customer.back.btn"
+28. Wait For Emergency Call Button,wait_until_visible,,"mobile.customer.menu.emergency.Emergency_call"
+29. Click Emergency Call Button,tap,,"mobile.customer.menu.emergency.Emergency_call"
+30. Switch To Web Session,switch_to,web,
+31. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+32. Click Customer Icon,click,,"admin.menu.customer_icon"
+33. Click Verified Customers,click,,"admin.menu.verified_customers"
+34. Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
+35. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+36. Scroll Grid,tab,7,"admin.customer.filter_name"
+37. Click Pencil Button,click,,"admin.customer.pencil_edit.btn"
+38.Wait For Popup,wait,1000,
+39.Verify Emergeny Number Matches,verify,{emergencyPhone},"admin.customer.input_Emergency_phone"
+40.Wait For Emergency Number,wait,3000,</t>
+  </si>
+  <si>
+    <t>1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3. Load User App,switch_to,user,
+4. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+5. Click Get Started,tap,,"mobile.customer.get_started.btn"
+6. Wait For Permission,wait_until_visible,,"mobile.customer.permission_allow.btn"
+7. Click Allow Permission,tap,,"mobile.customer.permission_allow.btn"
+8. Click Next,tap,,"mobile.customer.next.btn"
+9. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap,,"mobile.customer.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;customerPhone,"mobile.customer.edit_text.input"
+12. Click Continue,tap,,"mobile.customer.continue.btn"
+13.Wait For Otp,wait_until_visible,,"mobile.customer.edit_text.input""
+14. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+15. Wait For Landing Page,wait_until_visible,,"mobile.customer.ride_complete.+91"
+16. Switch To Web Session,switch_to,web,
+17.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+18. Click Customer Menu,click,,"admin.menu.customer_icon"
+19. Click Non Verified Customers Menu,click,,"admin.menu.customer_non_verified"
+20. Enter Customer Mobile Number,type,{customerPhone},"admin.menu.contact_Filter"
+21. Click Edit Customer,click,,"admin.customer.grid.btn_edit"
+22. Enter Customer Name,type,Customer{randomAlpha}&gt;&gt;customerName,"admin.customer.input_name"
+23. Enter Customer Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+24.Enter Emergency Contact,type,{randomPhone},"admin.customer.input_Emergency_phone"
+25. Click Gender Dropdown,click,,"admin.customer.non_verified.dropdown_gender"
+26. Select Male Gender,click,,"admin.customer.select_gender_male"
+27. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+28. Wait for Toast to Hide,wait,3000,,
+29. Click Submit Button,click,,"web.global.action.submit"
+30. Verify Customer Updated Successfully,verify,,"web.global.toast.updated"
+31. Click Customer Menu,click,,"admin.menu.customer_icon"
+32. Click Customer Menu,click,,"admin.menu.customer_icon"
+33. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
+34.Wait For Customer Filter,wait,3000,
+35. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+36.Wait For Customer,wait,2000,
+37. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
+38. Load User App,switch_to,user,
+39. Reload User App Completely,reload_app,user,
+40. Wait For Permission,wait_until_visible,,"mobile.customer.get_started.btn"
+41.Click Get Started,tap,,"mobile.customer.get_started.btn" 
+42.Click Allow Permission,tap,,"mobile.customer.permission_allow.btn" 
+43. Click Next,tap,,"mobile.customer.next.btn"
+44. Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+45. Click Close,tap,,"mobile.customer.cancel.btn"
+46. Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+47. Click Continue,tap,,"mobile.customer.continue.btn"
+48. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+49. Click Finish,tap,,"mobile.customer.finish.btn"
+50. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+51. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
+52. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+53.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+54. Drag Page Layout Upward,swipe,up,
+55. Click Select Language,tap,,"mobile.customer.Language.btn"
+56. Wait for Language Setting option,wait,3000,,
+57. Click Select Tamil Language,tap,,"mobile.customer.Language.Tamil.button"
+58. Click Select english Language Update,tap,,"mobile.customer.menu.Language.save_changes.btn"
+59. Wait for Language Setting option,wait,3000,,
+60. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+61. Wait For Page Load,wait,3000,
+62. Click Select Language,tap,,"mobile.customer.Language.btn"
+63. Wait for Language Setting option,wait,3000,,
+64. Click Select hindi Language,tap,,"mobile.customer.Language.Hindi.button"
+65. Click Select Tamil Language Update,tap,,"mobile.customer.menu.Language_Tamil.save_changes.btn"
+66. Wait for Profile,wait,3000,,
+67. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+68. Wait For Page Load,wait,3000
+69. Click Select Language,tap,,"mobile.customer.Language.btn"
+70. Wait for Language Setting option,wait,3000,,
+71. Click Select english Language,tap,,"mobile.customer.Language.English.button"
+72. Click Select hindi Language Update,tap,,"mobile.customer.menu.Language_Hindi.save_changes.btn"
+73. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+74. Drag Page Layout Upward,swipe,up,
+75. Wait For Manage Account,wait_until_visible,,"mobile.customer.manage_account.btn"
+76. Click Manage Account,tap,,"mobile.customer.manage_account.btn"
+77. Wait For Delete Account Mange,wait_until_visible,,"mobile.customer.delete.btn"
+78. Click Manage Account,tap,,"mobile.customer.delete.btn"
+79. Wait For Delete Account Sure,wait_until_visible,,"mobile.customer.delete_sure.btn"
+80. Click Delete Account Sure,tap,,"mobile.customer.delete_sure.btn"
+81. Wait For Get_Started,wait_until_visible,,"mobile.customer.get_started.btn"
+82. Switch To Web Session,switch_to,web,
+83. Click Customer Menu,click,,"admin.menu.customer_icon"
+84. Click Customer DropDown,click,,"admin.menu.customer_icon"
+85. Click Delete Customer,click,,"admin.menu.customer_deleted"
+86.Wait For Delete Cusotmer,wait,3000,
+87. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+88. Wait For Delete Cusotmer,wait,3000,</t>
+  </si>
+  <si>
+    <t>1. Reload User App Completely,reload_app,user,
+2. Reload Driver App Completely,reload_app,driver,
+3.  Switch To Web Session,switch_to,web,
+4. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+5. Click drivers menu,click,,"admin.drivers.menu.icon"
+6. Click Add Driver menu,click,,"admin.drivers.add_menu.link"
+7. Verify Add Driver,verify,,"admin.drivers.add_page.header"
+8. Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
+9. Select Auto Ride Option,click,,"admin.drivers.service_dropdown.auto_ride"
+10.Click Driver Type Dropdown,click,,"admin.drivers.driver_type.dropdown"
+11.Select pilot Option,click,,"admin.drivers.driver_type.dropdown_pilot"
+12. Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "admin.drivers.fullname.input"
+13. Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "admin.drivers.email.input"
+14. Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "admin.drivers.phone.input"
+15. Click Whatspp, click, , "admin.drivers.whatsapp.checkbox"
+16. Enter Whatspp Number, type, {autoPhone}, "admin.drivers.whatsapp_phone.input"
+17. Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "admin.drivers.profile_image.file"
+18. Select Source,click,,"admin.drivers.source_dropdown.select"
+19. Select Instagram,click,,"admin.drivers.instagram_option.span"
+20. Select Male Gender, click, , "admin.drivers.male_gender.div"
+21. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
+22. Select  Auto Option,click,,"admin.drivers.vehicle_option.pinkauto"
+23. Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
+24. Enter Plate No, type, KL-01-AB-1234, "admin.drivers.plateno.input"
+25. Enter Model Name, type, petrol, "admin.drivers.modelname.input"
+26. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "admin.drivers.vehicle_image.file"
+27. Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
+28. Enter Bank Location, type, PARK STREET, "admin.drivers.banklocation.input"
+29. Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
+30. Enter Account Holder Name, type,{autoName}, "admin.drivers.accountholder.input"
+31. Enter Payment Email Address, type, {autoEmail}, "admin.drivers.paymentemail.input"
+32. Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
+33. Click Submit, click, , "web.global.action.submit"
+34. Verify Driver Added, verify,, "web.global.toast.success"
+35. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+36. Click drivers menu,click,,"admin.drivers.menu.icon"
+37. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+38. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+39. Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
+40. Click Doc Icon,click,,"admin.drivers.docs.icon"
+41. Driver Required Documents,verify,,"admin.drivers.required_docs.header"
+42. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+43. Add Driving License,click,,"admin.drivers.docs.edit_icon"
+44. Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "admin.drivers.profile_image.file"
+45. Enter Expiry Date,set_date,2026-12-12,"admin.drivers.doc_expiry.input"
+46. Click Submit, click, , "web.global.action.submit"
+47. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+48. Click Approve Driver,click,,"admin.drivers.docs.approval"
+49. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+50. Click Dashboard,click,,"web.global.menu.dashboard"
+51. Click drivers menu,click,,"admin.drivers.menu.icon"
+52. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+53. Approved Drivers List,verify,,"admin.drivers.approved_page.header"
+54. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+55. Wait For Get_Started,wait_until_visible,,"admin.drivers.name_filter.input"
+56. Load Driver App,switch_to,driver,
+57. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+58. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+59. Click Agree,tap,,"mobile.driver.agree.btn"
+60. Click Get Started,tap,,"mobile.driver.get_started.btn"
+61. Click Next,tap,,"mobile.driver.next.btn"
+62. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+63. Click Close,tap,,"mobile.driver.cancel.btn"
+64. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+65. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+66. Click Continue,tap,,"mobile.driver.continue.btn"
+67. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+68.Enter Account Holder,type,{autoName},"mobile.driver.bank_details.account_holder_name"
+69.Enter Account Number,type,50100123456789,"mobile.driver.bank_details.account_number"
+70.Enter Confirm Account Number,type,50100123456789,"mobile.driver.bank_details.confirm_account_number"
+71.Enter IFSC Code,type,HDFC0001234,"mobile.driver.bank_details.confirm_ifsc_code"
+72.Wait For Keyboard Minimises,hide_keyboard,,
+73.Enter Upi Id,type,sujanpariyar07@fam,"mobile.driver.bank_details.upi_id"
+74.Wait For Keyboard Minimises,hide_keyboard,,
+75.Click Submit,click,,"mobile.driver.bank_details.submit_btn"
+76. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+77. Wait for Toast to Hide,wait,3000,,
+78. Click Select All Agree,tap,,"mobile.driver.independent_contractor.checkbox_Select_All"
+79. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+80. Click Agree,tap,,"mobile.driver.agree_continue.btn"
+81. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+82. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+83. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+84.Wait For Hamburger Menu,wait,3000
+85. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+86.Wait For Driver Profile Load,wait,3000,
+87. Drag Page Layout Upward,swipe,up,
+88.Wait For Language Menu,wait,3000,
+89. Click Language menu,tap,,"mobile.driver.Language.btn"
+90. Wait for Language Setting option,wait,3000,,
+91. Click Select Tamil Language,tap,,"mobile.driver.Language.Tamil.button"
+92. Click Select Tamil Language Update,tap,,"mobile.driver.menu.Language.save_changes.btn"
+93. Wait for Language Setting option,wait,3000,,
+94. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+95. Drag Page Layout Upward,swipe,up,
+96.Wait For Page Load,wait,3000,
+97. Click Language menu,tap,,"mobile.driver.Language.btn"
+98. Wait for Language Setting option,wait,3000,,
+99. Click Select Hindi Language,tap,,"mobile.driver.Language.Hindi.button"
+100. Click Select Hindi Language Update,tap,,"mobile.driver.menu.Language_Tamil.save_changes.btn"
+101.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+102.Drag Page Layout Upward,swipe,up,
+103.Wait For Page Load,wait,3000,
+104.Click Language menu,tap,,"mobile.driver.Language.btn"
+105.Wait for Language Setting option,wait,3000,,
+106.Click Select English Language,tap,,"mobile.driver.Language.English.button"
+107.Click Select English Language Update,tap,,"mobile.driver.menu.Language_Hindi.save_changes.btn"
+108. Wait for Language Setting option,wait,3000,,
+109.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+110.Drag Page Layout Upward,swipe,up,
+111.Wait for Manage Account Loading,wait,3000,,
+112.Click Manage Account,tap_coordinate,503:2084,COORDINATE_MODE
+113.Click Delete Account,tap,,"mobile.driver.delete.btn"
+114.Click Delete Account Sure,tap,,"mobile.driver.delete_sure.btn"
+115.Switch To Web Session,switch_to,web,
+116. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+117. Click drivers menu,click,,"admin.drivers.menu.icon"
+118.Click Delete Driver,click,,"admin.drivers.delete_drivers.menu"
+119.Wait For Load,wait,1000,
+120. Enter Driver Name,type,{autoName},"admin.drivers.name_filter.input" 
+121.Wait For Load,wait,3000,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3.Load Driver App,switch_to,driver,
+4.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+5.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+6.Click Agree,tap,,"mobile.driver.agree.btn"
+7.Click Get Started,tap,,"mobile.driver.get_started.btn"
+8.Click Next,tap,,"mobile.driver.next.btn"
+9.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+10.Click Close,tap,,"mobile.driver.cancel.btn"
+11.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+12.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+13 Click Continue,tap,,"mobile.driver.continue.btn"
+14. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+15.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+16.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+17.Wait For Pageload,wait,3000,
+17.1.Click Online Toggle,tap_coordinate,982:1932,
+18.Load User App,switch_to,user,
+19.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+20.Click Get Started,tap,,"mobile.customer.get_started.btn"
+21.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+22.Click Next,tap,,"mobile.customer.next.btn"
+23.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+24.Click Close,tap,,"mobile.customer.cancel.btn"
+25.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+26.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+27. Click Continue,tap,,"mobile.customer.continue.btn"
+28. Enter OTP,type,123456,"mobile.customer.edit_text.input"
+29. Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+30. Click Finish,tap,,"mobile.customer.finish.btn"
+31. Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+32. Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+33. Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+34. Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+35. Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+36. Select Destination,tap,,"mobile.customer.destination_suggestion_first"
+37.Wait For Entrance,wait_until_visible,,"mobile.customer.destination_entrance_location"
+38.Click Entrance,tap,,"mobile.customer.destination_entrance_location"
+39. Click Confirm,tap,,"mobile.customer.confirm.btn"
+39.1.Wait For Ride,wait,5000,
+40. Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+41. Ride Now,tap,,"mobile.customer.ride_now.btn"
+42. Load Driver App,switch_to,driver,
+43.Wait for Accept,wait_until_visible,,"mobie.driver.auto_ride_accept.button"
+44.Click  Accept Ride,tap,,"mobie.driver.auto_ride_accept.button"
+45.Fetch Ride Code from DB,fetch_db_value,ride_otp,"SELECT otp FROM we1.user_ride_booking ORDER BY id DESC LIMIT 1"
+46.Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
+47.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+48.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+49.Ride Arrived,tap,,"mobile.driver.arrived.btn"
+50.Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+51.Yes Arrived,tap,,"mobile.driver.yes.btn"
+52.Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
+53.Start Ride,tap,,"mobile.driver.start_ride.btn"
+54.wait for Otp,wait_until_visible,,"mobile.driver.otp_view.input"
+55.Enter OTP,type,{ride_otp},"mobile.driver.otp_view.input"
+56.Wait for Start Button,wait_until_visible,,"mobile.driver.start.btn"
+57.Start Ride Button,tap,,"mobile.driver.start.btn"
+58.Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
+59.Complete Ride,tap,,"mobile.driver.complete_ride.btn"
+60.Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
+61.Collect Payment,tap,,"mobile.driver.collect_payment.btn"
+62.Load User App,switch_to,user,
+63.Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+64.Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
+65. Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+66. Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
+67. Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
+68. Give Review,tap,,"mobile.customer.give_review.btn"
+69. Give Rating,tap_coordinate,348:1619,
+70. Submit Rating,tap,,"mobile.customer.submit_rating.btn"
+71.Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
+72.Trip Finished,tap,,"mobile.customer.done.btn"
+73. Load Driver App,switch_to,driver,
+74.Wait  For Proceed,wait_until_visible,,"mobile.driver.payment.proceed_btn"
+75.Click For Proceed,tap,,"mobile.driver.payment.proceed_btn"
+76. Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+77. Confirm Payment,tap,,"mobile.driver.yes.btn"
+78.Wait For Give Review Button,wait_until_visible,,"mobile.driver.give_review.btn"
+79.Click Give Review Button,tap,,"mobile.driver.give_review.btn"
+80.Wait For Rating,wait,2000,
+81. Give Rating,tap_coordinate,348:1545,
+82. Submit Rating,tap,,"mobile.driver.submit_rating.btn"
+83.Wait for Complete Button,wait_until_visible,,"mobile.driver.complete.btn"
+84.Click Complete Button,tap,,"mobile.driver.complete.btn"
+85.Wait For  ride complete submit button,wait_until_visible,,"mobile.driver.ride_complete_submit.btn"
+86.Click Ride Complete Submit Button,tap,,"mobile.driver.ride_complete_submit.btn"
+</t>
+  </si>
+  <si>
+    <t>TC_CA_06_Customer_Language_Check</t>
+  </si>
+  <si>
+    <t>TC_CA_07_Driver_Language_Check</t>
+  </si>
+  <si>
+    <t>TC_CA_08_Autoride_Complete_Test</t>
   </si>
 </sst>
 </file>
@@ -2617,6 +2970,90 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D250DB7C-844B-4BAE-BD85-886B660DFD66}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B31CB41-AC3C-4084-88C1-98C363B7ABCB}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2659,25 +3096,25 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="H2" s="2"/>
     </row>
@@ -2698,7 +3135,91 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A659562-16FE-472A-9348-C2754F8B87F9}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2740,13 +3261,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>57</v>
+        <v>84</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>9</v>
@@ -2815,13 +3336,13 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>34</v>
@@ -2893,13 +3414,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>37</v>
@@ -2968,13 +3489,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>13</v>
@@ -3033,7 +3554,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>19</v>
@@ -3044,25 +3565,25 @@
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3128,19 +3649,19 @@
         <v>38</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
@@ -3167,6 +3688,90 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0586A9D0-0ABC-41A4-8FF3-8503F348B496}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{437C624E-95B4-48EB-A315-8931C834404A}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3209,22 +3814,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
@@ -3250,8 +3855,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A659562-16FE-472A-9348-C2754F8B87F9}">
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0962450F-C7D8-41FC-90CD-CAAFB127F74F}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3293,28 +3898,28 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>43</v>
+        <v>81</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3332,88 +3937,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D250DB7C-844B-4BAE-BD85-886B660DFD66}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
92th Commit:Swipe Keyword Implemented
</commit_message>
<xml_diff>
--- a/we1_hybrid_regression.xlsx
+++ b/we1_hybrid_regression.xlsx
@@ -8,25 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B23434-8C2C-4C9A-B87D-A168AC24F989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89234CCC-3091-490C-BA71-9CAB72755CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
-    <sheet name="HybridAddCustomer" sheetId="44" r:id="rId2"/>
-    <sheet name="HybridUnApprovedAutoDriver" sheetId="46" r:id="rId3"/>
-    <sheet name="HybridApprovedAutoDriver" sheetId="38" r:id="rId4"/>
-    <sheet name="HybridSubscriptionPlanTest" sheetId="40" r:id="rId5"/>
-    <sheet name="DriverAppWalletVerification" sheetId="48" r:id="rId6"/>
-    <sheet name="CustomerAppWalletCheck" sheetId="55" r:id="rId7"/>
-    <sheet name="NonVerifiedAndDeletedCustomer" sheetId="50" r:id="rId8"/>
-    <sheet name="CustomerAppEmergencyNumber" sheetId="56" r:id="rId9"/>
-    <sheet name="CustomerLanguageCheck" sheetId="52" r:id="rId10"/>
-    <sheet name="DriverLanguageCheck" sheetId="53" r:id="rId11"/>
+    <sheet name="HybridSubscriptionPlanTest" sheetId="40" r:id="rId2"/>
+    <sheet name="DriverAppWalletVerification" sheetId="48" r:id="rId3"/>
+    <sheet name="CustomerAppWalletCheck" sheetId="55" r:id="rId4"/>
+    <sheet name="NonVerifiedAndDeletedCustomer" sheetId="50" r:id="rId5"/>
+    <sheet name="CustomerAppEmergencyNumber" sheetId="56" r:id="rId6"/>
+    <sheet name="CustomerLanguageCheck" sheetId="52" r:id="rId7"/>
+    <sheet name="DriverLanguageCheck" sheetId="53" r:id="rId8"/>
+    <sheet name="RideCustomerReportIssue" sheetId="58" r:id="rId9"/>
+    <sheet name="AutoRideTestOtpUi" sheetId="57" r:id="rId10"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId11"/>
     <sheet name="AutoRideTestOtpDb" sheetId="54" r:id="rId12"/>
-    <sheet name="AutoRideTestOtpUi" sheetId="57" r:id="rId13"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId14"/>
+    <sheet name="HybridAddCustomer" sheetId="44" r:id="rId13"/>
+    <sheet name="HybridUnApprovedAutoDriver" sheetId="46" r:id="rId14"/>
+    <sheet name="HybridApprovedAutoDriver" sheetId="38" r:id="rId15"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="105">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -1334,83 +1335,6 @@
 18.Click Online Toggle Button,tap,,"mobile.driver.online_toggle.btn"</t>
   </si>
   <si>
-    <t>1. Load Driver App,switch_to,driver,
-2.Reload Driver App Completely,reload_app,driver,
-3. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-4. Load Super Admin,switch_to,web,
-5.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
-6. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-7. Click Settings Menu,click,,"web.global.menu.settings"
-8. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
-9. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
-10.Wait For On,wait,2000,
-11. Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
-12. Click Submit Button,click,,"web.global.action.submit"
-13. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
-14. Load Driver App,switch_to,driver,
-15. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-16. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-17. Click Agree,tap,,"mobile.driver.agree.btn"
-18. Click Get Started,tap,,"mobile.driver.get_started.btn"
-19. Click Next,tap,,"mobile.driver.next.btn"
-20. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-21. Click Close,tap,,"mobile.driver.cancel.btn"
-22. Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
-23. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-24. Click Continue,tap,,"mobile.driver.continue.btn"
-25. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-26. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-27. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-28. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-29.wait for Wallet,wait_until_visible,"mobile.driver.wallet.btn"
-30.Click Wallet,tap,,"mobile.driver.wallet.btn"
-31.Wait For Topup,wait_until_visible,,"mobile.driver.top_up.btn"
-32.Click Topup,tap,,"mobile.driver.top_up.btn"
-33.Wait For Topup Sum,wait_until_visible,,"mobile.driver.top_up.btn"
-34.Click Hundered,tap,,"mobile.driver.top_up_amount.hundred"
-35.Click Proceed,tap,,"mobile.driver.top_up.proceed"
-36.Wait For Contact No,wait_until_visible,,"mobile.driver.top_up.contact_no_box"
-37.Enter Driver Mobile,type,regression.approved_driver.phone,"mobile.driver.top_up.contact_no_box"
-38.Wait For Payment Options,wait_until_visible,,"mobile.driver.top_up.payment_option"
-39.Wait For Net Banking,wait,5000,
-40.Click Net Banking,tap,,"mobile.driver.top_up.net_banking"
-41.Wait For Bob,wait,5000,
-42.Click Bob,tap_coordinate,288:1325,
-43.Wait For Success,wait_until_visible,,"mobile.driver.top_up.succes_popup"
-44.Click Success,tap,,"mobile.driver.top_up.succes_popup"
-45.Wait For Wallet  Back,wait_until_visible,,"mobile.driver.wallet.btn"
-46.Click Back,tap,,"mobile.driver.back.btn"
-47.Drag Page Layout Upward,swipe,up,
-48.Click Back,tap,,"mobile.driver.back.btn"
-49.Reload Driver App Completely,reload_app,driver,
-50. Switch To Web Session,switch_to,web,
-51.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-52. Click Settings Menu,click,,"admin.setting.sidebar.menu"
-53. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
-54. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
-55.Wait For off,wait,2000,
-56. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
-57. Click Submit Button,click,,"web.global.action.submit"
-58. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
-59. Switch To Driver Session,switch_to,driver,
-60. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-61. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-62. Click Agree,tap,,"mobile.driver.agree.btn"
-63. Click Get Started,tap,,"mobile.driver.get_started.btn"
-64. Click Next,tap,,"mobile.driver.next.btn"
-65. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-66. Click Close,tap,,"mobile.driver.cancel.btn"
-67. Enter Mobile Number,type,regression.approved_driver.phone ,"mobile.driver.edit_text.input"
-68. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-69. Click Continue,tap,,"mobile.driver.continue.btn"
-70. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-71. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-72. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-73.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-74.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
-75.Check Wallet absent,element_absent,,"mobile.driver.wallet.btn"</t>
-  </si>
-  <si>
     <t>SA_TS_07</t>
   </si>
   <si>
@@ -1428,15 +1352,9 @@
     <t>SA_TS_0A</t>
   </si>
   <si>
-    <t>TC_CA_0A_Hybrid_Add_Customer</t>
-  </si>
-  <si>
     <t>SA_TS_0B</t>
   </si>
   <si>
-    <t>TC_CA_0B_Hybrid_Unapproved_Auto_Driver</t>
-  </si>
-  <si>
     <t>TC_CA_01_Hybrid_Subscription_Plan_Test</t>
   </si>
   <si>
@@ -1462,9 +1380,6 @@
   </si>
   <si>
     <t>SA_TS_0C</t>
-  </si>
-  <si>
-    <t>TC_CA_0C_Hybrid_Approved_Auto_Driver</t>
   </si>
   <si>
     <r>
@@ -2154,120 +2069,13 @@
     <t>Auto Ride Complete Life Cycle Test With Otp Fetched From DB</t>
   </si>
   <si>
-    <t>TC_CA_08_Autoride_Test_Otp_DB</t>
-  </si>
-  <si>
     <t>Auto Ride Test With Otp Fetched From UI</t>
   </si>
   <si>
-    <t>TC_CA_09_Autoride_Test_Otp_Ui</t>
-  </si>
-  <si>
     <t>SA_TS_10</t>
   </si>
   <si>
     <t>TC_CA_10_test_data_cleanup</t>
-  </si>
-  <si>
-    <t>1.Reload User App Completely,reload_app,user,
-2.Reload Driver App Completely,reload_app,driver,
-3.Load Super Admin,switch_to,web,
-4.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-5.Click Subscription Plan,click,,"admin.subscription.menu_link"
-6.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
-7.Verify Driver Subscription Plan Lists ,verify,,"admin.subscription.driver.header"
-8.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_add"
-9.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
-10.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
-11.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "admin.subscription.common.name.input"
-12.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
-13.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.input"
-14.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.input"
-15.Enter Number Of Days, type,100, "admin.subscription.common.days.alt_input"
-16.Enter Number Of Free Rides, type,2, "admin.subscription.driver.free_rides.input"
-17.Enter Price, type,5000, "admin.subscription.common.price.input"
-18.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.driver.desc_english.textarea"
-19.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.driver.desc_arabic.textarea"
-20.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.driver.desc_tamil.textarea"
-21.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.driver.desc_hindi.textarea"
-22.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
-23.Select On,click,,"admin.subscription.common.status.option_on"
-24.Click Submit ,click,,"web.global.action.submit"
-25.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
-26.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-27.Click Subscription Plan,click,,"admin.subscription.menu_link"
-28.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
-29.Verify Customer Subscription Plan Lists ,verify,,"admin.subscription.customer.header"
-30.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
-31.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
-32.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
-33.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "admin.subscription.common.name.input"
-34.Enter Customer Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
-35.Enter Customer Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
-36.Enter Customer Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
-37.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
-38.Enter Number Of Free Rides, type,2, "admin.subscription.customer.free_rides.input"
-39.Enter Price, type,5000, "admin.subscription.common.price.input"
-40.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.customer.desc_english.textarea"
-41.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.customer.desc_arabic.textarea"
-42.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.customer.desc_tamil.textarea"
-43.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.customer.desc_hindi.textarea"
-44.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
-45.Select On,click,,"admin.subscription.common.status.option_on"
-46.Click Submit ,click,,"web.global.action.submit"
-47.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
-48.Load User App,switch_to,user,
-49.Wait for Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-50.Click Get Started,tap,,"mobile.customer.get_started.btn"
-51.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-52.Click Next,tap,,"mobile.customer.next.btn"
-53.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-54.Click Close,tap,,"mobile.customer.cancel.btn"
-55.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
-56.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-57.Click Continue,tap,,"mobile.customer.continue.btn"
-58.Enter OTP,type,123456,"mobile.customer.otp_input"
-59.Click Finish,tap,,"mobile.customer.finish.btn"
-60.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-61.Profile, tap,,"mobile.customer.home_page.profile_icon"
-62.Click Subscription,tap_if_present,,"mobile.customer.subscription.btn"
-63.Wait Customer Plan,wait_if_present,,"mobile.customer.dynamic_subscription.plan"
-64.Click Customer Plan,tap_if_present,,"mobile.customer.dynamic_subscription.plan"
-65.Load Driver App,switch_to,driver,
-66.Wait for Popup,wait_until_visible,,"mobile.driver.permission_allow.btn"
-67.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-68.Click Agree,tap,,"mobile.driver.agree.btn"
-69.Click Get Started,tap,,"mobile.driver.get_started.btn"
-70.Click Next,tap,,"mobile.driver.next.btn"
-71.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-72.Click Close,tap,,"mobile.driver.cancel.btn"
-73.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
-74.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-75.Click Continue,tap,,"mobile.driver.continue.btn"
-76.Enter OTP,type,123456,"mobile.driver.edit_text.input"
-77.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-78.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-79.wait for page load,wait,5000,
-80.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
-81.wait for page load,wait,5000,
-82.Click Subscription,tap,,"mobile.driver.subscription.btn"
-83.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
-84.Click Driver Plan,tap,,"mobile.driver.dynamic_subscription.plan"
-85.Load Super Admin,switch_to,web,
-86.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-87.Click Subscription Plan,click,,"admin.subscription.menu_link"
-88.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
-89.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
-90.Click Delete Customer Subscription Plan,click,,"admin.subscription.customer.delete.icon"
-91.Confirm Delete Customer Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
-92.Wait For Deletion,wait,2000,
-93.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-94.Click Subscription Plan,click,,"admin.subscription.menu_link"
-95.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
-96.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
-97.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
-98.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
-99.Wait For Deletion,wait,2000,</t>
   </si>
   <si>
     <t>1.Load User App,switch_to,user,
@@ -2627,6 +2435,301 @@
 86.Wait For Delete Cusotmer,wait,3000,
 87. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
 88. Wait For Delete Cusotmer,wait,3000,</t>
+  </si>
+  <si>
+    <t>Customer Report Issue For Completed Ride</t>
+  </si>
+  <si>
+    <t>1. Load User App,switch_to,user,
+2.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+3.Click Get Started,tap,,"mobile.customer.get_started.btn"
+4.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+5.Click Next,tap,,"mobile.customer.next.btn"
+6.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+7.Click Close,tap,,"mobile.customer.cancel.btn"
+8.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+9.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+10.Click Continue,tap,,"mobile.customer.continue.btn"
+11.Enter OTP,type,123456,"mobile.customer.otp_input"
+12.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+13.Click Finish,tap,,"mobile.customer.finish.btn"
+14.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+15. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
+16. Click Profile Menu,tap,,"mobile.customer.home_page.profile_icon"
+17.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+18.Click My Orders,tap,,"mobile.customer.profile.my_orders_btn"
+19.Wait For My Orders Heading,wait_until_visible,,"mobile.customer.profile.my_orders_heading"
+20.Click Today Button,tap,,"mobile.customer.my_orders.today_dropdown"
+21.Wait For Popup,wait_until_visible,,"mobile.customer.my_orders.today_popup_heading"
+22.Click All,tap,,"mobile.customer.my_orders.all_orders_button"
+23.Click Apply Filter Button,tap,,"mobile.customer.my_orders.apply_filter"
+24.Wait For Rides List To Load,wait,3000,
+25.Swipe Top Bar,swipe,left,"mobile.customer.my_orders.order_status_top_bar"
+26.Wait For Rides List To Load,wait,2000,
+27.Click Completed Rides,tap,,"mobile.customer.my_orders.completed"
+28.Wait For Rides List To Load,wait,5000,
+29.Click Completed Ride,tap_coordinate,532:961,
+30.Wait For Three Dot Menu,wait_until_visible,,"mobile.customer.my_orders.three_dot_menu"
+31.Click Three Dot Menu,tap,,"mobile.customer.my_orders.three_dot_menu"
+32.Click Report Issue Popup,tap,,"mobile.customer.my_orders.report_issue"
+33.Type Issue Description,type,Bad Behaviour Of Driver,"mobile.customer.my_orders.report_issue.description_fld"
+34.Click Add Image,tap,,"mobile.customer.my_orders.report_issue.add_image"
+35.Click Camera  Icon,tap,,"mobile.customer.my_orders.report_issue.add_image_camera"
+36.Click Allow Notification,tap_if_present,,"mobile.customer.my_orders.report_issue.camera_allow_notification"
+37.Wait For Camera Shutter,wait_until_visible,,"mobile.customer.my_orders.report_issue.add_image_camera_shutter"
+38.Clilck Camera Shutter,tap,,"mobile.customer.my_orders.report_issue.add_image_camera_shutter"
+39.Wait For Done,wait_until_visible,,"mobile.customer.my_orders.report_issue.add_image_done"
+40.Click Done,tap,,"mobile.customer.my_orders.report_issue.add_image_done"
+41.Wait For Crop,wait_until_visible,,"mobile.customer.my_orders.report_issue.crop_done"
+42.Click Crop,tap,,"mobile.customer.my_orders.report_issue.crop_done"
+43.Wait For Submit Issue Button,wait_until_visible,,"mobile.customer.my_orders.report_issue.submit_issue_btn"
+44.Click Submit Issue Button,tap,,"mobile.customer.my_orders.report_issue.submit_issue_btn"
+45.Wait For Report Issue Chat Button,wait_until_visible,,"mobile.customer.my_orders.report_issue.chat_btn"
+46.Extract Ticket ID From Ui,store_text,ticket_id,"mobile.customer.my_orders.report_issue.ticket_id_field"
+47.Click Chat Button,tap,,"mobile.customer.my_orders.report_issue.chat_btn"
+48.Wait For Chat Box,wait_until_visible,,"mobile.customer.my_orders.report_issue.chat_box"
+49.Type Chat,type,Hi today had an bad experince from your driver with above ride id please look into it take necessary action thank you,"mobile.customer.my_orders.report_issue.chat_box"
+50.Enter Chat,tap,,"mobile.customer.my_orders.report_issue.chat_box_enter_btn"
+51.Switch To Web Session,switch_to,web,
+52.Click Dashboard,click,,"web.global.menu.dashboard"
+53.Click Report Issue,click,,"admin.report_issue.side_bar.menu"
+54.Click Customer Report Issue,click,,"admin.report_issue.side_bar_sub_menu.customer_report_issues"
+55.Filter Created By,type,regression customer,"admin.report_issue.customer_report_issues.created_by_filter_input"
+56.Scroll Grid,tab,5,"admin.report_issue.customer_report_issues.created_by_filter_input"
+57.Filter Resolved Status,type,Unresolved,"admin.report_issue.customer_report_issues.status_filter_input"
+58.Scroll Grid,tab,1,"admin.report_issue.customer_report_issues.status_filter_input"
+59.Wait For Grid Load,wait,2000,
+60.View Eye Icon,click,,"admin.report_issue.customer_report_issues.eye_icon"
+61.Close Eye Icon,click,,"admin.report_issue.customer_report_issues.close_eye_icon"
+62.Click Chat Icon,click,,"admin.report_issue.customer_report_issues.chat_icon"
+63.Reply Customer Issue,type,Thank you for raising the issue strict action will be taken against the driver we apolgize for inconvince,"admin.report_issue.customer_report_issues.chat_box"
+64.Click Enter Chat,click,,"admin.report_issue.customer_report_issues.chat_box_enter_btn"
+65.Close Chat Box,click,,"admin.report_issue.customer_report_issues.close_chat_icon"
+66.Click Resolved Issue,click,,"admin.report_issue.customer_report_issues.resolve_thumbs_icon"      
+67.Confirm Resolved Issue,click,,"admin.report_issue.customer_report_issues.resolve_confirm_yes"
+68. Load User App,switch_to,user,
+69.Wait For Chat Box,wait_until_visible,,"mobile.customer.my_orders.report_issue.chat_box"
+70.Click Back Button,tap,,"mobile.customer.my_orders.report_issue.back_btn"
+71.Wait For Chat Button,wait_until_visible,,"mobile.customer.my_orders.report_issue.chat_btn"
+72.Click Back Button,tap,,"mobile.customer.my_orders.report_issue.back_btn"
+73.Wait For Three Dot Menu,wait_until_visible,,"mobile.customer.my_orders.three_dot_menu"
+74. Click Back Button,tap,,"mobile.customer.my_orders.report_issue.back_btn"
+75.Wait for My Orders Heading,wait_until_visible,,"mobile.customer.profile.my_orders_heading" 
+76.Click Back Button,tap,,"mobile.customer.my_orders.report_issue.back_btn"
+77.Wait For  Profile Load,wait,2000,
+78.Swipe Up Page,swipe,up,
+79.Wait For Profile Load,wait,2000, 
+80.Click Report Issue,click,,"mobile.customer.profile.report_issue"
+81.Wait for Add Issue,wait_until_visible,,"mobile.customer.report_issue.add_issue_btn" 
+82.Click Add Issue Button,click,,"mobile.customer.report_issue.add_issue_btn"
+83.Wait For Issue To Load,wait,5000,
+84.Click Resolved Issue,tap_coordinate,911:716,
+85.Wait For Resolved Issue To Load,wait,5000,</t>
+  </si>
+  <si>
+    <t>1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3.Load Super Admin,switch_to,web,
+4.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+5.Click Subscription Plan,click,,"admin.subscription.menu_link"
+6.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
+7.Verify Driver Subscription Plan Lists ,verify,,"admin.subscription.driver.header"
+8.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_add"
+9.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+10.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
+11.Enter Driver Plan Name, type, DriverPlan{randomAlpha}&gt;&gt; driverSubscriptionName, "admin.subscription.common.name.input"
+12.Enter Driver Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+13.Enter Driver Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.input"
+14.Enter Driver Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.input"
+15.Enter Number Of Days, type,100, "admin.subscription.common.days.alt_input"
+16.Enter Number Of Free Rides, type,2, "admin.subscription.driver.free_rides.input"
+17.Enter Price, type,50, "admin.subscription.common.price.input"
+18.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.driver.desc_english.textarea"
+19.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.driver.desc_arabic.textarea"
+20.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.driver.desc_tamil.textarea"
+21.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.driver.desc_hindi.textarea"
+22.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+23.Select On,click,,"admin.subscription.common.status.option_on"
+24.Click Submit ,click,,"web.global.action.submit"
+25.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
+26.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+27.Click Subscription Plan,click,,"admin.subscription.menu_link"
+28.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
+29.Verify Customer Subscription Plan Lists ,verify,,"admin.subscription.customer.header"
+30.Click  Add New Subscription,click,,"admin.subscription.common.add_new.btn_widget"
+31.Open Service Category Dropdown,click,,"admin.subscription.common.category.dropdown"
+32.Select Auto Ride,click,,"admin.subscription.common.category.option_autoride"
+33.Enter Customer Plan Name, type,CustomerPlan{randomAlpha}&gt;&gt; customerSubscriptionName, "admin.subscription.common.name.input"
+34.Enter Customer Plan Name Arabic, type,عضو ذهبي, "admin.subscription.common.name_arabic.input"
+35.Enter Customer Plan Name Tamil, type,தங்க உறுப்பினர், "admin.subscription.common.name_tamil.alt_input"
+36.Enter Customer Plan Name Hindi, type,गोल्ड मेंबर, "admin.subscription.common.name_hindi.alt_input"
+37.Enter Number Of Days, type,100, "admin.subscription.common.days.input"
+38.Enter Number Of Free Rides, type,2, "admin.subscription.customer.free_rides.input"
+39.Enter Price, type,50, "admin.subscription.common.price.input"
+40.Enter Plan Description English, type,A premium tier status offering exclusive benefits and high-level rewards to loyal users, "admin.subscription.customer.desc_english.textarea"
+41.Enter Plan Description Arabic, type,فئة عضوية مميزة تمنح المستخدمين المخلصين مزايا حصرية ومكافآت رفيعة المستوى, "admin.subscription.customer.desc_arabic.textarea"
+42.Enter Plan Description Tamil, type,இது விசுவாசமான பயனர்களுக்கு பிரத்யேக நன்மைகள் மற்றும் சலுகைகளை வழங்கும் ஒரு பிரீமியம் உறுப்பினர் நிலையாகும், "admin.subscription.customer.desc_tamil.textarea"
+43.Enter Plan Description Hindi, type,यह एक प्रीमियम सदस्यता स्तर है जो वफादार उपयोगकर्ताओं को विशेष लाभ और पुरस्कार प्रदान करता है, "admin.subscription.customer.desc_hindi.textarea"
+44.Open status Dropdown,click,,"admin.subscription.common.status.dropdown"
+45.Select On,click,,"admin.subscription.common.status.option_on"
+46.Click Submit ,click,,"web.global.action.submit"
+47.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
+48.Load User App,switch_to,user,
+49.Wait for Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+50.Click Get Started,tap,,"mobile.customer.get_started.btn"
+51.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+52.Click Next,tap,,"mobile.customer.next.btn"
+53.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+54.Click Close,tap,,"mobile.customer.cancel.btn"
+55.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
+56.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+57.Click Continue,tap,,"mobile.customer.continue.btn"
+58.Enter OTP,type,123456,"mobile.customer.otp_input"
+59.Click Finish,tap,,"mobile.customer.finish.btn"
+60.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+61.Profile, tap,,"mobile.customer.home_page.profile_icon"
+62.Click Subscription,tap_if_present,,"mobile.customer.subscription.btn"
+63.Wait Customer Plan,wait_if_present,,"mobile.customer.dynamic_subscription.plan"
+64.Click Customer Plan,tap_if_present,,"mobile.customer.dynamic_subscription.plan"
+65.Load Driver App,switch_to,driver,
+66.Wait for Popup,wait_until_visible,,"mobile.driver.permission_allow.btn"
+67.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+68.Click Agree,tap,,"mobile.driver.agree.btn"
+69.Click Get Started,tap,,"mobile.driver.get_started.btn"
+70.Click Next,tap,,"mobile.driver.next.btn"
+71.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+72.Click Close,tap,,"mobile.driver.cancel.btn"
+73.Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+74.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+75.Click Continue,tap,,"mobile.driver.continue.btn"
+76.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+77.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+78.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+79.wait for page load,wait,5000,
+80.Click Hamburge,tap_coordinate ,75:209,COORDINATE_MODE
+81.wait for page load,wait,5000,
+82.Click Subscription,tap,,"mobile.driver.subscription.btn"
+83.Wait Driver Plan,wait_until_visible,,"mobile.driver.dynamic_subscription.plan"
+84.Click Driver Plan,tap_if_present,,"mobile.driver.dynamic_subscription.plan"
+85.Click Pay Button,tap,,"mobile.diver.subscription.pay_btn"
+86.Select Wallet Payment,tap,,"mobile.diver.subscription.select_wallet"
+87.Click Proceed to Pay,tap,,"mobile.diver.subscription.proceed_to_pay"
+88.Wait For Payment,wait,5000,
+89.Cancel Subscription,tap_coordinate ,971:362,COORDINATE_MODE
+90.Confirm Cancel Subscrption,tap,,"mobile.diver.subscription.confirm_cancel_subscription"
+88.Load Super Admin,switch_to,web,
+89.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+90.Click Subscription Plan,click,,"admin.subscription.menu_link"
+91.Click Customer subscription plan,click,,"admin.subscription.customer.tab"
+92.Filter Services List,type,{customerSubscriptionName},"admin.subscription.common.filter.input"
+93.Click Delete Customer Subscription Plan,click,,"admin.subscription.customer.delete.icon"
+94.Confirm Delete Customer Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+95.Wait For Deletion,wait,2000,
+96.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+97.Click Subscription Plan,click,,"admin.subscription.menu_link"
+98.Click Driver subscription plan,click,,"admin.subscription.driver.tab"
+99.Filter Services List,type,{driverSubscriptionName},"admin.subscription.common.filter.input"
+100.Click Delete Driver  Subscription Plan,click,,"admin.subscription.driver.delete.icon"
+101.Confirm Delete Driver Subscription Plan,click,,"admin.subscription.common.dialog.btn_delete_confirm"
+102.Wait For Deletion,wait,2000,</t>
+  </si>
+  <si>
+    <t>1. Load Driver App,switch_to,driver,
+2.Reload Driver App Completely,reload_app,driver,
+3. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+4. Load Super Admin,switch_to,web,
+5.Wait For Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"
+6. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+7. Click Settings Menu,click,,"web.global.menu.settings"
+8. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+9. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+10.Wait For On,wait,2000,
+11. Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+12. Click Submit Button,click,,"web.global.action.submit"
+13. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+14. Load Driver App,switch_to,driver,
+15. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+16. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+17. Click Agree,tap,,"mobile.driver.agree.btn"
+18. Click Get Started,tap,,"mobile.driver.get_started.btn"
+19. Click Next,tap,,"mobile.driver.next.btn"
+20. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+21. Click Close,tap,,"mobile.driver.cancel.btn"
+22. Enter Mobile Number,type,regression.approved_driver.phone,"mobile.driver.edit_text.input"
+23. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+24. Click Continue,tap,,"mobile.driver.continue.btn"
+25. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+26. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+27. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+28. Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+29.wait for Wallet,wait_until_visible,"mobile.driver.wallet.btn"
+30.Click Wallet,tap,,"mobile.driver.wallet.btn"
+31.Wait For Topup,wait_until_visible,,"mobile.driver.top_up.btn"
+32.Click Topup,tap,,"mobile.driver.top_up.btn"
+33.Wait For Topup Sum,wait_until_visible,,"mobile.driver.top_up.btn"
+34.Click Hundered,tap,,"mobile.driver.top_up_amount.hundred"
+35.Click Proceed,tap,,"mobile.driver.top_up.proceed"
+36.Wait For Contact No,wait_until_visible,,"mobile.driver.top_up.contact_no_box"
+37.Enter Driver Mobile,type,regression.approved_driver.phone,"mobile.driver.top_up.contact_no_box"
+38.Wait For Payment Options,wait_until_visible,,"mobile.driver.top_up.payment_option"
+39.Wait For Net Banking,wait,5000,
+40.Click Net Banking,tap,,"mobile.driver.top_up.net_banking"
+41.Wait For Bob,wait,5000,
+42.Click Bob,tap_coordinate,277:1461,
+43.Wait For Success,wait_until_visible,,"mobile.driver.top_up.succes_popup"
+44.Click Success,tap,,"mobile.driver.top_up.succes_popup"
+45.Wait For Wallet  Back,wait_until_visible,,"mobile.driver.wallet.btn"
+46.Click Back,tap,,"mobile.driver.back.btn"
+47.Drag Page Layout Upward,swipe,up,
+48.Click Back,tap,,"mobile.driver.back.btn"
+49.Reload Driver App Completely,reload_app,driver,
+50. Switch To Web Session,switch_to,web,
+51.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+52. Click Settings Menu,click,,"admin.setting.sidebar.menu"
+53. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+54. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+55.Wait For off,wait,2000,
+56. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
+57. Click Submit Button,click,,"web.global.action.submit"
+58. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+59. Switch To Driver Session,switch_to,driver,
+60. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+61. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+62. Click Agree,tap,,"mobile.driver.agree.btn"
+63. Click Get Started,tap,,"mobile.driver.get_started.btn"
+64. Click Next,tap,,"mobile.driver.next.btn"
+65. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+66. Click Close,tap,,"mobile.driver.cancel.btn"
+67. Enter Mobile Number,type,regression.approved_driver.phone ,"mobile.driver.edit_text.input"
+68. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+69. Click Continue,tap,,"mobile.driver.continue.btn"
+70. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+71. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+72. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+73.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+74.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
+75.Check Wallet absent,element_absent,,"mobile.driver.wallet.btn"</t>
+  </si>
+  <si>
+    <t>TC_CA_0A_Autoride_Test_Otp_DB</t>
+  </si>
+  <si>
+    <t>TC_CA_0B_Hybrid_Add_Customer</t>
+  </si>
+  <si>
+    <t>TC_CA_0C_Hybrid_Unapproved_Auto_Driver</t>
+  </si>
+  <si>
+    <t>SA_TS_0D</t>
+  </si>
+  <si>
+    <t>TC_CA_0D_Hybrid_Approved_Auto_Driver</t>
+  </si>
+  <si>
+    <t>TC_CA_08_Completed_Ride_Customer_Report_Issue</t>
+  </si>
+  <si>
+    <t>TC_CA_09_Autoride_Test_Otp_Ui</t>
   </si>
 </sst>
 </file>
@@ -3074,7 +3177,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D250DB7C-844B-4BAE-BD85-886B660DFD66}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77578C42-408B-4BD1-8455-A36E9774F1FD}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3116,28 +3219,28 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>79</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>64</v>
+        <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3158,25 +3261,24 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B31CB41-AC3C-4084-88C1-98C363B7ABCB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
@@ -3192,50 +3294,43 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>87</v>
+        <v>8</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>88</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>85</v>
+        <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="H2" s="2"/>
+        <v>10</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
+      <c r="C3" s="1"/>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="E3" s="7"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3282,22 +3377,22 @@
     </row>
     <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>50</v>
@@ -3324,164 +3419,6 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77578C42-408B-4BD1-8455-A36E9774F1FD}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="29.109375" customWidth="1"/>
-    <col min="5" max="5" width="71.44140625" customWidth="1"/>
-    <col min="6" max="6" width="40.44140625" customWidth="1"/>
-    <col min="7" max="7" width="61.88671875" customWidth="1"/>
-    <col min="8" max="8" width="32.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="26.77734375" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" customWidth="1"/>
-    <col min="5" max="5" width="69.33203125" customWidth="1"/>
-    <col min="6" max="6" width="31.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="7"/>
-    </row>
-  </sheetData>
-  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35E5A465-4C2B-4523-8755-30CE3021A8BD}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3530,7 +3467,7 @@
         <v>33</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>59</v>
+        <v>99</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>34</v>
@@ -3560,7 +3497,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42DE31E4-5C3B-413E-B08A-861302F9F4DC}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3602,13 +3539,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>61</v>
+        <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>37</v>
@@ -3635,7 +3572,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8946E02E-8751-499F-BD67-2B828D4C435E}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3677,13 +3614,13 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>71</v>
+        <v>102</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>13</v>
@@ -3707,7 +3644,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA5DCFAC-B912-41EA-9964-A3839A72D798}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3753,19 +3690,19 @@
         <v>17</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>48</v>
@@ -3791,7 +3728,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD2DD3E8-3167-4AD5-B95A-26FB801D55E0}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3840,16 +3777,16 @@
         <v>47</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>46</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>53</v>
+        <v>97</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
@@ -3875,7 +3812,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0586A9D0-0ABC-41A4-8FF3-8503F348B496}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3921,25 +3858,25 @@
         <v>35</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>78</v>
-      </c>
       <c r="H2" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3959,7 +3896,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{437C624E-95B4-48EB-A315-8931C834404A}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4005,19 +3942,19 @@
         <v>41</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
@@ -4043,7 +3980,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0962450F-C7D8-41FC-90CD-CAAFB127F74F}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4089,19 +4026,19 @@
         <v>42</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>21</v>
@@ -4125,4 +4062,254 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D250DB7C-844B-4BAE-BD85-886B660DFD66}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B31CB41-AC3C-4084-88C1-98C363B7ABCB}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0BD74F5-8D47-475E-A6FE-D0E5567AC0D3}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="29.109375" customWidth="1"/>
+    <col min="5" max="5" width="71.44140625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
+    <col min="7" max="7" width="61.88671875" customWidth="1"/>
+    <col min="8" max="8" width="32.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>